<commit_message>
Record payment: ₹10,000.00 by Asif Sayyed (Son) for Pratap films and Photography
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H41</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1187,7 +1187,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2239,10 +2239,36 @@
         <v/>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>c44e46e8</v>
+      </c>
+      <c r="B41" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D41" s="3">
+        <v>46273</v>
+      </c>
+      <c r="E41" s="1">
+        <v>10000</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G41" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H41" t="str">
+        <v>3rd installment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H40"/>
+  <autoFilter ref="A1:H41"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H41"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2857,11 +2883,11 @@
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
-        <v>80000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="33">
@@ -2988,11 +3014,11 @@
       </c>
       <c r="D39" s="1">
         <f>SUM(D2:D38)</f>
-        <v>297266</v>
+        <v>307266</v>
       </c>
       <c r="E39" s="1">
         <f>SUM(E2:E38)</f>
-        <v>831000</v>
+        <v>821000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹8,000.00 by Asif Sayyed (Son) for Aluminum Shop Partition
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H42</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1187,7 +1187,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2265,10 +2265,36 @@
         <v>3rd installment</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>7cdb194e</v>
+      </c>
+      <c r="B42" t="str">
+        <v>aaedf833</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Aluminum Shop Partition</v>
+      </c>
+      <c r="D42" s="3">
+        <v>46278</v>
+      </c>
+      <c r="E42" s="1">
+        <v>8000</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G42" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Completed payment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H41"/>
+  <autoFilter ref="A1:H42"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H42"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2389,11 +2415,11 @@
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>23000</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>8000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3014,11 +3040,11 @@
       </c>
       <c r="D39" s="1">
         <f>SUM(D2:D38)</f>
-        <v>307266</v>
+        <v>315266</v>
       </c>
       <c r="E39" s="1">
         <f>SUM(E2:E38)</f>
-        <v>821000</v>
+        <v>813000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Ice Cream, vada pav, Irani Cafe, Milk — ₹3,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H42</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -799,388 +799,408 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B20" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C20" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D20" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B21" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C21" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D21" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F21" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B22" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C22" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D22" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F22" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B23" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D23" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B24" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D24" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B25" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>30b69ec5</v>
+        <v>a78dd739</v>
       </c>
       <c r="B26" t="str">
-        <v>Mummy sadi</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B27" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C27" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B28" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C28" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D28" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B29" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D29" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B30" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B31" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C31" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>beb44857</v>
+        <v>0421ab42</v>
       </c>
       <c r="B32" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C32" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D32" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E32" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F32" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B33" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C33" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D33" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F33" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B34" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C34" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D34" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B35" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D35" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B36" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C36" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E36" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F36" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B37" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C37" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D37" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E37" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F37" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
+        <v>bd5f8d26</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D38" s="1">
+        <v>6190</v>
+      </c>
+      <c r="E38" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
         <v>db4969e8</v>
       </c>
-      <c r="B38" t="str">
+      <c r="B39" t="str">
         <v>Tushar Traders Oil</v>
       </c>
-      <c r="C38" t="str">
+      <c r="C39" t="str">
         <v>Food &amp; Catering</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D39" s="1">
         <v>5100</v>
       </c>
-      <c r="E38" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F38" t="str">
+      <c r="E39" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
         <v>Tushar Traders Oil</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F38"/>
+  <autoFilter ref="A1:F39"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F39"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2301,7 +2321,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2671,36 +2691,36 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B20" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C20" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B21" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C21" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -2709,17 +2729,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B22" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C22" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2728,17 +2748,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C23" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2747,17 +2767,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C24" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2766,17 +2786,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2785,17 +2805,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Mummy sadi</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2804,17 +2824,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B27" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -2823,17 +2843,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B28" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C28" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -2842,17 +2862,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C29" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -2861,17 +2881,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -2880,17 +2900,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B31" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -2899,55 +2919,55 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B32" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C32" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>30000</v>
+        <v>4000</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
-        <v>70000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B33" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C33" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>30000</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>0</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B34" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C34" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -2956,17 +2976,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C35" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -2975,55 +2995,55 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B36" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B37" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C37" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B38" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C38" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -3032,24 +3052,43 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C39" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D39" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E39" s="1">
+        <f>C39-D39</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
         <v>Total</v>
       </c>
-      <c r="C39" s="1">
-        <f>SUM(C2:C38)</f>
-        <v>1128266</v>
-      </c>
-      <c r="D39" s="1">
-        <f>SUM(D2:D38)</f>
+      <c r="C40" s="1">
+        <f>SUM(C2:C39)</f>
+        <v>1131266</v>
+      </c>
+      <c r="D40" s="1">
+        <f>SUM(D2:D39)</f>
         <v>315266</v>
       </c>
-      <c r="E39" s="1">
-        <f>SUM(E2:E38)</f>
-        <v>813000</v>
+      <c r="E40" s="1">
+        <f>SUM(E2:E39)</f>
+        <v>816000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹3,000.00 by Asif Sayyed (Son) for Ice Cream, vada pav, Irani Cafe, Milk
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H43</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1207,7 +1207,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2311,10 +2311,36 @@
         <v>Completed payment</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>ecbdb657</v>
+      </c>
+      <c r="B43" t="str">
+        <v>dc70b2a1</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+      </c>
+      <c r="D43" s="3">
+        <v>46278</v>
+      </c>
+      <c r="E43" s="1">
+        <v>3000</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G43" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H43" t="str">
+        <v>payed</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H42"/>
+  <autoFilter ref="A1:H43"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2701,11 +2727,11 @@
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -3079,11 +3105,11 @@
       </c>
       <c r="D40" s="1">
         <f>SUM(D2:D39)</f>
-        <v>315266</v>
+        <v>318266</v>
       </c>
       <c r="E40" s="1">
         <f>SUM(E2:E39)</f>
-        <v>816000</v>
+        <v>813000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance — ₹4,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H43</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1059,148 +1059,168 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B33" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C33" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D33" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F33" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B34" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C34" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D34" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F34" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B35" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C35" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D35" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B36" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C36" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D36" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B37" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C37" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D37" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E37" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F37" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B38" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C38" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D38" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E38" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F38" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
+        <v>bd5f8d26</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D39" s="1">
+        <v>6190</v>
+      </c>
+      <c r="E39" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
         <v>db4969e8</v>
       </c>
-      <c r="B39" t="str">
+      <c r="B40" t="str">
         <v>Tushar Traders Oil</v>
       </c>
-      <c r="C39" t="str">
+      <c r="C40" t="str">
         <v>Food &amp; Catering</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D40" s="1">
         <v>5100</v>
       </c>
-      <c r="E39" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F39" t="str">
+      <c r="E40" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
         <v>Tushar Traders Oil</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F39"/>
+  <autoFilter ref="A1:F40"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2347,7 +2367,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2964,55 +2984,55 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B33" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C33" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B34" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C34" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>30000</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
-        <v>0</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B35" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C35" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -3021,17 +3041,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B36" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C36" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -3040,55 +3060,55 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B37" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C37" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B38" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C38" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B39" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C39" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -3097,24 +3117,43 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C40" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D40" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E40" s="1">
+        <f>C40-D40</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
         <v>Total</v>
       </c>
-      <c r="C40" s="1">
-        <f>SUM(C2:C39)</f>
-        <v>1131266</v>
-      </c>
-      <c r="D40" s="1">
-        <f>SUM(D2:D39)</f>
+      <c r="C41" s="1">
+        <f>SUM(C2:C40)</f>
+        <v>1135266</v>
+      </c>
+      <c r="D41" s="1">
+        <f>SUM(D2:D40)</f>
         <v>318266</v>
       </c>
-      <c r="E40" s="1">
-        <f>SUM(E2:E39)</f>
-        <v>813000</v>
+      <c r="E41" s="1">
+        <f>SUM(E2:E40)</f>
+        <v>817000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹4,000.00 by Asif Sayyed (Son) for Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H44</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1227,7 +1227,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2357,10 +2357,36 @@
         <v>payed</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>b8049298</v>
+      </c>
+      <c r="B44" t="str">
+        <v>84c049af</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+      </c>
+      <c r="D44" s="3">
+        <v>46279</v>
+      </c>
+      <c r="E44" s="1">
+        <v>4000</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G44" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H44" t="str">
+        <v>payed</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H43"/>
+  <autoFilter ref="A1:H44"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H44"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2994,11 +3020,11 @@
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>4000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -3144,11 +3170,11 @@
       </c>
       <c r="D41" s="1">
         <f>SUM(D2:D40)</f>
-        <v>318266</v>
+        <v>322266</v>
       </c>
       <c r="E41" s="1">
         <f>SUM(E2:E40)</f>
-        <v>817000</v>
+        <v>813000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Asif Radimant dress, jokey inner ware, white tighty, sliper — ₹7,100.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H44</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -579,493 +579,493 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>0e8bf89b</v>
+        <v>f68b08a7</v>
       </c>
       <c r="B9" t="str">
-        <v>Bari ka saman</v>
+        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
       </c>
       <c r="C9" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>2200</v>
+        <v>7100</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Bari ka saman</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>1aa31869</v>
+        <v>0e8bf89b</v>
       </c>
       <c r="B10" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="C10" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D10" s="1">
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="E10" s="2" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>0beedebe</v>
+        <v>1aa31869</v>
       </c>
       <c r="B11" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="C11" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D11" s="1">
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="E11" s="2" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2a74d868</v>
+        <v>0beedebe</v>
       </c>
       <c r="B12" t="str">
-        <v>Colour &amp; plumber</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="C12" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D12" s="1">
-        <v>800</v>
+        <v>4600</v>
       </c>
       <c r="E12" s="2" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>05d27deb</v>
+        <v>2a74d868</v>
       </c>
       <c r="B13" t="str">
-        <v>Cream House Lunch</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="C13" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D13" s="1">
-        <v>1124</v>
+        <v>800</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>Cream House Lunch</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>631875ca</v>
+        <v>05d27deb</v>
       </c>
       <c r="B14" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="C14" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D14" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F14" t="str">
-        <v>Hall decoration</v>
+        <v>Cream House Lunch</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B15" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C15" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D15" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F15" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B16" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B17" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C17" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F17" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B18" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C18" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D18" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E18" s="2" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B19" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C19" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D19" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F19" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>dc70b2a1</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B20" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C20" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D20" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F20" t="str">
-        <v>internal expense</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B21" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C21" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D21" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F21" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B22" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C22" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D22" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F22" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B23" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C23" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D23" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F23" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B24" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D24" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B25" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B26" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>30b69ec5</v>
+        <v>a78dd739</v>
       </c>
       <c r="B27" t="str">
-        <v>Mummy sadi</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B28" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C28" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B29" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C29" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D29" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B30" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D30" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B31" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B32" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C32" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B33" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C33" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D33" s="1">
         <v>4000</v>
@@ -1079,148 +1079,168 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B34" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C34" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D34" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F34" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B35" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C35" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D35" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E35" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F35" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B36" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C36" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D36" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B37" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C37" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D37" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B38" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C38" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D38" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E38" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F38" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B39" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C39" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D39" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E39" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F39" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
+        <v>bd5f8d26</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D40" s="1">
+        <v>6190</v>
+      </c>
+      <c r="E40" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
         <v>db4969e8</v>
       </c>
-      <c r="B40" t="str">
+      <c r="B41" t="str">
         <v>Tushar Traders Oil</v>
       </c>
-      <c r="C40" t="str">
+      <c r="C41" t="str">
         <v>Food &amp; Catering</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D41" s="1">
         <v>5100</v>
       </c>
-      <c r="E40" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F40" t="str">
+      <c r="E41" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
         <v>Tushar Traders Oil</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F40"/>
+  <autoFilter ref="A1:F41"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F41"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2393,7 +2413,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2554,36 +2574,36 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Bari ka saman</v>
+        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
       </c>
       <c r="B9" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>2200</v>
+        <v>7100</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>0</v>
+        <v>7100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="B10" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C10" s="1">
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -2592,17 +2612,17 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="B11" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C11" s="1">
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -2611,17 +2631,17 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Colour &amp; plumber</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="B12" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C12" s="1">
-        <v>800</v>
+        <v>4600</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>800</v>
+        <v>4600</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -2630,17 +2650,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Cream House Lunch</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="B13" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C13" s="1">
-        <v>1124</v>
+        <v>800</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>1124</v>
+        <v>800</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -2649,55 +2669,55 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="B14" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C14" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>1124</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>128000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B15" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C15" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -2706,17 +2726,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B17" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -2725,17 +2745,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B18" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C18" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -2744,55 +2764,55 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B19" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C19" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B20" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C20" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>50000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B21" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C21" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -2801,17 +2821,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B22" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C22" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2820,17 +2840,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B23" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C23" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2839,17 +2859,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C24" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2858,17 +2878,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2877,17 +2897,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2896,17 +2916,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Mummy sadi</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -2915,17 +2935,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B28" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -2934,17 +2954,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B29" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C29" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -2953,17 +2973,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C30" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -2972,17 +2992,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -2991,17 +3011,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B32" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3010,10 +3030,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B33" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C33" s="1">
         <v>4000</v>
@@ -3029,55 +3049,55 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B34" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C34" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>30000</v>
+        <v>4000</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
-        <v>70000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B35" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C35" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>30000</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
-        <v>0</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B36" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C36" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -3086,17 +3106,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B37" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C37" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -3105,55 +3125,55 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B38" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C38" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B39" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C39" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B40" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C40" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -3162,24 +3182,43 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C41" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D41" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E41" s="1">
+        <f>C41-D41</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
         <v>Total</v>
       </c>
-      <c r="C41" s="1">
-        <f>SUM(C2:C40)</f>
-        <v>1135266</v>
-      </c>
-      <c r="D41" s="1">
-        <f>SUM(D2:D40)</f>
+      <c r="C42" s="1">
+        <f>SUM(C2:C41)</f>
+        <v>1142366</v>
+      </c>
+      <c r="D42" s="1">
+        <f>SUM(D2:D41)</f>
         <v>322266</v>
       </c>
-      <c r="E41" s="1">
-        <f>SUM(E2:E40)</f>
-        <v>813000</v>
+      <c r="E42" s="1">
+        <f>SUM(E2:E41)</f>
+        <v>820100</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E42"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹7,100.00 by Asif Sayyed (Son) for Asif Radimant dress, jokey inner ware, white tighty, sliper
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H45</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1247,7 +1247,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2403,10 +2403,36 @@
         <v>payed</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>cf880b55</v>
+      </c>
+      <c r="B45" t="str">
+        <v>f68b08a7</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+      </c>
+      <c r="D45" s="3">
+        <v>46279</v>
+      </c>
+      <c r="E45" s="1">
+        <v>7100</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G45" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H45" t="str">
+        <v>paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H44"/>
+  <autoFilter ref="A1:H45"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H45"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2584,11 +2610,11 @@
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>7100</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>7100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -3209,11 +3235,11 @@
       </c>
       <c r="D42" s="1">
         <f>SUM(D2:D41)</f>
-        <v>322266</v>
+        <v>329366</v>
       </c>
       <c r="E42" s="1">
         <f>SUM(E2:E41)</f>
-        <v>820100</v>
+        <v>813000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Mummy Hospital Expence Mate Docter — ₹2,900.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H45</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -959,16 +959,16 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B28" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D28" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
@@ -979,113 +979,113 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B29" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C29" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B30" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C30" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D30" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B31" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D31" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B32" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B33" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C33" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B34" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C34" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D34" s="1">
         <v>4000</v>
@@ -1099,148 +1099,168 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B35" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C35" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D35" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E35" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F35" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B36" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C36" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D36" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E36" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F36" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B37" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C37" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D37" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B38" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C38" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D38" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B39" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C39" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D39" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E39" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F39" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B40" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C40" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D40" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E40" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F40" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
+        <v>bd5f8d26</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D41" s="1">
+        <v>6190</v>
+      </c>
+      <c r="E41" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
         <v>db4969e8</v>
       </c>
-      <c r="B41" t="str">
+      <c r="B42" t="str">
         <v>Tushar Traders Oil</v>
       </c>
-      <c r="C41" t="str">
+      <c r="C42" t="str">
         <v>Food &amp; Catering</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D42" s="1">
         <v>5100</v>
       </c>
-      <c r="E41" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F41" t="str">
+      <c r="E42" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
         <v>Tushar Traders Oil</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F41"/>
+  <autoFilter ref="A1:F42"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F42"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2439,7 +2459,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2961,36 +2981,36 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C28" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>0</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
-        <v>0</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B29" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -2999,17 +3019,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B30" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C30" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3018,17 +3038,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C31" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3037,17 +3057,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3056,17 +3076,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B33" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3075,10 +3095,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B34" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C34" s="1">
         <v>4000</v>
@@ -3094,55 +3114,55 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B35" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C35" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>30000</v>
+        <v>4000</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
-        <v>70000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B36" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C36" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>30000</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
-        <v>0</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B37" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C37" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -3151,17 +3171,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B38" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C38" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -3170,55 +3190,55 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B39" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C39" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B40" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C40" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B41" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C41" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -3227,24 +3247,43 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C42" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D42" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E42" s="1">
+        <f>C42-D42</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
         <v>Total</v>
       </c>
-      <c r="C42" s="1">
-        <f>SUM(C2:C41)</f>
-        <v>1142366</v>
-      </c>
-      <c r="D42" s="1">
-        <f>SUM(D2:D41)</f>
+      <c r="C43" s="1">
+        <f>SUM(C2:C42)</f>
+        <v>1145266</v>
+      </c>
+      <c r="D43" s="1">
+        <f>SUM(D2:D42)</f>
         <v>329366</v>
       </c>
-      <c r="E42" s="1">
-        <f>SUM(E2:E41)</f>
-        <v>813000</v>
+      <c r="E43" s="1">
+        <f>SUM(E2:E42)</f>
+        <v>815900</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹2,900.00 by Asif Sayyed (Son) for Mummy Hospital Expence Mate Docter
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H46</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1267,7 +1267,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2347,19 +2347,19 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>7cdb194e</v>
+        <v>7ac7100a</v>
       </c>
       <c r="B42" t="str">
-        <v>aaedf833</v>
+        <v>b1e7073e</v>
       </c>
       <c r="C42" t="str">
-        <v>Aluminum Shop Partition</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="D42" s="3">
-        <v>46278</v>
+        <v>46276</v>
       </c>
       <c r="E42" s="1">
-        <v>8000</v>
+        <v>2900</v>
       </c>
       <c r="F42" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2368,24 +2368,24 @@
         <v>UPI</v>
       </c>
       <c r="H42" t="str">
-        <v>Completed payment</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ecbdb657</v>
+        <v>7cdb194e</v>
       </c>
       <c r="B43" t="str">
-        <v>dc70b2a1</v>
+        <v>aaedf833</v>
       </c>
       <c r="C43" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Aluminum Shop Partition</v>
       </c>
       <c r="D43" s="3">
         <v>46278</v>
       </c>
       <c r="E43" s="1">
-        <v>3000</v>
+        <v>8000</v>
       </c>
       <c r="F43" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2394,24 +2394,24 @@
         <v>UPI</v>
       </c>
       <c r="H43" t="str">
-        <v>payed</v>
+        <v>Completed payment</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>b8049298</v>
+        <v>ecbdb657</v>
       </c>
       <c r="B44" t="str">
-        <v>84c049af</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="C44" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="D44" s="3">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="E44" s="1">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="F44" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2425,19 +2425,19 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>cf880b55</v>
+        <v>b8049298</v>
       </c>
       <c r="B45" t="str">
-        <v>f68b08a7</v>
+        <v>84c049af</v>
       </c>
       <c r="C45" t="str">
-        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="D45" s="3">
         <v>46279</v>
       </c>
       <c r="E45" s="1">
-        <v>7100</v>
+        <v>4000</v>
       </c>
       <c r="F45" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2446,13 +2446,39 @@
         <v>UPI</v>
       </c>
       <c r="H45" t="str">
+        <v>payed</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>cf880b55</v>
+      </c>
+      <c r="B46" t="str">
+        <v>f68b08a7</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+      </c>
+      <c r="D46" s="3">
+        <v>46279</v>
+      </c>
+      <c r="E46" s="1">
+        <v>7100</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G46" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H46" t="str">
         <v>paid</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H45"/>
+  <autoFilter ref="A1:H46"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H46"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2991,11 +3017,11 @@
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>2900</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
-        <v>2900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3274,11 +3300,11 @@
       </c>
       <c r="D43" s="1">
         <f>SUM(D2:D42)</f>
-        <v>329366</v>
+        <v>332266</v>
       </c>
       <c r="E43" s="1">
         <f>SUM(E2:E42)</f>
-        <v>815900</v>
+        <v>813000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Garva Biryani, hardware expense, flower — ₹410.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H46</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -779,216 +779,216 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>209d43b7</v>
+        <v>766bfdf7</v>
       </c>
       <c r="B19" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="C19" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D19" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B20" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C20" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D20" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>dc70b2a1</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B21" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C21" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D21" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F21" t="str">
-        <v>internal expense</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B22" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C22" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D22" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B23" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C23" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D23" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F23" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B24" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C24" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D24" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F24" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B25" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B26" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B27" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B28" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C28" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B29" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D29" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
@@ -999,113 +999,113 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B30" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C30" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B31" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C31" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D31" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B32" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D32" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B33" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C33" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B34" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C34" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B35" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C35" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D35" s="1">
         <v>4000</v>
@@ -1119,148 +1119,168 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B36" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C36" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D36" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E36" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F36" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B37" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C37" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D37" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E37" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F37" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B38" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C38" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D38" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B39" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C39" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D39" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B40" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C40" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D40" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E40" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F40" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B41" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C41" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D41" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E41" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F41" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
+        <v>bd5f8d26</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D42" s="1">
+        <v>6190</v>
+      </c>
+      <c r="E42" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
         <v>db4969e8</v>
       </c>
-      <c r="B42" t="str">
+      <c r="B43" t="str">
         <v>Tushar Traders Oil</v>
       </c>
-      <c r="C42" t="str">
+      <c r="C43" t="str">
         <v>Food &amp; Catering</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D43" s="1">
         <v>5100</v>
       </c>
-      <c r="E42" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F42" t="str">
+      <c r="E43" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
         <v>Tushar Traders Oil</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F42"/>
+  <autoFilter ref="A1:F43"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2485,7 +2505,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2836,74 +2856,74 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="B19" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C19" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
-        <v>0</v>
+        <v>410</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B20" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C20" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B21" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C21" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>50000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B22" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C22" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2912,17 +2932,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B23" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C23" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2931,17 +2951,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B24" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C24" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2950,17 +2970,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2969,17 +2989,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2988,17 +3008,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -3007,17 +3027,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B28" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -3026,17 +3046,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C29" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -3045,17 +3065,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B30" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3064,17 +3084,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B31" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C31" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3083,17 +3103,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C32" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3102,17 +3122,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B33" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3121,17 +3141,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B34" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -3140,10 +3160,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B35" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C35" s="1">
         <v>4000</v>
@@ -3159,55 +3179,55 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B36" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C36" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>30000</v>
+        <v>4000</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
-        <v>70000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B37" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C37" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>30000</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
-        <v>0</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B38" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C38" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -3216,17 +3236,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B39" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C39" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -3235,55 +3255,55 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B40" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C40" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B41" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C41" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B42" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C42" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
@@ -3292,24 +3312,43 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C43" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D43" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E43" s="1">
+        <f>C43-D43</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
         <v>Total</v>
       </c>
-      <c r="C43" s="1">
-        <f>SUM(C2:C42)</f>
-        <v>1145266</v>
-      </c>
-      <c r="D43" s="1">
-        <f>SUM(D2:D42)</f>
+      <c r="C44" s="1">
+        <f>SUM(C2:C43)</f>
+        <v>1145676</v>
+      </c>
+      <c r="D44" s="1">
+        <f>SUM(D2:D43)</f>
         <v>332266</v>
       </c>
-      <c r="E43" s="1">
-        <f>SUM(E2:E42)</f>
-        <v>813000</v>
+      <c r="E44" s="1">
+        <f>SUM(E2:E43)</f>
+        <v>813410</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E44"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹410.00 by Asif Sayyed (Son) for Garva Biryani, hardware expense, flower
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H47</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1287,7 +1287,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2393,19 +2393,19 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>7cdb194e</v>
+        <v>5da4a0cf</v>
       </c>
       <c r="B43" t="str">
-        <v>aaedf833</v>
+        <v>766bfdf7</v>
       </c>
       <c r="C43" t="str">
-        <v>Aluminum Shop Partition</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="D43" s="3">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="E43" s="1">
-        <v>8000</v>
+        <v>410</v>
       </c>
       <c r="F43" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2414,24 +2414,24 @@
         <v>UPI</v>
       </c>
       <c r="H43" t="str">
-        <v>Completed payment</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ecbdb657</v>
+        <v>7cdb194e</v>
       </c>
       <c r="B44" t="str">
-        <v>dc70b2a1</v>
+        <v>aaedf833</v>
       </c>
       <c r="C44" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Aluminum Shop Partition</v>
       </c>
       <c r="D44" s="3">
         <v>46278</v>
       </c>
       <c r="E44" s="1">
-        <v>3000</v>
+        <v>8000</v>
       </c>
       <c r="F44" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2440,24 +2440,24 @@
         <v>UPI</v>
       </c>
       <c r="H44" t="str">
-        <v>payed</v>
+        <v>Completed payment</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>b8049298</v>
+        <v>ecbdb657</v>
       </c>
       <c r="B45" t="str">
-        <v>84c049af</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="C45" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="D45" s="3">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="E45" s="1">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="F45" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2471,19 +2471,19 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>cf880b55</v>
+        <v>b8049298</v>
       </c>
       <c r="B46" t="str">
-        <v>f68b08a7</v>
+        <v>84c049af</v>
       </c>
       <c r="C46" t="str">
-        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="D46" s="3">
         <v>46279</v>
       </c>
       <c r="E46" s="1">
-        <v>7100</v>
+        <v>4000</v>
       </c>
       <c r="F46" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2492,13 +2492,39 @@
         <v>UPI</v>
       </c>
       <c r="H46" t="str">
+        <v>payed</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>cf880b55</v>
+      </c>
+      <c r="B47" t="str">
+        <v>f68b08a7</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+      </c>
+      <c r="D47" s="3">
+        <v>46279</v>
+      </c>
+      <c r="E47" s="1">
+        <v>7100</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G47" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H47" t="str">
         <v>paid</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H46"/>
+  <autoFilter ref="A1:H47"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H47"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2866,11 +2892,11 @@
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>410</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
-        <v>410</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -3339,11 +3365,11 @@
       </c>
       <c r="D44" s="1">
         <f>SUM(D2:D43)</f>
-        <v>332266</v>
+        <v>332676</v>
       </c>
       <c r="E44" s="1">
         <f>SUM(E2:E43)</f>
-        <v>813410</v>
+        <v>813000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Untracked expenses Petrol, Food, small bills — ₹9,150.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H47</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1277,10 +1277,30 @@
         <v>Tushar Traders Oil</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>9961a7bb</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="D44" s="1">
+        <v>9150</v>
+      </c>
+      <c r="E44" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F43"/>
+  <autoFilter ref="A1:F44"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F44"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2531,7 +2551,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3357,24 +3377,43 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C44" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D44" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="1">
+        <f>C44-D44</f>
+        <v>9150</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
         <v>Total</v>
       </c>
-      <c r="C44" s="1">
-        <f>SUM(C2:C43)</f>
-        <v>1145676</v>
-      </c>
-      <c r="D44" s="1">
-        <f>SUM(D2:D43)</f>
+      <c r="C45" s="1">
+        <f>SUM(C2:C44)</f>
+        <v>1154826</v>
+      </c>
+      <c r="D45" s="1">
+        <f>SUM(D2:D44)</f>
         <v>332676</v>
       </c>
-      <c r="E44" s="1">
-        <f>SUM(E2:E43)</f>
-        <v>813000</v>
+      <c r="E45" s="1">
+        <f>SUM(E2:E44)</f>
+        <v>822150</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹9,150.00 by Asif Sayyed (Son) for Untracked expenses Petrol, Food, small bills
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H48</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1307,7 +1307,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2387,19 +2387,19 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>7ac7100a</v>
+        <v>233eee35</v>
       </c>
       <c r="B42" t="str">
-        <v>b1e7073e</v>
+        <v>9961a7bb</v>
       </c>
       <c r="C42" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
       <c r="D42" s="3">
-        <v>46276</v>
+        <v>46273</v>
       </c>
       <c r="E42" s="1">
-        <v>2900</v>
+        <v>9150</v>
       </c>
       <c r="F42" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2408,24 +2408,24 @@
         <v>UPI</v>
       </c>
       <c r="H42" t="str">
-        <v>paid</v>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>5da4a0cf</v>
+        <v>7ac7100a</v>
       </c>
       <c r="B43" t="str">
-        <v>766bfdf7</v>
+        <v>b1e7073e</v>
       </c>
       <c r="C43" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="D43" s="3">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="E43" s="1">
-        <v>410</v>
+        <v>2900</v>
       </c>
       <c r="F43" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2434,24 +2434,24 @@
         <v>UPI</v>
       </c>
       <c r="H43" t="str">
-        <v>Paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>7cdb194e</v>
+        <v>5da4a0cf</v>
       </c>
       <c r="B44" t="str">
-        <v>aaedf833</v>
+        <v>766bfdf7</v>
       </c>
       <c r="C44" t="str">
-        <v>Aluminum Shop Partition</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="D44" s="3">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="E44" s="1">
-        <v>8000</v>
+        <v>410</v>
       </c>
       <c r="F44" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2460,24 +2460,24 @@
         <v>UPI</v>
       </c>
       <c r="H44" t="str">
-        <v>Completed payment</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ecbdb657</v>
+        <v>7cdb194e</v>
       </c>
       <c r="B45" t="str">
-        <v>dc70b2a1</v>
+        <v>aaedf833</v>
       </c>
       <c r="C45" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Aluminum Shop Partition</v>
       </c>
       <c r="D45" s="3">
         <v>46278</v>
       </c>
       <c r="E45" s="1">
-        <v>3000</v>
+        <v>8000</v>
       </c>
       <c r="F45" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2486,24 +2486,24 @@
         <v>UPI</v>
       </c>
       <c r="H45" t="str">
-        <v>payed</v>
+        <v>Completed payment</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>b8049298</v>
+        <v>ecbdb657</v>
       </c>
       <c r="B46" t="str">
-        <v>84c049af</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="C46" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="D46" s="3">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="E46" s="1">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="F46" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2517,19 +2517,19 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>cf880b55</v>
+        <v>b8049298</v>
       </c>
       <c r="B47" t="str">
-        <v>f68b08a7</v>
+        <v>84c049af</v>
       </c>
       <c r="C47" t="str">
-        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="D47" s="3">
         <v>46279</v>
       </c>
       <c r="E47" s="1">
-        <v>7100</v>
+        <v>4000</v>
       </c>
       <c r="F47" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2538,13 +2538,39 @@
         <v>UPI</v>
       </c>
       <c r="H47" t="str">
+        <v>payed</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>cf880b55</v>
+      </c>
+      <c r="B48" t="str">
+        <v>f68b08a7</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+      </c>
+      <c r="D48" s="3">
+        <v>46279</v>
+      </c>
+      <c r="E48" s="1">
+        <v>7100</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G48" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H48" t="str">
         <v>paid</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H47"/>
+  <autoFilter ref="A1:H48"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H48"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3387,11 +3413,11 @@
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>9150</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
-        <v>9150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -3404,11 +3430,11 @@
       </c>
       <c r="D45" s="1">
         <f>SUM(D2:D44)</f>
-        <v>332676</v>
+        <v>341826</v>
       </c>
       <c r="E45" s="1">
         <f>SUM(E2:E44)</f>
-        <v>822150</v>
+        <v>813000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹30,000.00 by Asif Sayyed (Son) for Day night Flower Decoration - (hall)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H49</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1307,7 +1307,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H49"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2567,10 +2567,36 @@
         <v>paid</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>1fb7d868</v>
+      </c>
+      <c r="B49" t="str">
+        <v>631875ca</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Day night Flower Decoration - (hall)</v>
+      </c>
+      <c r="D49" s="3">
+        <v>46280</v>
+      </c>
+      <c r="E49" s="1">
+        <v>30000</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G49" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H49" t="str">
+        <v>2nd installment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H48"/>
+  <autoFilter ref="A1:H49"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H49"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2862,11 +2888,11 @@
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>128000</v>
+        <v>98000</v>
       </c>
     </row>
     <row r="16">
@@ -3430,11 +3456,11 @@
       </c>
       <c r="D45" s="1">
         <f>SUM(D2:D44)</f>
-        <v>341826</v>
+        <v>371826</v>
       </c>
       <c r="E45" s="1">
         <f>SUM(E2:E44)</f>
-        <v>813000</v>
+        <v>783000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Mandva — ₹37,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H50</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -899,116 +899,116 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>c7e8b352</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="B25" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mandva</v>
       </c>
       <c r="C25" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D25" s="1">
-        <v>7604</v>
+        <v>37000</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B26" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B27" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B28" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B29" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C29" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B30" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D30" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
@@ -1019,113 +1019,113 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B31" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C31" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B32" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C32" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D32" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B33" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D33" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B34" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C34" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B35" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C35" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B36" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C36" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D36" s="1">
         <v>4000</v>
@@ -1139,168 +1139,188 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B37" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C37" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D37" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E37" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F37" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B38" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C38" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D38" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E38" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F38" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B39" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C39" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D39" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B40" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C40" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D40" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
       </c>
       <c r="F40" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B41" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C41" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D41" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E41" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F41" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B42" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C42" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D42" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E42" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F42" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B43" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C43" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D43" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E43" s="2" t="str">
         <v/>
       </c>
       <c r="F43" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D44" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E44" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B44" t="str">
+      <c r="B45" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C44" t="str">
+      <c r="C45" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D45" s="1">
         <v>9150</v>
       </c>
-      <c r="E44" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F44" t="str">
+      <c r="E45" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F44"/>
+  <autoFilter ref="A1:F45"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F45"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2629,7 +2649,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3094,36 +3114,36 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mandva</v>
       </c>
       <c r="B25" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C25" s="1">
-        <v>7604</v>
+        <v>37000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>0</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>0</v>
+        <v>37000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -3132,17 +3152,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -3151,17 +3171,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -3170,17 +3190,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B29" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -3189,17 +3209,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C30" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3208,17 +3228,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B31" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3227,17 +3247,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B32" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C32" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3246,17 +3266,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C33" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3265,17 +3285,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B34" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -3284,17 +3304,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B35" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -3303,10 +3323,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B36" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C36" s="1">
         <v>4000</v>
@@ -3322,55 +3342,55 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B37" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C37" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>30000</v>
+        <v>4000</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
-        <v>70000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B38" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C38" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>30000</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
-        <v>0</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B39" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C39" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -3379,17 +3399,17 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B40" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C40" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -3398,55 +3418,55 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B41" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C41" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B42" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C42" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B43" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C43" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
@@ -3455,17 +3475,17 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B44" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C44" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
@@ -3474,24 +3494,43 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C45" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D45" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E45" s="1">
+        <f>C45-D45</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
         <v>Total</v>
       </c>
-      <c r="C45" s="1">
-        <f>SUM(C2:C44)</f>
-        <v>1154826</v>
-      </c>
-      <c r="D45" s="1">
-        <f>SUM(D2:D44)</f>
+      <c r="C46" s="1">
+        <f>SUM(C2:C45)</f>
+        <v>1191826</v>
+      </c>
+      <c r="D46" s="1">
+        <f>SUM(D2:D45)</f>
         <v>401826</v>
       </c>
-      <c r="E45" s="1">
-        <f>SUM(E2:E44)</f>
-        <v>753000</v>
+      <c r="E46" s="1">
+        <f>SUM(E2:E45)</f>
+        <v>790000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹5,000.00 by Asif Sayyed (Son) for Mandva
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H51</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1327,7 +1327,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H51"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2639,10 +2639,36 @@
         <v>3rd instalment</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>ac587329</v>
+      </c>
+      <c r="B51" t="str">
+        <v>4d3bd5b1</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Mandva</v>
+      </c>
+      <c r="D51" s="3">
+        <v>46284</v>
+      </c>
+      <c r="E51" s="1">
+        <v>5000</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G51" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H50"/>
+  <autoFilter ref="A1:H51"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H51"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3124,11 +3150,11 @@
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>37000</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="26">
@@ -3521,11 +3547,11 @@
       </c>
       <c r="D46" s="1">
         <f>SUM(D2:D45)</f>
-        <v>401826</v>
+        <v>406826</v>
       </c>
       <c r="E46" s="1">
         <f>SUM(E2:E45)</f>
-        <v>790000</v>
+        <v>785000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹2,00,000.00 by Umar Sayyed (Father) for Huseni Caterers
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H52</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1327,7 +1327,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H52"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2665,10 +2665,36 @@
         <v/>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>59d53a62</v>
+      </c>
+      <c r="B52" t="str">
+        <v>168b7bbd</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Huseni Caterers</v>
+      </c>
+      <c r="D52" s="3">
+        <v>46292</v>
+      </c>
+      <c r="E52" s="1">
+        <v>200000</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H51"/>
+  <autoFilter ref="A1:H52"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H52"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3074,11 +3100,11 @@
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>250000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>525000</v>
+        <v>325000</v>
       </c>
     </row>
     <row r="22">
@@ -3547,11 +3573,11 @@
       </c>
       <c r="D46" s="1">
         <f>SUM(D2:D45)</f>
-        <v>406826</v>
+        <v>606826</v>
       </c>
       <c r="E46" s="1">
         <f>SUM(E2:E45)</f>
-        <v>785000</v>
+        <v>585000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹75,000.00 by Umar Sayyed (Father) for Soyarik mangal karyalay
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H53</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1327,7 +1327,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H53"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2691,10 +2691,36 @@
         <v/>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>faf0435d</v>
+      </c>
+      <c r="B53" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="D53" s="3">
+        <v>46292</v>
+      </c>
+      <c r="E53" s="1">
+        <v>75000</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H52"/>
+  <autoFilter ref="A1:H53"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H53"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3499,11 +3525,11 @@
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>90000</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
-        <v>90000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="43">
@@ -3573,11 +3599,11 @@
       </c>
       <c r="D46" s="1">
         <f>SUM(D2:D45)</f>
-        <v>606826</v>
+        <v>681826</v>
       </c>
       <c r="E46" s="1">
         <f>SUM(E2:E45)</f>
-        <v>585000</v>
+        <v>510000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Crackers — ₹5,500.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H54</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -679,356 +679,356 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>05d27deb</v>
+        <v>0cf8885b</v>
       </c>
       <c r="B14" t="str">
-        <v>Cream House Lunch</v>
+        <v>Crackers</v>
       </c>
       <c r="C14" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D14" s="1">
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v/>
+        <v>+91 86557 63847</v>
       </c>
       <c r="F14" t="str">
-        <v>Cream House Lunch</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>631875ca</v>
+        <v>05d27deb</v>
       </c>
       <c r="B15" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="C15" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D15" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v>Hall decoration</v>
+        <v>Cream House Lunch</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B16" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C16" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D16" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F16" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B17" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F17" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B18" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C18" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F18" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>766bfdf7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B19" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C19" t="str">
         <v>Miscellaneous</v>
       </c>
       <c r="D19" s="1">
-        <v>410</v>
+        <v>2609</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v/>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>209d43b7</v>
+        <v>766bfdf7</v>
       </c>
       <c r="B20" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="C20" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D20" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E20" s="2" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B21" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C21" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D21" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F21" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>dc70b2a1</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B22" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C22" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D22" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F22" t="str">
-        <v>internal expense</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B23" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C23" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D23" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F23" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B24" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C24" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D24" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F24" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>4d3bd5b1</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B25" t="str">
-        <v>Mandva</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C25" t="str">
-        <v>Decoration</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D25" s="1">
-        <v>37000</v>
+        <v>3675</v>
       </c>
       <c r="E25" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>c7e8b352</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="B26" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mandva</v>
       </c>
       <c r="C26" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D26" s="1">
-        <v>7604</v>
+        <v>37000</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B27" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B28" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B29" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B30" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C30" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B31" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D31" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
@@ -1039,113 +1039,113 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B32" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C32" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B33" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C33" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D33" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B34" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D34" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B35" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C35" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B36" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C36" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B37" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C37" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D37" s="1">
         <v>4000</v>
@@ -1159,168 +1159,188 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B38" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C38" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D38" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E38" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F38" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B39" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C39" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D39" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E39" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F39" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B40" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C40" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D40" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
       </c>
       <c r="F40" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B41" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C41" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D41" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E41" s="2" t="str">
         <v/>
       </c>
       <c r="F41" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B42" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C42" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D42" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E42" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F42" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B43" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C43" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D43" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E43" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F43" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B44" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C44" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D44" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E44" s="2" t="str">
         <v/>
       </c>
       <c r="F44" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D45" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E45" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B46" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C45" t="str">
+      <c r="C46" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D46" s="1">
         <v>9150</v>
       </c>
-      <c r="E45" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F45" t="str">
+      <c r="E46" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F45"/>
+  <autoFilter ref="A1:F46"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F46"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2753,7 +2773,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3009,74 +3029,74 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Cream House Lunch</v>
+        <v>Crackers</v>
       </c>
       <c r="B14" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C14" s="1">
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>1124</v>
+        <v>0</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>0</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="B15" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C15" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>75000</v>
+        <v>1124</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>68000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B16" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C16" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>75000</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>0</v>
+        <v>68000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -3085,17 +3105,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B18" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -3104,17 +3124,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B19" t="str">
         <v>Miscellaneous</v>
       </c>
       <c r="C19" s="1">
-        <v>410</v>
+        <v>2609</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>410</v>
+        <v>2609</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -3123,17 +3143,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="B20" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C20" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -3142,55 +3162,55 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B21" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C21" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>450000</v>
+        <v>500</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>125000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B22" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C22" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>450000</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>0</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B23" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C23" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -3199,17 +3219,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B24" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C24" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -3218,55 +3238,55 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Mandva</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B25" t="str">
-        <v>Decoration</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C25" s="1">
-        <v>37000</v>
+        <v>3675</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>5000</v>
+        <v>3675</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>32000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mandva</v>
       </c>
       <c r="B26" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C26" s="1">
-        <v>7604</v>
+        <v>37000</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>5000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
-        <v>0</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -3275,17 +3295,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -3294,17 +3314,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -3313,17 +3333,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B30" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3332,17 +3352,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C31" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3351,17 +3371,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B32" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3370,17 +3390,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B33" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C33" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3389,17 +3409,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C34" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -3408,17 +3428,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B35" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -3427,17 +3447,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B36" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -3446,10 +3466,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B37" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C37" s="1">
         <v>4000</v>
@@ -3465,55 +3485,55 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B38" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C38" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>30000</v>
+        <v>4000</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
-        <v>70000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B39" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C39" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>30000</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
-        <v>0</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B40" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C40" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -3522,17 +3542,17 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B41" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C41" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -3541,55 +3561,55 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B42" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C42" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>90000</v>
+        <v>2000</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B43" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C43" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>90000</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
-        <v>0</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B44" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C44" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
@@ -3598,17 +3618,17 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B45" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C45" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
@@ -3617,24 +3637,43 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C46" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D46" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E46" s="1">
+        <f>C46-D46</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
         <v>Total</v>
       </c>
-      <c r="C46" s="1">
-        <f>SUM(C2:C45)</f>
-        <v>1191826</v>
-      </c>
-      <c r="D46" s="1">
-        <f>SUM(D2:D45)</f>
+      <c r="C47" s="1">
+        <f>SUM(C2:C46)</f>
+        <v>1197326</v>
+      </c>
+      <c r="D47" s="1">
+        <f>SUM(D2:D46)</f>
         <v>881826</v>
       </c>
-      <c r="E46" s="1">
-        <f>SUM(E2:E45)</f>
-        <v>310000</v>
+      <c r="E47" s="1">
+        <f>SUM(E2:E46)</f>
+        <v>315500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹5,500.00 by Asif Sayyed (Son) for Crackers
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H55</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1347,7 +1347,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H55"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2763,10 +2763,36 @@
         <v/>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>37a1eaeb</v>
+      </c>
+      <c r="B55" t="str">
+        <v>0cf8885b</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Crackers</v>
+      </c>
+      <c r="D55" s="3">
+        <v>46293</v>
+      </c>
+      <c r="E55" s="1">
+        <v>5500</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G55" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H55" t="str">
+        <v>Paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H54"/>
+  <autoFilter ref="A1:H55"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H55"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3039,11 +3065,11 @@
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>5500</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>5500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3664,11 +3690,11 @@
       </c>
       <c r="D47" s="1">
         <f>SUM(D2:D46)</f>
-        <v>881826</v>
+        <v>887326</v>
       </c>
       <c r="E47" s="1">
         <f>SUM(E2:E46)</f>
-        <v>315500</v>
+        <v>310000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹10,000.00 by Asif Sayyed (Son) for Mandva
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H57</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1347,7 +1347,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2815,10 +2815,36 @@
         <v>5 th installment</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>ccf68d33</v>
+      </c>
+      <c r="B57" t="str">
+        <v>4d3bd5b1</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Mandva</v>
+      </c>
+      <c r="D57" s="3">
+        <v>46296</v>
+      </c>
+      <c r="E57" s="1">
+        <v>10000</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G57" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H57" t="str">
+        <v>second installment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
+  <autoFilter ref="A1:H57"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H57"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3319,11 +3345,11 @@
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
-        <v>32000</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="27">
@@ -3716,11 +3742,11 @@
       </c>
       <c r="D47" s="1">
         <f>SUM(D2:D46)</f>
-        <v>897326</v>
+        <v>907326</v>
       </c>
       <c r="E47" s="1">
         <f>SUM(E2:E46)</f>
-        <v>300000</v>
+        <v>290000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update budget item: Day night Flower Decoration - (hall) — ₹1,58,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -728,7 +728,7 @@
         <v>Decoration</v>
       </c>
       <c r="D16" s="1">
-        <v>143000</v>
+        <v>158000</v>
       </c>
       <c r="E16" s="2" t="str">
         <v>9536673041</v>
@@ -3151,7 +3151,7 @@
         <v>Decoration</v>
       </c>
       <c r="C16" s="1">
-        <v>143000</v>
+        <v>158000</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>68000</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="17">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="C47" s="1">
         <f>SUM(C2:C46)</f>
-        <v>1197326</v>
+        <v>1212326</v>
       </c>
       <c r="D47" s="1">
         <f>SUM(D2:D46)</f>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="E47" s="1">
         <f>SUM(E2:E46)</f>
-        <v>290000</v>
+        <v>305000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹33,000.00 by Asif Sayyed (Son) for Day night Flower Decoration - (hall)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H58</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1347,7 +1347,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H58"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2841,10 +2841,36 @@
         <v>second installment</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>a6e10a8c</v>
+      </c>
+      <c r="B58" t="str">
+        <v>631875ca</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Day night Flower Decoration - (hall)</v>
+      </c>
+      <c r="D58" s="3">
+        <v>46297</v>
+      </c>
+      <c r="E58" s="1">
+        <v>33000</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G58" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H58" t="str">
+        <v>4th installment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H57"/>
+  <autoFilter ref="A1:H58"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H58"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3155,11 +3181,11 @@
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>75000</v>
+        <v>108000</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>83000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="17">
@@ -3742,11 +3768,11 @@
       </c>
       <c r="D47" s="1">
         <f>SUM(D2:D46)</f>
-        <v>907326</v>
+        <v>940326</v>
       </c>
       <c r="E47" s="1">
         <f>SUM(E2:E46)</f>
-        <v>305000</v>
+        <v>272000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update budget item: Ganesh Bhondve Mandva + decoration — ₹39,500.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -799,19 +799,19 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>766bfdf7</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="B20" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="C20" t="str">
-        <v>Miscellaneous</v>
+        <v>Decoration</v>
       </c>
       <c r="D20" s="1">
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v/>
+        <v>9168993010</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -819,122 +819,122 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>209d43b7</v>
+        <v>766bfdf7</v>
       </c>
       <c r="B21" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="C21" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D21" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B22" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C22" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D22" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>dc70b2a1</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B23" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C23" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D23" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F23" t="str">
-        <v>internal expense</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B24" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C24" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D24" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F24" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B25" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C25" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D25" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E25" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F25" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>4d3bd5b1</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B26" t="str">
-        <v>Mandva</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C26" t="str">
-        <v>Decoration</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D26" s="1">
-        <v>37000</v>
+        <v>3675</v>
       </c>
       <c r="E26" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="27">
@@ -2667,7 +2667,7 @@
         <v>4d3bd5b1</v>
       </c>
       <c r="C51" t="str">
-        <v>Mandva</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D51" s="3">
         <v>46284</v>
@@ -2823,7 +2823,7 @@
         <v>4d3bd5b1</v>
       </c>
       <c r="C57" t="str">
-        <v>Mandva</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D57" s="3">
         <v>46296</v>
@@ -3247,36 +3247,36 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="B20" t="str">
-        <v>Miscellaneous</v>
+        <v>Decoration</v>
       </c>
       <c r="C20" s="1">
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>410</v>
+        <v>15000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>0</v>
+        <v>24500</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="B21" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C21" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -3285,55 +3285,55 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B22" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C22" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>450000</v>
+        <v>500</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>125000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B23" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C23" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>450000</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
-        <v>0</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B24" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C24" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -3342,17 +3342,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B25" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C25" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -3361,21 +3361,21 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Mandva</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B26" t="str">
-        <v>Decoration</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C26" s="1">
-        <v>37000</v>
+        <v>3675</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>3675</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
-        <v>22000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C47" s="1">
         <f>SUM(C2:C46)</f>
-        <v>1212326</v>
+        <v>1214826</v>
       </c>
       <c r="D47" s="1">
         <f>SUM(D2:D46)</f>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="E47" s="1">
         <f>SUM(E2:E46)</f>
-        <v>272000</v>
+        <v>274500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: miscellaneous ratjaka (chicken, tags, bartan) — ₹5,412.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H58</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -939,116 +939,116 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>c7e8b352</v>
+        <v>a1def8e4</v>
       </c>
       <c r="B27" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="C27" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D27" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B28" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B29" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B30" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B31" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C31" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B32" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D32" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
@@ -1059,113 +1059,113 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B33" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C33" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B34" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C34" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D34" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B35" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D35" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B36" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C36" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B37" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C37" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D37" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B38" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C38" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D38" s="1">
         <v>4000</v>
@@ -1179,168 +1179,188 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B39" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C39" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D39" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E39" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F39" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B40" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C40" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D40" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E40" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F40" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B41" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C41" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D41" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E41" s="2" t="str">
         <v/>
       </c>
       <c r="F41" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B42" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C42" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D42" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E42" s="2" t="str">
         <v/>
       </c>
       <c r="F42" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B43" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C43" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D43" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E43" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F43" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B44" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C44" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D44" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E44" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F44" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B45" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C45" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D45" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E45" s="2" t="str">
         <v/>
       </c>
       <c r="F45" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D46" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E46" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B46" t="str">
+      <c r="B47" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C46" t="str">
+      <c r="C47" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D47" s="1">
         <v>9150</v>
       </c>
-      <c r="E46" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F46" t="str">
+      <c r="E47" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F46"/>
+  <autoFilter ref="A1:F47"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F47"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2877,7 +2897,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3380,36 +3400,36 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="B27" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C27" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>0</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
-        <v>0</v>
+        <v>5412</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -3418,17 +3438,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -3437,17 +3457,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3456,17 +3476,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B31" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3475,17 +3495,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C32" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3494,17 +3514,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B33" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3513,17 +3533,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B34" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C34" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -3532,17 +3552,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C35" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -3551,17 +3571,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B36" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -3570,17 +3590,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B37" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C37" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -3589,10 +3609,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B38" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C38" s="1">
         <v>4000</v>
@@ -3608,55 +3628,55 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B39" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C39" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>40000</v>
+        <v>4000</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
-        <v>60000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B40" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C40" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>40000</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
-        <v>0</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B41" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C41" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -3665,17 +3685,17 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B42" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C42" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
@@ -3684,55 +3704,55 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B43" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C43" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>90000</v>
+        <v>2000</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B44" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C44" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>90000</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
-        <v>0</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B45" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C45" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
@@ -3741,17 +3761,17 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B46" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C46" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
@@ -3760,24 +3780,43 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C47" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D47" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E47" s="1">
+        <f>C47-D47</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
         <v>Total</v>
       </c>
-      <c r="C47" s="1">
-        <f>SUM(C2:C46)</f>
-        <v>1214826</v>
-      </c>
-      <c r="D47" s="1">
-        <f>SUM(D2:D46)</f>
+      <c r="C48" s="1">
+        <f>SUM(C2:C47)</f>
+        <v>1220238</v>
+      </c>
+      <c r="D48" s="1">
+        <f>SUM(D2:D47)</f>
         <v>940326</v>
       </c>
-      <c r="E47" s="1">
-        <f>SUM(E2:E46)</f>
-        <v>274500</v>
+      <c r="E48" s="1">
+        <f>SUM(E2:E47)</f>
+        <v>279912</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹5,412.00 by Asif Sayyed (Son) for miscellaneous ratjaka (chicken, tags, bartan)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H59</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1367,7 +1367,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2887,10 +2887,36 @@
         <v>4th installment</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>718175b7</v>
+      </c>
+      <c r="B59" t="str">
+        <v>a1def8e4</v>
+      </c>
+      <c r="C59" t="str">
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+      </c>
+      <c r="D59" s="3">
+        <v>46297</v>
+      </c>
+      <c r="E59" s="1">
+        <v>5412</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G59" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H59" t="str">
+        <v>paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H58"/>
+  <autoFilter ref="A1:H59"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H59"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3410,11 +3436,11 @@
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>5412</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
-        <v>5412</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -3807,11 +3833,11 @@
       </c>
       <c r="D48" s="1">
         <f>SUM(D2:D47)</f>
-        <v>940326</v>
+        <v>945738</v>
       </c>
       <c r="E48" s="1">
         <f>SUM(E2:E47)</f>
-        <v>279912</v>
+        <v>274500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹15,000.00 by Umar Sayyed (Father) for Soyarik mangal karyalay
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H60</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1367,7 +1367,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2913,10 +2913,36 @@
         <v>paid</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>fc7adcbd</v>
+      </c>
+      <c r="B60" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="D60" s="3">
+        <v>46300</v>
+      </c>
+      <c r="E60" s="1">
+        <v>15000</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H60" t="str">
+        <v>payment done</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H59"/>
+  <autoFilter ref="A1:H60"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H60"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3759,11 +3785,11 @@
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>90000</v>
+        <v>105000</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -3833,11 +3859,11 @@
       </c>
       <c r="D48" s="1">
         <f>SUM(D2:D47)</f>
-        <v>945738</v>
+        <v>960738</v>
       </c>
       <c r="E48" s="1">
         <f>SUM(E2:E47)</f>
-        <v>274500</v>
+        <v>259500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: chair arrangment soyarik gardan — ₹3,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H60</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -659,16 +659,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2a74d868</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="B13" t="str">
-        <v>Colour &amp; plumber</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="C13" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D13" s="1">
-        <v>800</v>
+        <v>3000</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
@@ -679,19 +679,19 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>0cf8885b</v>
+        <v>2a74d868</v>
       </c>
       <c r="B14" t="str">
-        <v>Crackers</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="C14" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D14" s="1">
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>+91 86557 63847</v>
+        <v/>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -699,139 +699,139 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>05d27deb</v>
+        <v>0cf8885b</v>
       </c>
       <c r="B15" t="str">
-        <v>Cream House Lunch</v>
+        <v>Crackers</v>
       </c>
       <c r="C15" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D15" s="1">
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v/>
+        <v>+91 86557 63847</v>
       </c>
       <c r="F15" t="str">
-        <v>Cream House Lunch</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>631875ca</v>
+        <v>05d27deb</v>
       </c>
       <c r="B16" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="C16" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D16" s="1">
-        <v>158000</v>
+        <v>1124</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>Hall decoration</v>
+        <v>Cream House Lunch</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B17" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C17" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D17" s="1">
-        <v>12150</v>
+        <v>158000</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F17" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B18" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F18" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B19" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C19" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F19" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>4d3bd5b1</v>
+        <v>070f7b33</v>
       </c>
       <c r="B20" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C20" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D20" s="1">
-        <v>39500</v>
+        <v>2609</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v>9168993010</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>766bfdf7</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="B21" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="C21" t="str">
-        <v>Miscellaneous</v>
+        <v>Decoration</v>
       </c>
       <c r="D21" s="1">
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v/>
+        <v>9168993010</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -839,236 +839,236 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>209d43b7</v>
+        <v>766bfdf7</v>
       </c>
       <c r="B22" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="C22" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D22" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B23" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C23" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D23" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F23" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>dc70b2a1</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B24" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C24" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D24" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F24" t="str">
-        <v>internal expense</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B25" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C25" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D25" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E25" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F25" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B26" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C26" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D26" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E26" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F26" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>a1def8e4</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B27" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C27" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D27" s="1">
-        <v>5412</v>
+        <v>3675</v>
       </c>
       <c r="E27" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F27" t="str">
-        <v/>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>c7e8b352</v>
+        <v>a1def8e4</v>
       </c>
       <c r="B28" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="C28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D28" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B29" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B30" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B31" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B32" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C32" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B33" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D33" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
@@ -1079,113 +1079,113 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B34" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C34" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B35" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C35" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D35" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B36" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C36" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D36" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B37" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C37" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D37" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B38" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C38" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D38" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B39" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C39" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D39" s="1">
         <v>4000</v>
@@ -1199,168 +1199,188 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B40" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C40" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D40" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E40" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F40" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B41" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C41" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D41" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E41" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F41" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B42" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C42" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D42" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E42" s="2" t="str">
         <v/>
       </c>
       <c r="F42" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B43" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C43" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D43" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E43" s="2" t="str">
         <v/>
       </c>
       <c r="F43" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B44" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C44" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D44" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E44" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F44" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B45" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C45" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D45" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E45" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F45" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B46" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C46" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D46" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E46" s="2" t="str">
         <v/>
       </c>
       <c r="F46" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D47" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E47" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B47" t="str">
+      <c r="B48" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C47" t="str">
+      <c r="C48" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D48" s="1">
         <v>9150</v>
       </c>
-      <c r="E47" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F47" t="str">
+      <c r="E48" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F47"/>
+  <autoFilter ref="A1:F48"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F48"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2949,7 +2969,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3186,36 +3206,36 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Colour &amp; plumber</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="B13" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C13" s="1">
-        <v>800</v>
+        <v>3000</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Crackers</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="B14" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C14" s="1">
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -3224,17 +3244,17 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Cream House Lunch</v>
+        <v>Crackers</v>
       </c>
       <c r="B15" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C15" s="1">
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -3243,55 +3263,55 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="B16" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C16" s="1">
-        <v>158000</v>
+        <v>1124</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>108000</v>
+        <v>1124</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B17" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C17" s="1">
-        <v>12150</v>
+        <v>158000</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>108000</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>0</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -3300,17 +3320,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B19" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -3319,55 +3339,55 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B20" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C20" s="1">
-        <v>39500</v>
+        <v>2609</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2609</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>24500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="B21" t="str">
-        <v>Miscellaneous</v>
+        <v>Decoration</v>
       </c>
       <c r="C21" s="1">
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>410</v>
+        <v>15000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>0</v>
+        <v>24500</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="B22" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C22" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -3376,55 +3396,55 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B23" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C23" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>450000</v>
+        <v>500</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
-        <v>125000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B24" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C24" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>450000</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
-        <v>0</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B25" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C25" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -3433,17 +3453,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B26" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C26" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -3452,17 +3472,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B27" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C27" s="1">
-        <v>5412</v>
+        <v>3675</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>5412</v>
+        <v>3675</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -3471,17 +3491,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="B28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C28" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -3490,17 +3510,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -3509,17 +3529,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3528,17 +3548,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3547,17 +3567,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B32" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3566,17 +3586,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C33" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3585,17 +3605,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B34" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -3604,17 +3624,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B35" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C35" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -3623,17 +3643,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B36" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C36" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -3642,17 +3662,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B37" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C37" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -3661,17 +3681,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B38" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C38" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -3680,10 +3700,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B39" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C39" s="1">
         <v>4000</v>
@@ -3699,55 +3719,55 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B40" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C40" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>40000</v>
+        <v>4000</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
-        <v>60000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B41" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C41" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>40000</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
-        <v>0</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B42" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C42" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
@@ -3756,17 +3776,17 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B43" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C43" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
@@ -3775,17 +3795,17 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B44" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C44" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
@@ -3794,17 +3814,17 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B45" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C45" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
@@ -3813,17 +3833,17 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B46" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C46" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
@@ -3832,17 +3852,17 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B47" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C47" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
@@ -3851,24 +3871,43 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C48" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D48" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E48" s="1">
+        <f>C48-D48</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
         <v>Total</v>
       </c>
-      <c r="C48" s="1">
-        <f>SUM(C2:C47)</f>
-        <v>1220238</v>
-      </c>
-      <c r="D48" s="1">
-        <f>SUM(D2:D47)</f>
+      <c r="C49" s="1">
+        <f>SUM(C2:C48)</f>
+        <v>1223238</v>
+      </c>
+      <c r="D49" s="1">
+        <f>SUM(D2:D48)</f>
         <v>960738</v>
       </c>
-      <c r="E48" s="1">
-        <f>SUM(E2:E47)</f>
-        <v>259500</v>
+      <c r="E49" s="1">
+        <f>SUM(E2:E48)</f>
+        <v>262500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E49"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹2,000.00 by Umar Sayyed (Father) for chair arrangment soyarik gardan
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H61</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1387,7 +1387,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H61"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2959,10 +2959,36 @@
         <v>payment done</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>384605f7</v>
+      </c>
+      <c r="B61" t="str">
+        <v>22ff3fb2</v>
+      </c>
+      <c r="C61" t="str">
+        <v>chair arrangment soyarik gardan</v>
+      </c>
+      <c r="D61" s="3">
+        <v>46300</v>
+      </c>
+      <c r="E61" s="1">
+        <v>2000</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H60"/>
+  <autoFilter ref="A1:H61"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3216,11 +3242,11 @@
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>3000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="14">
@@ -3898,11 +3924,11 @@
       </c>
       <c r="D49" s="1">
         <f>SUM(D2:D48)</f>
-        <v>960738</v>
+        <v>962738</v>
       </c>
       <c r="E49" s="1">
         <f>SUM(E2:E48)</f>
-        <v>262500</v>
+        <v>260500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: tampo traveller — ₹7,500.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H61</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1339,48 +1339,68 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B47" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C47" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D47" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E47" s="2" t="str">
         <v/>
       </c>
       <c r="F47" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D48" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E48" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B48" t="str">
+      <c r="B49" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C48" t="str">
+      <c r="C49" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D49" s="1">
         <v>9150</v>
       </c>
-      <c r="E48" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F48" t="str">
+      <c r="E49" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F48"/>
+  <autoFilter ref="A1:F49"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F49"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2995,7 +3015,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3878,36 +3898,36 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B47" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C47" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>0</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
-        <v>0</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B48" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C48" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
@@ -3916,24 +3936,43 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C49" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D49" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E49" s="1">
+        <f>C49-D49</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
         <v>Total</v>
       </c>
-      <c r="C49" s="1">
-        <f>SUM(C2:C48)</f>
-        <v>1223238</v>
-      </c>
-      <c r="D49" s="1">
-        <f>SUM(D2:D48)</f>
+      <c r="C50" s="1">
+        <f>SUM(C2:C49)</f>
+        <v>1230738</v>
+      </c>
+      <c r="D50" s="1">
+        <f>SUM(D2:D49)</f>
         <v>962738</v>
       </c>
-      <c r="E49" s="1">
-        <f>SUM(E2:E48)</f>
-        <v>260500</v>
+      <c r="E50" s="1">
+        <f>SUM(E2:E49)</f>
+        <v>268000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E50"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹7,500.00 by Umar Sayyed (Father) for tampo traveller
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H62</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1407,7 +1407,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H62"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3005,10 +3005,36 @@
         <v/>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>d08ebf7d</v>
+      </c>
+      <c r="B62" t="str">
+        <v>9b3747da</v>
+      </c>
+      <c r="C62" t="str">
+        <v>tampo traveller</v>
+      </c>
+      <c r="D62" s="3">
+        <v>46300</v>
+      </c>
+      <c r="E62" s="1">
+        <v>7500</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G62" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H62" t="str">
+        <v>cash</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H61"/>
+  <autoFilter ref="A1:H62"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H62"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3908,11 +3934,11 @@
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
-        <v>7500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -3963,11 +3989,11 @@
       </c>
       <c r="D50" s="1">
         <f>SUM(D2:D49)</f>
-        <v>962738</v>
+        <v>970238</v>
       </c>
       <c r="E50" s="1">
         <f>SUM(E2:E49)</f>
-        <v>268000</v>
+        <v>260500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹2,400.00 by Asif Sayyed (Son) for Ganesh Bhondve Mandva + decoration
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H63</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1407,7 +1407,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3031,10 +3031,36 @@
         <v>cash</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>3adcd8de</v>
+      </c>
+      <c r="B63" t="str">
+        <v>4d3bd5b1</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Ganesh Bhondve Mandva + decoration</v>
+      </c>
+      <c r="D63" s="3">
+        <v>46302</v>
+      </c>
+      <c r="E63" s="1">
+        <v>2400</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G63" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H63" t="str">
+        <v>Final payment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H62"/>
+  <autoFilter ref="A1:H63"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H63"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3440,11 +3466,11 @@
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>17400</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>24500</v>
+        <v>22100</v>
       </c>
     </row>
     <row r="22">
@@ -3989,11 +4015,11 @@
       </c>
       <c r="D50" s="1">
         <f>SUM(D2:D49)</f>
-        <v>970238</v>
+        <v>972638</v>
       </c>
       <c r="E50" s="1">
         <f>SUM(E2:E49)</f>
-        <v>260500</v>
+        <v>258100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹20,000.00 by Asif Sayyed (Son) for Day night Flower Decoration - (hall)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H64</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1407,7 +1407,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3057,10 +3057,36 @@
         <v>Final payment</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>4f298a0d</v>
+      </c>
+      <c r="B64" t="str">
+        <v>631875ca</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Day night Flower Decoration - (hall)</v>
+      </c>
+      <c r="D64" s="3">
+        <v>46302</v>
+      </c>
+      <c r="E64" s="1">
+        <v>20000</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G64" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H64" t="str">
+        <v>Installment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H63"/>
+  <autoFilter ref="A1:H64"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H64"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3390,11 +3416,11 @@
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>108000</v>
+        <v>128000</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>50000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="18">
@@ -4015,11 +4041,11 @@
       </c>
       <c r="D50" s="1">
         <f>SUM(D2:D49)</f>
-        <v>972638</v>
+        <v>992638</v>
       </c>
       <c r="E50" s="1">
         <f>SUM(E2:E49)</f>
-        <v>258100</v>
+        <v>238100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update payment: ₹24,000.00 by Asif Sayyed (Son) for Ganesh Bhondve Mandva + decoration
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -3045,7 +3045,7 @@
         <v>46302</v>
       </c>
       <c r="E63" s="1">
-        <v>2400</v>
+        <v>24000</v>
       </c>
       <c r="F63" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3492,11 +3492,11 @@
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>17400</v>
+        <v>39000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>22100</v>
+        <v>500</v>
       </c>
     </row>
     <row r="22">
@@ -4041,11 +4041,11 @@
       </c>
       <c r="D50" s="1">
         <f>SUM(D2:D49)</f>
-        <v>992638</v>
+        <v>1014238</v>
       </c>
       <c r="E50" s="1">
         <f>SUM(E2:E49)</f>
-        <v>238100</v>
+        <v>216500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update budget item: Day night Flower Decoration - (hall) — ₹1,61,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -748,7 +748,7 @@
         <v>Decoration</v>
       </c>
       <c r="D17" s="1">
-        <v>158000</v>
+        <v>161000</v>
       </c>
       <c r="E17" s="2" t="str">
         <v>9536673041</v>
@@ -3412,7 +3412,7 @@
         <v>Decoration</v>
       </c>
       <c r="C17" s="1">
-        <v>158000</v>
+        <v>161000</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
@@ -3420,7 +3420,7 @@
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>30000</v>
+        <v>33000</v>
       </c>
     </row>
     <row r="18">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C50" s="1">
         <f>SUM(C2:C49)</f>
-        <v>1230738</v>
+        <v>1233738</v>
       </c>
       <c r="D50" s="1">
         <f>SUM(D2:D49)</f>
@@ -4045,7 +4045,7 @@
       </c>
       <c r="E50" s="1">
         <f>SUM(E2:E49)</f>
-        <v>216500</v>
+        <v>219500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹1,25,000.00 by Umar Sayyed (Father) for Huseni Caterers
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H66</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1407,7 +1407,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3109,10 +3109,36 @@
         <v>Payment done</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>658c49d2</v>
+      </c>
+      <c r="B66" t="str">
+        <v>168b7bbd</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Huseni Caterers</v>
+      </c>
+      <c r="D66" s="3">
+        <v>46303</v>
+      </c>
+      <c r="E66" s="1">
+        <v>125000</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H66" t="str">
+        <v>Final payment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H65"/>
+  <autoFilter ref="A1:H66"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H66"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3575,11 +3601,11 @@
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>450000</v>
+        <v>575000</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
-        <v>125000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -4067,11 +4093,11 @@
       </c>
       <c r="D50" s="1">
         <f>SUM(D2:D49)</f>
-        <v>1047238</v>
+        <v>1172238</v>
       </c>
       <c r="E50" s="1">
         <f>SUM(E2:E49)</f>
-        <v>186500</v>
+        <v>61500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹30,000.00 by Asif Sayyed (Son) for Pratap films and Photography
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H67</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1407,7 +1407,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3135,10 +3135,36 @@
         <v>Final payment</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>80e653df</v>
+      </c>
+      <c r="B67" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D67" s="3">
+        <v>46303</v>
+      </c>
+      <c r="E67" s="1">
+        <v>30000</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G67" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H67" t="str">
+        <v>Second last installment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H66"/>
+  <autoFilter ref="A1:H67"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H67"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3924,11 +3950,11 @@
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>40000</v>
+        <v>70000</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
-        <v>60000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="42">
@@ -4093,11 +4119,11 @@
       </c>
       <c r="D50" s="1">
         <f>SUM(D2:D49)</f>
-        <v>1172238</v>
+        <v>1202238</v>
       </c>
       <c r="E50" s="1">
         <f>SUM(E2:E49)</f>
-        <v>61500</v>
+        <v>31500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: car decoration, Dj, Petrol, Haldi Celender — ₹30,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H67</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -659,16 +659,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>22ff3fb2</v>
+        <v>c1c67a32</v>
       </c>
       <c r="B13" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>car decoration, Dj, Petrol, Haldi Celender</v>
       </c>
       <c r="C13" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Decoration</v>
       </c>
       <c r="D13" s="1">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
@@ -679,16 +679,16 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2a74d868</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="B14" t="str">
-        <v>Colour &amp; plumber</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="C14" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D14" s="1">
-        <v>800</v>
+        <v>3000</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
@@ -699,19 +699,19 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>0cf8885b</v>
+        <v>2a74d868</v>
       </c>
       <c r="B15" t="str">
-        <v>Crackers</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="C15" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D15" s="1">
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>+91 86557 63847</v>
+        <v/>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -719,139 +719,139 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>05d27deb</v>
+        <v>0cf8885b</v>
       </c>
       <c r="B16" t="str">
-        <v>Cream House Lunch</v>
+        <v>Crackers</v>
       </c>
       <c r="C16" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D16" s="1">
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v/>
+        <v>+91 86557 63847</v>
       </c>
       <c r="F16" t="str">
-        <v>Cream House Lunch</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>631875ca</v>
+        <v>05d27deb</v>
       </c>
       <c r="B17" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="C17" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D17" s="1">
-        <v>161000</v>
+        <v>1124</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F17" t="str">
-        <v>Hall decoration</v>
+        <v>Cream House Lunch</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B18" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C18" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D18" s="1">
-        <v>12150</v>
+        <v>161000</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F18" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B19" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F19" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B20" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C20" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F20" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>4d3bd5b1</v>
+        <v>070f7b33</v>
       </c>
       <c r="B21" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C21" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D21" s="1">
-        <v>39500</v>
+        <v>2609</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v>9168993010</v>
+        <v/>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>766bfdf7</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="B22" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="C22" t="str">
-        <v>Miscellaneous</v>
+        <v>Decoration</v>
       </c>
       <c r="D22" s="1">
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v/>
+        <v>9168993010</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -859,236 +859,236 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>209d43b7</v>
+        <v>766bfdf7</v>
       </c>
       <c r="B23" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="C23" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D23" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B24" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C24" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D24" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F24" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>dc70b2a1</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B25" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C25" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D25" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E25" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F25" t="str">
-        <v>internal expense</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B26" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C26" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D26" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E26" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F26" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B27" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C27" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D27" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E27" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F27" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>a1def8e4</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B28" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C28" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D28" s="1">
-        <v>5412</v>
+        <v>3675</v>
       </c>
       <c r="E28" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>c7e8b352</v>
+        <v>a1def8e4</v>
       </c>
       <c r="B29" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="C29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D29" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B30" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B31" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B32" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B33" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C33" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B34" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D34" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
@@ -1099,113 +1099,113 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B35" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C35" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B36" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C36" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D36" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B37" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C37" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D37" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B38" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C38" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D38" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B39" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C39" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D39" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B40" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C40" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D40" s="1">
         <v>4000</v>
@@ -1219,188 +1219,208 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B41" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C41" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D41" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E41" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F41" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B42" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C42" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D42" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E42" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F42" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B43" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C43" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D43" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E43" s="2" t="str">
         <v/>
       </c>
       <c r="F43" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B44" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C44" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D44" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E44" s="2" t="str">
         <v/>
       </c>
       <c r="F44" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B45" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C45" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D45" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E45" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F45" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B46" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C46" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D46" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E46" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F46" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B47" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C47" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D47" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E47" s="2" t="str">
         <v/>
       </c>
       <c r="F47" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B48" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C48" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D48" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E48" s="2" t="str">
         <v/>
       </c>
       <c r="F48" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D49" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E49" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B49" t="str">
+      <c r="B50" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C49" t="str">
+      <c r="C50" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D50" s="1">
         <v>9150</v>
       </c>
-      <c r="E49" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F49" t="str">
+      <c r="E50" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F49"/>
+  <autoFilter ref="A1:F50"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F50"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3171,7 +3191,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3408,55 +3428,55 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>car decoration, Dj, Petrol, Haldi Celender</v>
       </c>
       <c r="B13" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Decoration</v>
       </c>
       <c r="C13" s="1">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>1000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Colour &amp; plumber</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="B14" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C14" s="1">
-        <v>800</v>
+        <v>3000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>800</v>
+        <v>2000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Crackers</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="B15" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C15" s="1">
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -3465,17 +3485,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Cream House Lunch</v>
+        <v>Crackers</v>
       </c>
       <c r="B16" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C16" s="1">
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -3484,17 +3504,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="B17" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C17" s="1">
-        <v>161000</v>
+        <v>1124</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>161000</v>
+        <v>1124</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -3503,17 +3523,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B18" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C18" s="1">
-        <v>12150</v>
+        <v>161000</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>161000</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -3522,17 +3542,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -3541,17 +3561,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B20" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -3560,55 +3580,55 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B21" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C21" s="1">
-        <v>39500</v>
+        <v>2609</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>39000</v>
+        <v>2609</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="B22" t="str">
-        <v>Miscellaneous</v>
+        <v>Decoration</v>
       </c>
       <c r="C22" s="1">
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>410</v>
+        <v>39000</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="B23" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C23" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -3617,17 +3637,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B24" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C24" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -3636,17 +3656,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B25" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C25" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -3655,17 +3675,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B26" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C26" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -3674,17 +3694,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B27" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C27" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -3693,17 +3713,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B28" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C28" s="1">
-        <v>5412</v>
+        <v>3675</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>5412</v>
+        <v>3675</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -3712,17 +3732,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="B29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C29" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -3731,17 +3751,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3750,17 +3770,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3769,17 +3789,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3788,17 +3808,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B33" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3807,17 +3827,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C34" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -3826,17 +3846,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B35" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -3845,17 +3865,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B36" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C36" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -3864,17 +3884,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B37" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C37" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -3883,17 +3903,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B38" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C38" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -3902,17 +3922,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B39" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C39" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -3921,10 +3941,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B40" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C40" s="1">
         <v>4000</v>
@@ -3940,55 +3960,55 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B41" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C41" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B42" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C42" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B43" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C43" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
@@ -3997,17 +4017,17 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B44" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C44" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
@@ -4016,17 +4036,17 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B45" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C45" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
@@ -4035,17 +4055,17 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B46" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C46" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
@@ -4054,17 +4074,17 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B47" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C47" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
@@ -4073,17 +4093,17 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B48" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C48" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
@@ -4092,17 +4112,17 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B49" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C49" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
@@ -4111,24 +4131,43 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C50" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D50" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E50" s="1">
+        <f>C50-D50</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
         <v>Total</v>
       </c>
-      <c r="C50" s="1">
-        <f>SUM(C2:C49)</f>
-        <v>1233738</v>
-      </c>
-      <c r="D50" s="1">
-        <f>SUM(D2:D49)</f>
+      <c r="C51" s="1">
+        <f>SUM(C2:C50)</f>
+        <v>1263738</v>
+      </c>
+      <c r="D51" s="1">
+        <f>SUM(D2:D50)</f>
         <v>1202238</v>
       </c>
-      <c r="E50" s="1">
-        <f>SUM(E2:E49)</f>
-        <v>31500</v>
+      <c r="E51" s="1">
+        <f>SUM(E2:E50)</f>
+        <v>61500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹30,000.00 by Asif Sayyed (Son) for car decoration, Dj, Petrol, Haldi Celender
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H68</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1427,7 +1427,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2975,45 +2975,45 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>fc7adcbd</v>
+        <v>09899d1e</v>
       </c>
       <c r="B60" t="str">
-        <v>04ece648</v>
+        <v>c1c67a32</v>
       </c>
       <c r="C60" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>car decoration, Dj, Petrol, Haldi Celender</v>
       </c>
       <c r="D60" s="3">
-        <v>46300</v>
+        <v>46299</v>
       </c>
       <c r="E60" s="1">
-        <v>15000</v>
+        <v>30000</v>
       </c>
       <c r="F60" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G60" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H60" t="str">
-        <v>payment done</v>
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>384605f7</v>
+        <v>fc7adcbd</v>
       </c>
       <c r="B61" t="str">
-        <v>22ff3fb2</v>
+        <v>04ece648</v>
       </c>
       <c r="C61" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="D61" s="3">
         <v>46300</v>
       </c>
       <c r="E61" s="1">
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="F61" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3022,24 +3022,24 @@
         <v>Cash</v>
       </c>
       <c r="H61" t="str">
-        <v/>
+        <v>payment done</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>d08ebf7d</v>
+        <v>384605f7</v>
       </c>
       <c r="B62" t="str">
-        <v>9b3747da</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C62" t="str">
-        <v>tampo traveller</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D62" s="3">
         <v>46300</v>
       </c>
       <c r="E62" s="1">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="F62" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3048,50 +3048,50 @@
         <v>Cash</v>
       </c>
       <c r="H62" t="str">
-        <v>cash</v>
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>3adcd8de</v>
+        <v>d08ebf7d</v>
       </c>
       <c r="B63" t="str">
-        <v>4d3bd5b1</v>
+        <v>9b3747da</v>
       </c>
       <c r="C63" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>tampo traveller</v>
       </c>
       <c r="D63" s="3">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E63" s="1">
-        <v>24000</v>
+        <v>7500</v>
       </c>
       <c r="F63" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G63" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H63" t="str">
-        <v>Final payment</v>
+        <v>cash</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>4f298a0d</v>
+        <v>3adcd8de</v>
       </c>
       <c r="B64" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C64" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D64" s="3">
         <v>46302</v>
       </c>
       <c r="E64" s="1">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="F64" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3100,12 +3100,12 @@
         <v>UPI</v>
       </c>
       <c r="H64" t="str">
-        <v>Installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>da6b0ec5</v>
+        <v>4f298a0d</v>
       </c>
       <c r="B65" t="str">
         <v>631875ca</v>
@@ -3114,10 +3114,10 @@
         <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D65" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E65" s="1">
-        <v>33000</v>
+        <v>20000</v>
       </c>
       <c r="F65" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3126,65 +3126,91 @@
         <v>UPI</v>
       </c>
       <c r="H65" t="str">
-        <v>Payment done</v>
+        <v>Installment</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B66" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C66" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D66" s="3">
         <v>46303</v>
       </c>
       <c r="E66" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F66" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G66" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H66" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B67" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C67" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D67" s="3">
         <v>46303</v>
       </c>
       <c r="E67" s="1">
+        <v>125000</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G67" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H67" t="str">
+        <v>Final payment</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>80e653df</v>
+      </c>
+      <c r="B68" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D68" s="3">
+        <v>46303</v>
+      </c>
+      <c r="E68" s="1">
         <v>30000</v>
       </c>
-      <c r="F67" t="str">
-        <v>Asif Sayyed (Son)</v>
-      </c>
-      <c r="G67" t="str">
-        <v>UPI</v>
-      </c>
-      <c r="H67" t="str">
+      <c r="F68" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G68" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H68" t="str">
         <v>Second last installment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H67"/>
+  <autoFilter ref="A1:H68"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H68"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3438,11 +3464,11 @@
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4158,11 +4184,11 @@
       </c>
       <c r="D51" s="1">
         <f>SUM(D2:D50)</f>
-        <v>1202238</v>
+        <v>1232238</v>
       </c>
       <c r="E51" s="1">
         <f>SUM(E2:E50)</f>
-        <v>61500</v>
+        <v>31500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹1,000.00 by Umar Sayyed (Father) for chair arrangment soyarik gardan
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H69</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1427,7 +1427,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3207,10 +3207,36 @@
         <v>Second last installment</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>79cb1a7e</v>
+      </c>
+      <c r="B69" t="str">
+        <v>22ff3fb2</v>
+      </c>
+      <c r="C69" t="str">
+        <v>chair arrangment soyarik gardan</v>
+      </c>
+      <c r="D69" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E69" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G69" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H69" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H68"/>
+  <autoFilter ref="A1:H69"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H69"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3483,11 +3509,11 @@
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -4184,11 +4210,11 @@
       </c>
       <c r="D51" s="1">
         <f>SUM(D2:D50)</f>
-        <v>1232238</v>
+        <v>1233238</v>
       </c>
       <c r="E51" s="1">
         <f>SUM(E2:E50)</f>
-        <v>31500</v>
+        <v>30500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹500.00 by Asif Sayyed (Son) for Ganesh Bhondve Mandva + decoration
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H70</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1427,7 +1427,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3131,19 +3131,19 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>da6b0ec5</v>
+        <v>3e780b94</v>
       </c>
       <c r="B66" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C66" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D66" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E66" s="1">
-        <v>33000</v>
+        <v>500</v>
       </c>
       <c r="F66" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3152,91 +3152,117 @@
         <v>UPI</v>
       </c>
       <c r="H66" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B67" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C67" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D67" s="3">
         <v>46303</v>
       </c>
       <c r="E67" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F67" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G67" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H67" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B68" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C68" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D68" s="3">
         <v>46303</v>
       </c>
       <c r="E68" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F68" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G68" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H68" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
+        <v>80e653df</v>
+      </c>
+      <c r="B69" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D69" s="3">
+        <v>46303</v>
+      </c>
+      <c r="E69" s="1">
+        <v>30000</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G69" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H69" t="str">
+        <v>Second last installment</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
         <v>79cb1a7e</v>
       </c>
-      <c r="B69" t="str">
+      <c r="B70" t="str">
         <v>22ff3fb2</v>
       </c>
-      <c r="C69" t="str">
+      <c r="C70" t="str">
         <v>chair arrangment soyarik gardan</v>
       </c>
-      <c r="D69" s="3">
+      <c r="D70" s="3">
         <v>46306</v>
       </c>
-      <c r="E69" s="1">
+      <c r="E70" s="1">
         <v>1000</v>
       </c>
-      <c r="F69" t="str">
+      <c r="F70" t="str">
         <v>Umar Sayyed (Father)</v>
       </c>
-      <c r="G69" t="str">
+      <c r="G70" t="str">
         <v>Cash</v>
       </c>
-      <c r="H69" t="str">
+      <c r="H70" t="str">
         <v>final payment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H69"/>
+  <autoFilter ref="A1:H70"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H70"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3661,11 +3687,11 @@
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>39000</v>
+        <v>39500</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -4210,11 +4236,11 @@
       </c>
       <c r="D51" s="1">
         <f>SUM(D2:D50)</f>
-        <v>1233238</v>
+        <v>1233738</v>
       </c>
       <c r="E51" s="1">
         <f>SUM(E2:E50)</f>
-        <v>30500</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Delete payment ₹500.00 by Asif Sayyed (Son)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H70</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1427,7 +1427,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H70"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3131,7 +3131,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>3e780b94</v>
+        <v>141e8fbb</v>
       </c>
       <c r="B66" t="str">
         <v>4d3bd5b1</v>
@@ -3152,24 +3152,24 @@
         <v>UPI</v>
       </c>
       <c r="H66" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>141e8fbb</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B67" t="str">
-        <v>4d3bd5b1</v>
+        <v>631875ca</v>
       </c>
       <c r="C67" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D67" s="3">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E67" s="1">
-        <v>500</v>
+        <v>33000</v>
       </c>
       <c r="F67" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3178,117 +3178,91 @@
         <v>UPI</v>
       </c>
       <c r="H67" t="str">
-        <v>paid</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>da6b0ec5</v>
+        <v>658c49d2</v>
       </c>
       <c r="B68" t="str">
-        <v>631875ca</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C68" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D68" s="3">
         <v>46303</v>
       </c>
       <c r="E68" s="1">
-        <v>33000</v>
+        <v>125000</v>
       </c>
       <c r="F68" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G68" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H68" t="str">
-        <v>Payment done</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>658c49d2</v>
+        <v>80e653df</v>
       </c>
       <c r="B69" t="str">
-        <v>168b7bbd</v>
+        <v>beb44857</v>
       </c>
       <c r="C69" t="str">
-        <v>Huseni Caterers</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D69" s="3">
         <v>46303</v>
       </c>
       <c r="E69" s="1">
-        <v>125000</v>
+        <v>30000</v>
       </c>
       <c r="F69" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G69" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H69" t="str">
-        <v>Final payment</v>
+        <v>Second last installment</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>80e653df</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B70" t="str">
-        <v>beb44857</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C70" t="str">
-        <v>Pratap films and Photography</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D70" s="3">
-        <v>46303</v>
+        <v>46306</v>
       </c>
       <c r="E70" s="1">
-        <v>30000</v>
+        <v>1000</v>
       </c>
       <c r="F70" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G70" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H70" t="str">
-        <v>Second last installment</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="str">
-        <v>79cb1a7e</v>
-      </c>
-      <c r="B71" t="str">
-        <v>22ff3fb2</v>
-      </c>
-      <c r="C71" t="str">
-        <v>chair arrangment soyarik gardan</v>
-      </c>
-      <c r="D71" s="3">
-        <v>46306</v>
-      </c>
-      <c r="E71" s="1">
-        <v>1000</v>
-      </c>
-      <c r="F71" t="str">
-        <v>Umar Sayyed (Father)</v>
-      </c>
-      <c r="G71" t="str">
-        <v>Cash</v>
-      </c>
-      <c r="H71" t="str">
         <v>final payment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H71"/>
+  <autoFilter ref="A1:H70"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H70"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3713,11 +3687,11 @@
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>40000</v>
+        <v>39500</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>-500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -4262,11 +4236,11 @@
       </c>
       <c r="D51" s="1">
         <f>SUM(D2:D50)</f>
-        <v>1234238</v>
+        <v>1233738</v>
       </c>
       <c r="E51" s="1">
         <f>SUM(E2:E50)</f>
-        <v>29500</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update budget item: Arbiya & Didi Sandle — ₹1,300.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -542,7 +542,7 @@
         <v>985ce939</v>
       </c>
       <c r="B7" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Arbiya &amp; Didi Sandle</v>
       </c>
       <c r="C7" t="str">
         <v>Clothing &amp; Jewellery</v>
@@ -2071,7 +2071,7 @@
         <v>985ce939</v>
       </c>
       <c r="C25" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Arbiya &amp; Didi Sandle</v>
       </c>
       <c r="D25" s="3">
         <v>46257</v>
@@ -3392,7 +3392,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Arbiya &amp; Didi Sandle</v>
       </c>
       <c r="B7" t="str">
         <v>Clothing &amp; Jewellery</v>

</xml_diff>

<commit_message>
Add budget item: Lucky Mattan Shop (Bakra for haldi) — ₹10,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H70</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -979,136 +979,136 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>a1def8e4</v>
+        <v>99d3617a</v>
       </c>
       <c r="B29" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Lucky Mattan Shop (Bakra for haldi)</v>
       </c>
       <c r="C29" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D29" s="1">
-        <v>5412</v>
+        <v>10000</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>Rahim</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>c7e8b352</v>
+        <v>a1def8e4</v>
       </c>
       <c r="B30" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="C30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D30" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B31" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B32" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B33" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C33" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B34" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C34" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B35" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D35" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
@@ -1119,113 +1119,113 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B36" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C36" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B37" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C37" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D37" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B38" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C38" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D38" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B39" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C39" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D39" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B40" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C40" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D40" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
       </c>
       <c r="F40" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B41" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C41" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D41" s="1">
         <v>4000</v>
@@ -1239,188 +1239,208 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B42" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C42" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D42" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E42" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F42" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B43" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C43" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D43" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E43" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F43" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B44" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C44" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D44" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E44" s="2" t="str">
         <v/>
       </c>
       <c r="F44" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B45" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C45" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D45" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E45" s="2" t="str">
         <v/>
       </c>
       <c r="F45" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B46" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C46" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D46" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E46" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F46" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B47" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C47" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D47" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E47" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F47" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B48" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C48" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D48" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E48" s="2" t="str">
         <v/>
       </c>
       <c r="F48" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B49" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C49" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D49" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E49" s="2" t="str">
         <v/>
       </c>
       <c r="F49" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D50" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E50" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B50" t="str">
+      <c r="B51" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C50" t="str">
+      <c r="C51" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D51" s="1">
         <v>9150</v>
       </c>
-      <c r="E50" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F50" t="str">
+      <c r="E51" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F50"/>
+  <autoFilter ref="A1:F51"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3269,7 +3289,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3810,36 +3830,36 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Lucky Mattan Shop (Bakra for haldi)</v>
       </c>
       <c r="B29" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C29" s="1">
-        <v>5412</v>
+        <v>10000</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>5412</v>
+        <v>0</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="B30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C30" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3848,17 +3868,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3867,17 +3887,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3886,17 +3906,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B33" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3905,17 +3925,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B34" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -3924,17 +3944,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C35" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -3943,17 +3963,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B36" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -3962,17 +3982,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B37" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C37" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -3981,17 +4001,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B38" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C38" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -4000,17 +4020,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B39" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C39" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -4019,17 +4039,17 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B40" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C40" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -4038,10 +4058,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B41" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C41" s="1">
         <v>4000</v>
@@ -4057,55 +4077,55 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B42" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C42" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B43" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C43" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B44" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C44" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
@@ -4114,17 +4134,17 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B45" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C45" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
@@ -4133,17 +4153,17 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B46" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C46" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
@@ -4152,17 +4172,17 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B47" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C47" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
@@ -4171,17 +4191,17 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B48" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C48" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
@@ -4190,17 +4210,17 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B49" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C49" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
@@ -4209,17 +4229,17 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B50" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C50" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
@@ -4228,24 +4248,43 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C51" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D51" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E51" s="1">
+        <f>C51-D51</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
         <v>Total</v>
       </c>
-      <c r="C51" s="1">
-        <f>SUM(C2:C50)</f>
-        <v>1263738</v>
-      </c>
-      <c r="D51" s="1">
-        <f>SUM(D2:D50)</f>
+      <c r="C52" s="1">
+        <f>SUM(C2:C51)</f>
+        <v>1273738</v>
+      </c>
+      <c r="D52" s="1">
+        <f>SUM(D2:D51)</f>
         <v>1233738</v>
       </c>
-      <c r="E51" s="1">
-        <f>SUM(E2:E50)</f>
-        <v>30000</v>
+      <c r="E52" s="1">
+        <f>SUM(E2:E51)</f>
+        <v>40000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E52"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹10,000.00 by Umar Sayyed (Father) for Lucky Mattan Shop (Bakra for haldi)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H71</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1447,7 +1447,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2995,71 +2995,71 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>09899d1e</v>
+        <v>45e7ae1c</v>
       </c>
       <c r="B60" t="str">
-        <v>c1c67a32</v>
+        <v>99d3617a</v>
       </c>
       <c r="C60" t="str">
-        <v>car decoration, Dj, Petrol, Haldi Celender</v>
+        <v>Lucky Mattan Shop (Bakra for haldi)</v>
       </c>
       <c r="D60" s="3">
-        <v>46299</v>
+        <v>46298</v>
       </c>
       <c r="E60" s="1">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="F60" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G60" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H60" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>fc7adcbd</v>
+        <v>09899d1e</v>
       </c>
       <c r="B61" t="str">
-        <v>04ece648</v>
+        <v>c1c67a32</v>
       </c>
       <c r="C61" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>car decoration, Dj, Petrol, Haldi Celender</v>
       </c>
       <c r="D61" s="3">
-        <v>46300</v>
+        <v>46299</v>
       </c>
       <c r="E61" s="1">
-        <v>15000</v>
+        <v>30000</v>
       </c>
       <c r="F61" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G61" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H61" t="str">
-        <v>payment done</v>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>384605f7</v>
+        <v>fc7adcbd</v>
       </c>
       <c r="B62" t="str">
-        <v>22ff3fb2</v>
+        <v>04ece648</v>
       </c>
       <c r="C62" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="D62" s="3">
         <v>46300</v>
       </c>
       <c r="E62" s="1">
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="F62" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3068,24 +3068,24 @@
         <v>Cash</v>
       </c>
       <c r="H62" t="str">
-        <v/>
+        <v>payment done</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>d08ebf7d</v>
+        <v>384605f7</v>
       </c>
       <c r="B63" t="str">
-        <v>9b3747da</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C63" t="str">
-        <v>tampo traveller</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D63" s="3">
         <v>46300</v>
       </c>
       <c r="E63" s="1">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="F63" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3094,50 +3094,50 @@
         <v>Cash</v>
       </c>
       <c r="H63" t="str">
-        <v>cash</v>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>3adcd8de</v>
+        <v>d08ebf7d</v>
       </c>
       <c r="B64" t="str">
-        <v>4d3bd5b1</v>
+        <v>9b3747da</v>
       </c>
       <c r="C64" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>tampo traveller</v>
       </c>
       <c r="D64" s="3">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E64" s="1">
-        <v>24000</v>
+        <v>7500</v>
       </c>
       <c r="F64" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G64" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H64" t="str">
-        <v>Final payment</v>
+        <v>cash</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>4f298a0d</v>
+        <v>3adcd8de</v>
       </c>
       <c r="B65" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C65" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D65" s="3">
         <v>46302</v>
       </c>
       <c r="E65" s="1">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="F65" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3146,24 +3146,24 @@
         <v>UPI</v>
       </c>
       <c r="H65" t="str">
-        <v>Installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>141e8fbb</v>
+        <v>4f298a0d</v>
       </c>
       <c r="B66" t="str">
-        <v>4d3bd5b1</v>
+        <v>631875ca</v>
       </c>
       <c r="C66" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D66" s="3">
         <v>46302</v>
       </c>
       <c r="E66" s="1">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="F66" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3172,24 +3172,24 @@
         <v>UPI</v>
       </c>
       <c r="H66" t="str">
-        <v>paid</v>
+        <v>Installment</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>da6b0ec5</v>
+        <v>141e8fbb</v>
       </c>
       <c r="B67" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C67" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D67" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E67" s="1">
-        <v>33000</v>
+        <v>500</v>
       </c>
       <c r="F67" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3198,91 +3198,117 @@
         <v>UPI</v>
       </c>
       <c r="H67" t="str">
-        <v>Payment done</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B68" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C68" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D68" s="3">
         <v>46303</v>
       </c>
       <c r="E68" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F68" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G68" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H68" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B69" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C69" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D69" s="3">
         <v>46303</v>
       </c>
       <c r="E69" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F69" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G69" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H69" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
+        <v>80e653df</v>
+      </c>
+      <c r="B70" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D70" s="3">
+        <v>46303</v>
+      </c>
+      <c r="E70" s="1">
+        <v>30000</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G70" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H70" t="str">
+        <v>Second last installment</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
         <v>79cb1a7e</v>
       </c>
-      <c r="B70" t="str">
+      <c r="B71" t="str">
         <v>22ff3fb2</v>
       </c>
-      <c r="C70" t="str">
+      <c r="C71" t="str">
         <v>chair arrangment soyarik gardan</v>
       </c>
-      <c r="D70" s="3">
+      <c r="D71" s="3">
         <v>46306</v>
       </c>
-      <c r="E70" s="1">
+      <c r="E71" s="1">
         <v>1000</v>
       </c>
-      <c r="F70" t="str">
+      <c r="F71" t="str">
         <v>Umar Sayyed (Father)</v>
       </c>
-      <c r="G70" t="str">
+      <c r="G71" t="str">
         <v>Cash</v>
       </c>
-      <c r="H70" t="str">
+      <c r="H71" t="str">
         <v>final payment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H70"/>
+  <autoFilter ref="A1:H71"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H71"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3840,11 +3866,11 @@
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -4275,11 +4301,11 @@
       </c>
       <c r="D52" s="1">
         <f>SUM(D2:D51)</f>
-        <v>1233738</v>
+        <v>1243738</v>
       </c>
       <c r="E52" s="1">
         <f>SUM(E2:E51)</f>
-        <v>40000</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Music in reception & sangit — ₹13,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H71</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1139,113 +1139,113 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>eebc3aaf</v>
+        <v>f31def6e</v>
       </c>
       <c r="B37" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="C37" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D37" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B38" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C38" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D38" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B39" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C39" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D39" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B40" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C40" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D40" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
       </c>
       <c r="F40" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B41" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C41" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D41" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E41" s="2" t="str">
         <v/>
       </c>
       <c r="F41" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B42" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C42" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D42" s="1">
         <v>4000</v>
@@ -1259,188 +1259,208 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B43" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C43" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D43" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E43" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F43" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B44" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C44" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D44" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E44" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F44" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B45" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C45" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D45" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E45" s="2" t="str">
         <v/>
       </c>
       <c r="F45" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B46" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C46" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D46" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E46" s="2" t="str">
         <v/>
       </c>
       <c r="F46" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B47" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C47" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D47" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E47" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F47" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B48" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C48" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D48" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E48" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F48" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B49" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C49" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D49" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E49" s="2" t="str">
         <v/>
       </c>
       <c r="F49" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B50" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C50" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D50" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E50" s="2" t="str">
         <v/>
       </c>
       <c r="F50" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D51" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E51" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B51" t="str">
+      <c r="B52" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C51" t="str">
+      <c r="C52" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D52" s="1">
         <v>9150</v>
       </c>
-      <c r="E51" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F51" t="str">
+      <c r="E52" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F51"/>
+  <autoFilter ref="A1:F52"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F52"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3315,7 +3335,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4008,36 +4028,36 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="B37" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C37" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>0</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
-        <v>0</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B38" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C38" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -4046,17 +4066,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B39" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C39" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -4065,17 +4085,17 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B40" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C40" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -4084,17 +4104,17 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B41" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C41" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -4103,10 +4123,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B42" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C42" s="1">
         <v>4000</v>
@@ -4122,55 +4142,55 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B43" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C43" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B44" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C44" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B45" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C45" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
@@ -4179,17 +4199,17 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B46" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C46" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
@@ -4198,17 +4218,17 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B47" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C47" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
@@ -4217,17 +4237,17 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B48" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C48" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
@@ -4236,17 +4256,17 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B49" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C49" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
@@ -4255,17 +4275,17 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B50" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C50" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
@@ -4274,17 +4294,17 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B51" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C51" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4293,24 +4313,43 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C52" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D52" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E52" s="1">
+        <f>C52-D52</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
         <v>Total</v>
       </c>
-      <c r="C52" s="1">
-        <f>SUM(C2:C51)</f>
-        <v>1273738</v>
-      </c>
-      <c r="D52" s="1">
-        <f>SUM(D2:D51)</f>
+      <c r="C53" s="1">
+        <f>SUM(C2:C52)</f>
+        <v>1286738</v>
+      </c>
+      <c r="D53" s="1">
+        <f>SUM(D2:D52)</f>
         <v>1243738</v>
       </c>
-      <c r="E52" s="1">
-        <f>SUM(E2:E51)</f>
-        <v>30000</v>
+      <c r="E53" s="1">
+        <f>SUM(E2:E52)</f>
+        <v>43000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹13,000.00 by Umar Sayyed (Father) for Music in reception & sangit
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H72</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1467,7 +1467,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3223,112 +3223,138 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>da6b0ec5</v>
+        <v>738b696a</v>
       </c>
       <c r="B68" t="str">
-        <v>631875ca</v>
+        <v>f31def6e</v>
       </c>
       <c r="C68" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="D68" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E68" s="1">
-        <v>33000</v>
+        <v>13000</v>
       </c>
       <c r="F68" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G68" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H68" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B69" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C69" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D69" s="3">
         <v>46303</v>
       </c>
       <c r="E69" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F69" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G69" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H69" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B70" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C70" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D70" s="3">
         <v>46303</v>
       </c>
       <c r="E70" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F70" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G70" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H70" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
+        <v>80e653df</v>
+      </c>
+      <c r="B71" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D71" s="3">
+        <v>46303</v>
+      </c>
+      <c r="E71" s="1">
+        <v>30000</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G71" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H71" t="str">
+        <v>Second last installment</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
         <v>79cb1a7e</v>
       </c>
-      <c r="B71" t="str">
+      <c r="B72" t="str">
         <v>22ff3fb2</v>
       </c>
-      <c r="C71" t="str">
+      <c r="C72" t="str">
         <v>chair arrangment soyarik gardan</v>
       </c>
-      <c r="D71" s="3">
+      <c r="D72" s="3">
         <v>46306</v>
       </c>
-      <c r="E71" s="1">
+      <c r="E72" s="1">
         <v>1000</v>
       </c>
-      <c r="F71" t="str">
+      <c r="F72" t="str">
         <v>Umar Sayyed (Father)</v>
       </c>
-      <c r="G71" t="str">
+      <c r="G72" t="str">
         <v>Cash</v>
       </c>
-      <c r="H71" t="str">
+      <c r="H72" t="str">
         <v>final payment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H71"/>
+  <autoFilter ref="A1:H72"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H72"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4038,11 +4064,11 @@
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>13000</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
-        <v>13000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -4340,11 +4366,11 @@
       </c>
       <c r="D53" s="1">
         <f>SUM(D2:D52)</f>
-        <v>1243738</v>
+        <v>1256738</v>
       </c>
       <c r="E53" s="1">
         <f>SUM(E2:E52)</f>
-        <v>43000</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: 3 kg asli ghee — ₹1,830.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H72</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -499,196 +499,196 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>bae4068a</v>
+        <v>70d7465c</v>
       </c>
       <c r="B5" t="str">
-        <v>A S leather zone - Groom jacket</v>
+        <v>3 kg asli ghee</v>
       </c>
       <c r="C5" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D5" s="1">
-        <v>3500</v>
+        <v>1830</v>
       </c>
       <c r="E5" s="2" t="str">
-        <v>08087832131</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Groom pre wedding jacket</v>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>aaedf833</v>
+        <v>bae4068a</v>
       </c>
       <c r="B6" t="str">
-        <v>Aluminum Shop Partition</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="C6" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D6" s="1">
-        <v>23000</v>
+        <v>3500</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v>8446627171</v>
+        <v>08087832131</v>
       </c>
       <c r="F6" t="str">
-        <v>Aluminum Shop Partition</v>
+        <v>Groom pre wedding jacket</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>985ce939</v>
+        <v>aaedf833</v>
       </c>
       <c r="B7" t="str">
-        <v>Arbiya &amp; Didi Sandle</v>
+        <v>Aluminum Shop Partition</v>
       </c>
       <c r="C7" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D7" s="1">
-        <v>1300</v>
+        <v>23000</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v/>
+        <v>8446627171</v>
       </c>
       <c r="F7" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Aluminum Shop Partition</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>a036f9f7</v>
+        <v>985ce939</v>
       </c>
       <c r="B8" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sandle</v>
       </c>
       <c r="C8" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D8" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="E8" s="2" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>f68b08a7</v>
+        <v>a036f9f7</v>
       </c>
       <c r="B9" t="str">
-        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="C9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>7100</v>
+        <v>550</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>Arbiya Bangals</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>0e8bf89b</v>
+        <v>f68b08a7</v>
       </c>
       <c r="B10" t="str">
-        <v>Bari ka saman</v>
+        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
       </c>
       <c r="C10" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D10" s="1">
-        <v>2200</v>
+        <v>7100</v>
       </c>
       <c r="E10" s="2" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Bari ka saman</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>1aa31869</v>
+        <v>0e8bf89b</v>
       </c>
       <c r="B11" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="C11" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D11" s="1">
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="E11" s="2" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>0beedebe</v>
+        <v>1aa31869</v>
       </c>
       <c r="B12" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="C12" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D12" s="1">
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="E12" s="2" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>c1c67a32</v>
+        <v>0beedebe</v>
       </c>
       <c r="B13" t="str">
-        <v>car decoration, Dj, Petrol, Haldi Celender</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="C13" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D13" s="1">
-        <v>30000</v>
+        <v>4600</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>22ff3fb2</v>
+        <v>c1c67a32</v>
       </c>
       <c r="B14" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>car decoration, Dj, Petrol, Haldi Celender</v>
       </c>
       <c r="C14" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Decoration</v>
       </c>
       <c r="D14" s="1">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
@@ -699,16 +699,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2a74d868</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="B15" t="str">
-        <v>Colour &amp; plumber</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="C15" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D15" s="1">
-        <v>800</v>
+        <v>3000</v>
       </c>
       <c r="E15" s="2" t="str">
         <v/>
@@ -719,19 +719,19 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>0cf8885b</v>
+        <v>2a74d868</v>
       </c>
       <c r="B16" t="str">
-        <v>Crackers</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="C16" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D16" s="1">
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v>+91 86557 63847</v>
+        <v/>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -739,139 +739,139 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>05d27deb</v>
+        <v>0cf8885b</v>
       </c>
       <c r="B17" t="str">
-        <v>Cream House Lunch</v>
+        <v>Crackers</v>
       </c>
       <c r="C17" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D17" s="1">
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v/>
+        <v>+91 86557 63847</v>
       </c>
       <c r="F17" t="str">
-        <v>Cream House Lunch</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>631875ca</v>
+        <v>05d27deb</v>
       </c>
       <c r="B18" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="C18" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D18" s="1">
-        <v>161000</v>
+        <v>1124</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F18" t="str">
-        <v>Hall decoration</v>
+        <v>Cream House Lunch</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B19" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C19" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D19" s="1">
-        <v>12150</v>
+        <v>161000</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F19" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B20" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B21" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C21" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F21" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>4d3bd5b1</v>
+        <v>070f7b33</v>
       </c>
       <c r="B22" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C22" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D22" s="1">
-        <v>39500</v>
+        <v>2609</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>9168993010</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>766bfdf7</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="B23" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="C23" t="str">
-        <v>Miscellaneous</v>
+        <v>Decoration</v>
       </c>
       <c r="D23" s="1">
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v/>
+        <v>9168993010</v>
       </c>
       <c r="F23" t="str">
         <v/>
@@ -879,256 +879,256 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>209d43b7</v>
+        <v>766bfdf7</v>
       </c>
       <c r="B24" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="C24" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D24" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B25" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C25" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D25" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E25" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F25" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>dc70b2a1</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B26" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C26" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D26" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E26" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F26" t="str">
-        <v>internal expense</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B27" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C27" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D27" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E27" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F27" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B28" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C28" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D28" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E28" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F28" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>99d3617a</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B29" t="str">
-        <v>Lucky Mattan Shop (Bakra for haldi)</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C29" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D29" s="1">
-        <v>10000</v>
+        <v>3675</v>
       </c>
       <c r="E29" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F29" t="str">
-        <v>Rahim</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>a1def8e4</v>
+        <v>99d3617a</v>
       </c>
       <c r="B30" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Lucky Mattan Shop (Bakra for haldi)</v>
       </c>
       <c r="C30" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D30" s="1">
-        <v>5412</v>
+        <v>10000</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>Rahim</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>c7e8b352</v>
+        <v>a1def8e4</v>
       </c>
       <c r="B31" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="C31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D31" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B32" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B33" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C33" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B34" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C34" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B35" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C35" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B36" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C36" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D36" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
@@ -1139,16 +1139,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>f31def6e</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B37" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C37" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D37" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
@@ -1159,113 +1159,113 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>eebc3aaf</v>
+        <v>f31def6e</v>
       </c>
       <c r="B38" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="C38" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D38" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B39" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C39" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D39" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B40" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C40" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D40" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
       </c>
       <c r="F40" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B41" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C41" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D41" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E41" s="2" t="str">
         <v/>
       </c>
       <c r="F41" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B42" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C42" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D42" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E42" s="2" t="str">
         <v/>
       </c>
       <c r="F42" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B43" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C43" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D43" s="1">
         <v>4000</v>
@@ -1279,188 +1279,208 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B44" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C44" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D44" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E44" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F44" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B45" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C45" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D45" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E45" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F45" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B46" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C46" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D46" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E46" s="2" t="str">
         <v/>
       </c>
       <c r="F46" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B47" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C47" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D47" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E47" s="2" t="str">
         <v/>
       </c>
       <c r="F47" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B48" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C48" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D48" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E48" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F48" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B49" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C49" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D49" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E49" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F49" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B50" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C50" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D50" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E50" s="2" t="str">
         <v/>
       </c>
       <c r="F50" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B51" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C51" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D51" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E51" s="2" t="str">
         <v/>
       </c>
       <c r="F51" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D52" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E52" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B52" t="str">
+      <c r="B53" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C52" t="str">
+      <c r="C53" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D52" s="1">
+      <c r="D53" s="1">
         <v>9150</v>
       </c>
-      <c r="E52" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F52" t="str">
+      <c r="E53" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F52"/>
+  <autoFilter ref="A1:F53"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F53"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3361,7 +3381,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3446,36 +3466,36 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>A S leather zone - Groom jacket</v>
+        <v>3 kg asli ghee</v>
       </c>
       <c r="B5" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C5" s="1">
-        <v>3500</v>
+        <v>1830</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
-        <v>0</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Aluminum Shop Partition</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="B6" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C6" s="1">
-        <v>23000</v>
+        <v>3500</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>23000</v>
+        <v>3500</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
@@ -3484,17 +3504,17 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Arbiya &amp; Didi Sandle</v>
+        <v>Aluminum Shop Partition</v>
       </c>
       <c r="B7" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C7" s="1">
-        <v>1300</v>
+        <v>23000</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>1300</v>
+        <v>23000</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
@@ -3503,17 +3523,17 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sandle</v>
       </c>
       <c r="B8" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C8" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
@@ -3522,17 +3542,17 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="B9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>7100</v>
+        <v>550</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>7100</v>
+        <v>550</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
@@ -3541,17 +3561,17 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Bari ka saman</v>
+        <v>Asif Radimant dress, jokey inner ware, white tighty, sliper</v>
       </c>
       <c r="B10" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C10" s="1">
-        <v>2200</v>
+        <v>7100</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>2200</v>
+        <v>7100</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -3560,17 +3580,17 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="B11" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C11" s="1">
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -3579,17 +3599,17 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="B12" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C12" s="1">
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -3598,17 +3618,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>car decoration, Dj, Petrol, Haldi Celender</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="B13" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C13" s="1">
-        <v>30000</v>
+        <v>4600</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>30000</v>
+        <v>4600</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -3617,17 +3637,17 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>car decoration, Dj, Petrol, Haldi Celender</v>
       </c>
       <c r="B14" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Decoration</v>
       </c>
       <c r="C14" s="1">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -3636,17 +3656,17 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Colour &amp; plumber</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="B15" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C15" s="1">
-        <v>800</v>
+        <v>3000</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>800</v>
+        <v>3000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -3655,17 +3675,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Crackers</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="B16" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C16" s="1">
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>5500</v>
+        <v>800</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -3674,17 +3694,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Cream House Lunch</v>
+        <v>Crackers</v>
       </c>
       <c r="B17" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C17" s="1">
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>1124</v>
+        <v>5500</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -3693,17 +3713,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="B18" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C18" s="1">
-        <v>161000</v>
+        <v>1124</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>161000</v>
+        <v>1124</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -3712,17 +3732,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B19" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C19" s="1">
-        <v>12150</v>
+        <v>161000</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>161000</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -3731,17 +3751,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -3750,17 +3770,17 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B21" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -3769,17 +3789,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B22" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C22" s="1">
-        <v>39500</v>
+        <v>2609</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>39500</v>
+        <v>2609</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -3788,17 +3808,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Garva Biryani, hardware expense, flower</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="B23" t="str">
-        <v>Miscellaneous</v>
+        <v>Decoration</v>
       </c>
       <c r="C23" s="1">
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>410</v>
+        <v>39500</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -3807,17 +3827,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Garva Biryani, hardware expense, flower</v>
       </c>
       <c r="B24" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C24" s="1">
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>410</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -3826,17 +3846,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B25" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C25" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -3845,17 +3865,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B26" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C26" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -3864,17 +3884,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B27" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C27" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -3883,17 +3903,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B28" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C28" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -3902,17 +3922,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Lucky Mattan Shop (Bakra for haldi)</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B29" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C29" s="1">
-        <v>10000</v>
+        <v>3675</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>3675</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -3921,17 +3941,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Lucky Mattan Shop (Bakra for haldi)</v>
       </c>
       <c r="B30" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C30" s="1">
-        <v>5412</v>
+        <v>10000</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>5412</v>
+        <v>10000</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -3940,17 +3960,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="B31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C31" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -3959,17 +3979,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -3978,17 +3998,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B33" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -3997,17 +4017,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B34" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -4016,17 +4036,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B35" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -4035,17 +4055,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B36" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C36" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -4054,17 +4074,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B37" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C37" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -4073,17 +4093,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="B38" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C38" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -4092,17 +4112,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B39" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C39" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -4111,17 +4131,17 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B40" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C40" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -4130,17 +4150,17 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B41" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C41" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -4149,17 +4169,17 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B42" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C42" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
@@ -4168,10 +4188,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B43" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C43" s="1">
         <v>4000</v>
@@ -4187,55 +4207,55 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B44" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C44" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B45" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C45" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B46" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C46" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
@@ -4244,17 +4264,17 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B47" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C47" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
@@ -4263,17 +4283,17 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B48" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C48" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
@@ -4282,17 +4302,17 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B49" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C49" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
@@ -4301,17 +4321,17 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B50" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C50" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
@@ -4320,17 +4340,17 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B51" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C51" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4339,17 +4359,17 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B52" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C52" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4358,24 +4378,43 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C53" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D53" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E53" s="1">
+        <f>C53-D53</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
         <v>Total</v>
       </c>
-      <c r="C53" s="1">
-        <f>SUM(C2:C52)</f>
-        <v>1286738</v>
-      </c>
-      <c r="D53" s="1">
-        <f>SUM(D2:D52)</f>
+      <c r="C54" s="1">
+        <f>SUM(C2:C53)</f>
+        <v>1288568</v>
+      </c>
+      <c r="D54" s="1">
+        <f>SUM(D2:D53)</f>
         <v>1256738</v>
       </c>
-      <c r="E53" s="1">
-        <f>SUM(E2:E52)</f>
-        <v>30000</v>
+      <c r="E54" s="1">
+        <f>SUM(E2:E53)</f>
+        <v>31830</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E54"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹1,830.00 by Umar Sayyed (Father) for 3 kg asli ghee
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H73</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1487,7 +1487,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3371,10 +3371,36 @@
         <v>final payment</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B73" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C73" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D73" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E73" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G73" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H72"/>
+  <autoFilter ref="A1:H73"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H73"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3476,11 +3502,11 @@
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>1830</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
-        <v>1830</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -4405,11 +4431,11 @@
       </c>
       <c r="D54" s="1">
         <f>SUM(D2:D53)</f>
-        <v>1256738</v>
+        <v>1258568</v>
       </c>
       <c r="E54" s="1">
         <f>SUM(E2:E53)</f>
-        <v>31830</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Meher Amount — ₹11,111.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H73</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1019,16 +1019,16 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>a1def8e4</v>
+        <v>08cd3226</v>
       </c>
       <c r="B31" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Meher Amount</v>
       </c>
       <c r="C31" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D31" s="1">
-        <v>5412</v>
+        <v>11111</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
@@ -1039,116 +1039,116 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>c7e8b352</v>
+        <v>a1def8e4</v>
       </c>
       <c r="B32" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="C32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D32" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B33" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C33" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B34" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C34" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B35" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C35" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B36" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C36" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B37" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C37" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D37" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
@@ -1159,16 +1159,16 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>f31def6e</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B38" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C38" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D38" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
@@ -1179,113 +1179,113 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>eebc3aaf</v>
+        <v>f31def6e</v>
       </c>
       <c r="B39" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="C39" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D39" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B40" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C40" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D40" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
       </c>
       <c r="F40" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B41" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C41" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D41" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E41" s="2" t="str">
         <v/>
       </c>
       <c r="F41" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B42" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C42" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D42" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E42" s="2" t="str">
         <v/>
       </c>
       <c r="F42" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B43" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C43" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D43" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E43" s="2" t="str">
         <v/>
       </c>
       <c r="F43" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B44" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C44" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D44" s="1">
         <v>4000</v>
@@ -1299,188 +1299,208 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B45" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C45" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D45" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E45" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F45" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B46" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C46" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D46" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E46" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F46" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B47" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C47" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D47" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E47" s="2" t="str">
         <v/>
       </c>
       <c r="F47" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B48" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C48" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D48" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E48" s="2" t="str">
         <v/>
       </c>
       <c r="F48" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B49" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C49" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D49" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E49" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F49" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B50" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C50" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D50" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E50" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F50" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B51" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C51" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D51" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E51" s="2" t="str">
         <v/>
       </c>
       <c r="F51" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B52" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C52" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D52" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E52" s="2" t="str">
         <v/>
       </c>
       <c r="F52" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D53" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E53" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B53" t="str">
+      <c r="B54" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C53" t="str">
+      <c r="C54" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D54" s="1">
         <v>9150</v>
       </c>
-      <c r="E53" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F53" t="str">
+      <c r="E54" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F53"/>
+  <autoFilter ref="A1:F54"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3407,7 +3427,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3986,36 +4006,36 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Meher Amount</v>
       </c>
       <c r="B31" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C31" s="1">
-        <v>5412</v>
+        <v>11111</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>5412</v>
+        <v>0</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
-        <v>0</v>
+        <v>11111</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="B32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C32" s="1">
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>5412</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -4024,17 +4044,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B33" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -4043,17 +4063,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B34" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -4062,17 +4082,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B35" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -4081,17 +4101,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B36" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -4100,17 +4120,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B37" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C37" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -4119,17 +4139,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B38" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C38" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -4138,17 +4158,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="B39" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C39" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -4157,17 +4177,17 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B40" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C40" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -4176,17 +4196,17 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B41" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C41" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -4195,17 +4215,17 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B42" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C42" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
@@ -4214,17 +4234,17 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B43" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C43" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
@@ -4233,10 +4253,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B44" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C44" s="1">
         <v>4000</v>
@@ -4252,55 +4272,55 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B45" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C45" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B46" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C46" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B47" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C47" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
@@ -4309,17 +4329,17 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B48" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C48" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
@@ -4328,17 +4348,17 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B49" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C49" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
@@ -4347,17 +4367,17 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B50" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C50" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
@@ -4366,17 +4386,17 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B51" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C51" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4385,17 +4405,17 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B52" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C52" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4404,17 +4424,17 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B53" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C53" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D53" s="1">
         <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E53" s="1">
         <f>C53-D53</f>
@@ -4423,24 +4443,43 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C54" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D54" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A54,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E54" s="1">
+        <f>C54-D54</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
         <v>Total</v>
       </c>
-      <c r="C54" s="1">
-        <f>SUM(C2:C53)</f>
-        <v>1288568</v>
-      </c>
-      <c r="D54" s="1">
-        <f>SUM(D2:D53)</f>
+      <c r="C55" s="1">
+        <f>SUM(C2:C54)</f>
+        <v>1299679</v>
+      </c>
+      <c r="D55" s="1">
+        <f>SUM(D2:D54)</f>
         <v>1258568</v>
       </c>
-      <c r="E54" s="1">
-        <f>SUM(E2:E53)</f>
-        <v>30000</v>
+      <c r="E55" s="1">
+        <f>SUM(E2:E54)</f>
+        <v>41111</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E55"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹11,111.00 by Umar Sayyed (Father) for Meher Amount
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H74</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1507,7 +1507,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3107,19 +3107,19 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>fc7adcbd</v>
+        <v>2b0b3096</v>
       </c>
       <c r="B62" t="str">
-        <v>04ece648</v>
+        <v>08cd3226</v>
       </c>
       <c r="C62" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Meher Amount</v>
       </c>
       <c r="D62" s="3">
-        <v>46300</v>
+        <v>46299</v>
       </c>
       <c r="E62" s="1">
-        <v>15000</v>
+        <v>11111</v>
       </c>
       <c r="F62" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3128,24 +3128,24 @@
         <v>Cash</v>
       </c>
       <c r="H62" t="str">
-        <v>payment done</v>
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>384605f7</v>
+        <v>fc7adcbd</v>
       </c>
       <c r="B63" t="str">
-        <v>22ff3fb2</v>
+        <v>04ece648</v>
       </c>
       <c r="C63" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="D63" s="3">
         <v>46300</v>
       </c>
       <c r="E63" s="1">
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="F63" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3154,24 +3154,24 @@
         <v>Cash</v>
       </c>
       <c r="H63" t="str">
-        <v/>
+        <v>payment done</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>d08ebf7d</v>
+        <v>384605f7</v>
       </c>
       <c r="B64" t="str">
-        <v>9b3747da</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C64" t="str">
-        <v>tampo traveller</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D64" s="3">
         <v>46300</v>
       </c>
       <c r="E64" s="1">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="F64" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3180,50 +3180,50 @@
         <v>Cash</v>
       </c>
       <c r="H64" t="str">
-        <v>cash</v>
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>3adcd8de</v>
+        <v>d08ebf7d</v>
       </c>
       <c r="B65" t="str">
-        <v>4d3bd5b1</v>
+        <v>9b3747da</v>
       </c>
       <c r="C65" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>tampo traveller</v>
       </c>
       <c r="D65" s="3">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E65" s="1">
-        <v>24000</v>
+        <v>7500</v>
       </c>
       <c r="F65" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G65" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H65" t="str">
-        <v>Final payment</v>
+        <v>cash</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>4f298a0d</v>
+        <v>3adcd8de</v>
       </c>
       <c r="B66" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C66" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D66" s="3">
         <v>46302</v>
       </c>
       <c r="E66" s="1">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="F66" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3232,24 +3232,24 @@
         <v>UPI</v>
       </c>
       <c r="H66" t="str">
-        <v>Installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>141e8fbb</v>
+        <v>4f298a0d</v>
       </c>
       <c r="B67" t="str">
-        <v>4d3bd5b1</v>
+        <v>631875ca</v>
       </c>
       <c r="C67" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D67" s="3">
         <v>46302</v>
       </c>
       <c r="E67" s="1">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="F67" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3258,154 +3258,154 @@
         <v>UPI</v>
       </c>
       <c r="H67" t="str">
-        <v>paid</v>
+        <v>Installment</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>738b696a</v>
+        <v>141e8fbb</v>
       </c>
       <c r="B68" t="str">
-        <v>f31def6e</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C68" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D68" s="3">
         <v>46302</v>
       </c>
       <c r="E68" s="1">
-        <v>13000</v>
+        <v>500</v>
       </c>
       <c r="F68" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G68" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H68" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>da6b0ec5</v>
+        <v>738b696a</v>
       </c>
       <c r="B69" t="str">
-        <v>631875ca</v>
+        <v>f31def6e</v>
       </c>
       <c r="C69" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="D69" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E69" s="1">
-        <v>33000</v>
+        <v>13000</v>
       </c>
       <c r="F69" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G69" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H69" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B70" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C70" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D70" s="3">
         <v>46303</v>
       </c>
       <c r="E70" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F70" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G70" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H70" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B71" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C71" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D71" s="3">
         <v>46303</v>
       </c>
       <c r="E71" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F71" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G71" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H71" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>79cb1a7e</v>
+        <v>80e653df</v>
       </c>
       <c r="B72" t="str">
-        <v>22ff3fb2</v>
+        <v>beb44857</v>
       </c>
       <c r="C72" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D72" s="3">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E72" s="1">
-        <v>1000</v>
+        <v>30000</v>
       </c>
       <c r="F72" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G72" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H72" t="str">
-        <v>final payment</v>
+        <v>Second last installment</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>fcb3d16a</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B73" t="str">
-        <v>70d7465c</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C73" t="str">
-        <v>3 kg asli ghee</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D73" s="3">
         <v>46306</v>
       </c>
       <c r="E73" s="1">
-        <v>1830</v>
+        <v>1000</v>
       </c>
       <c r="F73" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3414,13 +3414,39 @@
         <v>Cash</v>
       </c>
       <c r="H73" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B74" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C74" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D74" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E74" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F74" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G74" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H74" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H73"/>
+  <autoFilter ref="A1:H74"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H74"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4016,11 +4042,11 @@
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>11111</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
-        <v>11111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4470,11 +4496,11 @@
       </c>
       <c r="D55" s="1">
         <f>SUM(D2:D54)</f>
-        <v>1258568</v>
+        <v>1269679</v>
       </c>
       <c r="E55" s="1">
         <f>SUM(E2:E54)</f>
-        <v>41111</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Shadi & reception Rasam — ₹6,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H74</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1379,128 +1379,148 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>d1aee56d</v>
+        <v>c047acbd</v>
       </c>
       <c r="B49" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="C49" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D49" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E49" s="2" t="str">
         <v/>
       </c>
       <c r="F49" t="str">
-        <v>Shireen Dress</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B50" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C50" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D50" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E50" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F50" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B51" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C51" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D51" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E51" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F51" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B52" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C52" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D52" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E52" s="2" t="str">
         <v/>
       </c>
       <c r="F52" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B53" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C53" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D53" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E53" s="2" t="str">
         <v/>
       </c>
       <c r="F53" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D54" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E54" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B55" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C54" t="str">
+      <c r="C55" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D55" s="1">
         <v>9150</v>
       </c>
-      <c r="E54" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F54" t="str">
+      <c r="E55" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F54"/>
+  <autoFilter ref="A1:F55"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F55"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3453,7 +3473,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4374,36 +4394,36 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="B49" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C49" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
-        <v>0</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B50" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C50" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
@@ -4412,17 +4432,17 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B51" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C51" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4431,17 +4451,17 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B52" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C52" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4450,17 +4470,17 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B53" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C53" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D53" s="1">
         <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E53" s="1">
         <f>C53-D53</f>
@@ -4469,17 +4489,17 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B54" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C54" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D54" s="1">
         <f>SUMIF('Payments'!$C:$C,$A54,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E54" s="1">
         <f>C54-D54</f>
@@ -4488,24 +4508,43 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C55" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D55" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A55,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E55" s="1">
+        <f>C55-D55</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
         <v>Total</v>
       </c>
-      <c r="C55" s="1">
-        <f>SUM(C2:C54)</f>
-        <v>1299679</v>
-      </c>
-      <c r="D55" s="1">
-        <f>SUM(D2:D54)</f>
+      <c r="C56" s="1">
+        <f>SUM(C2:C55)</f>
+        <v>1305679</v>
+      </c>
+      <c r="D56" s="1">
+        <f>SUM(D2:D55)</f>
         <v>1269679</v>
       </c>
-      <c r="E55" s="1">
-        <f>SUM(E2:E54)</f>
-        <v>30000</v>
+      <c r="E56" s="1">
+        <f>SUM(E2:E55)</f>
+        <v>36000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E56"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹6,000.00 by Umar Sayyed (Father) for Shadi & reception Rasam
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H75</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1527,7 +1527,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3335,123 +3335,123 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>da6b0ec5</v>
+        <v>ad864ef1</v>
       </c>
       <c r="B70" t="str">
-        <v>631875ca</v>
+        <v>c047acbd</v>
       </c>
       <c r="C70" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="D70" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E70" s="1">
-        <v>33000</v>
+        <v>6000</v>
       </c>
       <c r="F70" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G70" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H70" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B71" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C71" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D71" s="3">
         <v>46303</v>
       </c>
       <c r="E71" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F71" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G71" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H71" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B72" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C72" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D72" s="3">
         <v>46303</v>
       </c>
       <c r="E72" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F72" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G72" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H72" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>79cb1a7e</v>
+        <v>80e653df</v>
       </c>
       <c r="B73" t="str">
-        <v>22ff3fb2</v>
+        <v>beb44857</v>
       </c>
       <c r="C73" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D73" s="3">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E73" s="1">
-        <v>1000</v>
+        <v>30000</v>
       </c>
       <c r="F73" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G73" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H73" t="str">
-        <v>final payment</v>
+        <v>Second last installment</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>fcb3d16a</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B74" t="str">
-        <v>70d7465c</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C74" t="str">
-        <v>3 kg asli ghee</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D74" s="3">
         <v>46306</v>
       </c>
       <c r="E74" s="1">
-        <v>1830</v>
+        <v>1000</v>
       </c>
       <c r="F74" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3460,13 +3460,39 @@
         <v>Cash</v>
       </c>
       <c r="H74" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B75" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C75" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D75" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E75" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F75" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H75" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H74"/>
+  <autoFilter ref="A1:H75"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H75"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4404,11 +4430,11 @@
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
-        <v>6000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -4535,11 +4561,11 @@
       </c>
       <c r="D56" s="1">
         <f>SUM(D2:D55)</f>
-        <v>1269679</v>
+        <v>1275679</v>
       </c>
       <c r="E56" s="1">
         <f>SUM(E2:E55)</f>
-        <v>36000</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Mom Miscellaneous Bangals, Area cleaning other expence — ₹15,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H75</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1059,116 +1059,116 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>c7e8b352</v>
+        <v>87751d8e</v>
       </c>
       <c r="B33" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
       </c>
       <c r="C33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D33" s="1">
-        <v>7604</v>
+        <v>15000</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B34" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C34" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B35" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C35" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B36" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C36" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B37" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C37" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D37" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B38" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C38" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D38" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
@@ -1179,16 +1179,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>f31def6e</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B39" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C39" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D39" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
@@ -1199,113 +1199,113 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>eebc3aaf</v>
+        <v>f31def6e</v>
       </c>
       <c r="B40" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="C40" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D40" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
       </c>
       <c r="F40" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B41" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C41" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D41" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E41" s="2" t="str">
         <v/>
       </c>
       <c r="F41" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B42" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C42" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D42" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E42" s="2" t="str">
         <v/>
       </c>
       <c r="F42" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B43" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C43" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D43" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E43" s="2" t="str">
         <v/>
       </c>
       <c r="F43" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B44" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C44" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D44" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E44" s="2" t="str">
         <v/>
       </c>
       <c r="F44" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B45" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C45" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D45" s="1">
         <v>4000</v>
@@ -1319,208 +1319,228 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B46" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C46" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D46" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E46" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F46" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B47" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C47" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D47" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E47" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F47" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B48" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C48" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D48" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E48" s="2" t="str">
         <v/>
       </c>
       <c r="F48" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>c047acbd</v>
+        <v>6d180155</v>
       </c>
       <c r="B49" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C49" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D49" s="1">
-        <v>6000</v>
+        <v>11840</v>
       </c>
       <c r="E49" s="2" t="str">
         <v/>
       </c>
       <c r="F49" t="str">
-        <v/>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>d1aee56d</v>
+        <v>c047acbd</v>
       </c>
       <c r="B50" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="C50" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D50" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E50" s="2" t="str">
         <v/>
       </c>
       <c r="F50" t="str">
-        <v>Shireen Dress</v>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B51" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C51" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D51" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E51" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F51" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B52" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C52" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D52" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E52" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F52" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B53" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C53" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D53" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E53" s="2" t="str">
         <v/>
       </c>
       <c r="F53" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B54" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C54" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D54" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E54" s="2" t="str">
         <v/>
       </c>
       <c r="F54" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D55" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E55" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B55" t="str">
+      <c r="B56" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C55" t="str">
+      <c r="C56" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D55" s="1">
+      <c r="D56" s="1">
         <v>9150</v>
       </c>
-      <c r="E55" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F55" t="str">
+      <c r="E56" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F55"/>
+  <autoFilter ref="A1:F56"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F56"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3499,7 +3519,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4116,36 +4136,36 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
       </c>
       <c r="B33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C33" s="1">
-        <v>7604</v>
+        <v>15000</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>0</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>0</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B34" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -4154,17 +4174,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B35" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -4173,17 +4193,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B36" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -4192,17 +4212,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B37" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C37" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -4211,17 +4231,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B38" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C38" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -4230,17 +4250,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B39" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C39" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -4249,17 +4269,17 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="B40" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C40" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -4268,17 +4288,17 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B41" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C41" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -4287,17 +4307,17 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B42" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C42" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
@@ -4306,17 +4326,17 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B43" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C43" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
@@ -4325,17 +4345,17 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B44" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C44" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
@@ -4344,10 +4364,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B45" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C45" s="1">
         <v>4000</v>
@@ -4363,55 +4383,55 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B46" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C46" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B47" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C47" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B48" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C48" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
@@ -4420,17 +4440,17 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B49" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C49" s="1">
-        <v>6000</v>
+        <v>11840</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>6000</v>
+        <v>11840</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
@@ -4439,17 +4459,17 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="B50" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C50" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
@@ -4458,17 +4478,17 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B51" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C51" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4477,17 +4497,17 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B52" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C52" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4496,17 +4516,17 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B53" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C53" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D53" s="1">
         <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E53" s="1">
         <f>C53-D53</f>
@@ -4515,17 +4535,17 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B54" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C54" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D54" s="1">
         <f>SUMIF('Payments'!$C:$C,$A54,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E54" s="1">
         <f>C54-D54</f>
@@ -4534,17 +4554,17 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B55" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C55" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D55" s="1">
         <f>SUMIF('Payments'!$C:$C,$A55,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E55" s="1">
         <f>C55-D55</f>
@@ -4553,24 +4573,43 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C56" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D56" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A56,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E56" s="1">
+        <f>C56-D56</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
         <v>Total</v>
       </c>
-      <c r="C56" s="1">
-        <f>SUM(C2:C55)</f>
-        <v>1305679</v>
-      </c>
-      <c r="D56" s="1">
-        <f>SUM(D2:D55)</f>
+      <c r="C57" s="1">
+        <f>SUM(C2:C56)</f>
+        <v>1320679</v>
+      </c>
+      <c r="D57" s="1">
+        <f>SUM(D2:D56)</f>
         <v>1275679</v>
       </c>
-      <c r="E56" s="1">
-        <f>SUM(E2:E55)</f>
-        <v>30000</v>
+      <c r="E57" s="1">
+        <f>SUM(E2:E56)</f>
+        <v>45000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹15,000.00 by Waheeda (mother) for Mom Miscellaneous Bangals, Area cleaning other expence
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H76</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1547,7 +1547,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2965,45 +2965,45 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>37a1eaeb</v>
+        <v>eb8cd69a</v>
       </c>
       <c r="B55" t="str">
-        <v>0cf8885b</v>
+        <v>87751d8e</v>
       </c>
       <c r="C55" t="str">
-        <v>Crackers</v>
+        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
       </c>
       <c r="D55" s="3">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="E55" s="1">
-        <v>5500</v>
+        <v>15000</v>
       </c>
       <c r="F55" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G55" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H55" t="str">
-        <v>Paid</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2190a07d</v>
+        <v>37a1eaeb</v>
       </c>
       <c r="B56" t="str">
-        <v>beb44857</v>
+        <v>0cf8885b</v>
       </c>
       <c r="C56" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Crackers</v>
       </c>
       <c r="D56" s="3">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="E56" s="1">
-        <v>10000</v>
+        <v>5500</v>
       </c>
       <c r="F56" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3012,21 +3012,21 @@
         <v>UPI</v>
       </c>
       <c r="H56" t="str">
-        <v>5 th installment</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ccf68d33</v>
+        <v>2190a07d</v>
       </c>
       <c r="B57" t="str">
-        <v>4d3bd5b1</v>
+        <v>beb44857</v>
       </c>
       <c r="C57" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D57" s="3">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="E57" s="1">
         <v>10000</v>
@@ -3038,24 +3038,24 @@
         <v>UPI</v>
       </c>
       <c r="H57" t="str">
-        <v>second installment</v>
+        <v>5 th installment</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>a6e10a8c</v>
+        <v>ccf68d33</v>
       </c>
       <c r="B58" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C58" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D58" s="3">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="E58" s="1">
-        <v>33000</v>
+        <v>10000</v>
       </c>
       <c r="F58" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3064,24 +3064,24 @@
         <v>UPI</v>
       </c>
       <c r="H58" t="str">
-        <v>4th installment</v>
+        <v>second installment</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>718175b7</v>
+        <v>a6e10a8c</v>
       </c>
       <c r="B59" t="str">
-        <v>a1def8e4</v>
+        <v>631875ca</v>
       </c>
       <c r="C59" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D59" s="3">
         <v>46297</v>
       </c>
       <c r="E59" s="1">
-        <v>5412</v>
+        <v>33000</v>
       </c>
       <c r="F59" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3090,30 +3090,30 @@
         <v>UPI</v>
       </c>
       <c r="H59" t="str">
-        <v>paid</v>
+        <v>4th installment</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>45e7ae1c</v>
+        <v>718175b7</v>
       </c>
       <c r="B60" t="str">
-        <v>99d3617a</v>
+        <v>a1def8e4</v>
       </c>
       <c r="C60" t="str">
-        <v>Lucky Mattan Shop (Bakra for haldi)</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="D60" s="3">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="E60" s="1">
-        <v>10000</v>
+        <v>5412</v>
       </c>
       <c r="F60" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G60" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H60" t="str">
         <v>paid</v>
@@ -3121,51 +3121,51 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>09899d1e</v>
+        <v>45e7ae1c</v>
       </c>
       <c r="B61" t="str">
-        <v>c1c67a32</v>
+        <v>99d3617a</v>
       </c>
       <c r="C61" t="str">
-        <v>car decoration, Dj, Petrol, Haldi Celender</v>
+        <v>Lucky Mattan Shop (Bakra for haldi)</v>
       </c>
       <c r="D61" s="3">
-        <v>46299</v>
+        <v>46298</v>
       </c>
       <c r="E61" s="1">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="F61" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G61" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H61" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2b0b3096</v>
+        <v>09899d1e</v>
       </c>
       <c r="B62" t="str">
-        <v>08cd3226</v>
+        <v>c1c67a32</v>
       </c>
       <c r="C62" t="str">
-        <v>Meher Amount</v>
+        <v>car decoration, Dj, Petrol, Haldi Celender</v>
       </c>
       <c r="D62" s="3">
         <v>46299</v>
       </c>
       <c r="E62" s="1">
-        <v>11111</v>
+        <v>30000</v>
       </c>
       <c r="F62" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G62" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H62" t="str">
         <v/>
@@ -3173,19 +3173,19 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>fc7adcbd</v>
+        <v>2b0b3096</v>
       </c>
       <c r="B63" t="str">
-        <v>04ece648</v>
+        <v>08cd3226</v>
       </c>
       <c r="C63" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Meher Amount</v>
       </c>
       <c r="D63" s="3">
-        <v>46300</v>
+        <v>46299</v>
       </c>
       <c r="E63" s="1">
-        <v>15000</v>
+        <v>11111</v>
       </c>
       <c r="F63" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3194,24 +3194,24 @@
         <v>Cash</v>
       </c>
       <c r="H63" t="str">
-        <v>payment done</v>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>384605f7</v>
+        <v>fc7adcbd</v>
       </c>
       <c r="B64" t="str">
-        <v>22ff3fb2</v>
+        <v>04ece648</v>
       </c>
       <c r="C64" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="D64" s="3">
         <v>46300</v>
       </c>
       <c r="E64" s="1">
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="F64" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3220,24 +3220,24 @@
         <v>Cash</v>
       </c>
       <c r="H64" t="str">
-        <v/>
+        <v>payment done</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>d08ebf7d</v>
+        <v>384605f7</v>
       </c>
       <c r="B65" t="str">
-        <v>9b3747da</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C65" t="str">
-        <v>tampo traveller</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D65" s="3">
         <v>46300</v>
       </c>
       <c r="E65" s="1">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="F65" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3246,50 +3246,50 @@
         <v>Cash</v>
       </c>
       <c r="H65" t="str">
-        <v>cash</v>
+        <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>3adcd8de</v>
+        <v>d08ebf7d</v>
       </c>
       <c r="B66" t="str">
-        <v>4d3bd5b1</v>
+        <v>9b3747da</v>
       </c>
       <c r="C66" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>tampo traveller</v>
       </c>
       <c r="D66" s="3">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E66" s="1">
-        <v>24000</v>
+        <v>7500</v>
       </c>
       <c r="F66" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G66" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H66" t="str">
-        <v>Final payment</v>
+        <v>cash</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>4f298a0d</v>
+        <v>3adcd8de</v>
       </c>
       <c r="B67" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C67" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D67" s="3">
         <v>46302</v>
       </c>
       <c r="E67" s="1">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="F67" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3298,24 +3298,24 @@
         <v>UPI</v>
       </c>
       <c r="H67" t="str">
-        <v>Installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>141e8fbb</v>
+        <v>4f298a0d</v>
       </c>
       <c r="B68" t="str">
-        <v>4d3bd5b1</v>
+        <v>631875ca</v>
       </c>
       <c r="C68" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D68" s="3">
         <v>46302</v>
       </c>
       <c r="E68" s="1">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="F68" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3324,50 +3324,50 @@
         <v>UPI</v>
       </c>
       <c r="H68" t="str">
-        <v>paid</v>
+        <v>Installment</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>738b696a</v>
+        <v>141e8fbb</v>
       </c>
       <c r="B69" t="str">
-        <v>f31def6e</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C69" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D69" s="3">
         <v>46302</v>
       </c>
       <c r="E69" s="1">
-        <v>13000</v>
+        <v>500</v>
       </c>
       <c r="F69" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G69" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H69" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>ad864ef1</v>
+        <v>738b696a</v>
       </c>
       <c r="B70" t="str">
-        <v>c047acbd</v>
+        <v>f31def6e</v>
       </c>
       <c r="C70" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="D70" s="3">
         <v>46302</v>
       </c>
       <c r="E70" s="1">
-        <v>6000</v>
+        <v>13000</v>
       </c>
       <c r="F70" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3381,123 +3381,123 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>da6b0ec5</v>
+        <v>ad864ef1</v>
       </c>
       <c r="B71" t="str">
-        <v>631875ca</v>
+        <v>c047acbd</v>
       </c>
       <c r="C71" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="D71" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E71" s="1">
-        <v>33000</v>
+        <v>6000</v>
       </c>
       <c r="F71" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G71" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H71" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B72" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C72" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D72" s="3">
         <v>46303</v>
       </c>
       <c r="E72" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F72" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G72" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H72" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B73" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C73" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D73" s="3">
         <v>46303</v>
       </c>
       <c r="E73" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F73" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G73" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H73" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>79cb1a7e</v>
+        <v>80e653df</v>
       </c>
       <c r="B74" t="str">
-        <v>22ff3fb2</v>
+        <v>beb44857</v>
       </c>
       <c r="C74" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D74" s="3">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E74" s="1">
-        <v>1000</v>
+        <v>30000</v>
       </c>
       <c r="F74" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G74" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H74" t="str">
-        <v>final payment</v>
+        <v>Second last installment</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>fcb3d16a</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B75" t="str">
-        <v>70d7465c</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C75" t="str">
-        <v>3 kg asli ghee</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D75" s="3">
         <v>46306</v>
       </c>
       <c r="E75" s="1">
-        <v>1830</v>
+        <v>1000</v>
       </c>
       <c r="F75" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3506,13 +3506,39 @@
         <v>Cash</v>
       </c>
       <c r="H75" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B76" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C76" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D76" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E76" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G76" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H76" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H75"/>
+  <autoFilter ref="A1:H76"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H76"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4146,11 +4172,11 @@
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -4600,11 +4626,11 @@
       </c>
       <c r="D57" s="1">
         <f>SUM(D2:D56)</f>
-        <v>1275679</v>
+        <v>1290679</v>
       </c>
       <c r="E57" s="1">
         <f>SUM(E2:E56)</f>
-        <v>45000</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Sehera, Har, Guche & Gajre — ₹9,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H76</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1399,16 +1399,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>c047acbd</v>
+        <v>5ddff322</v>
       </c>
       <c r="B50" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="C50" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="D50" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E50" s="2" t="str">
         <v/>
@@ -1419,128 +1419,148 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>d1aee56d</v>
+        <v>c047acbd</v>
       </c>
       <c r="B51" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="C51" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D51" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E51" s="2" t="str">
         <v/>
       </c>
       <c r="F51" t="str">
-        <v>Shireen Dress</v>
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B52" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C52" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D52" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E52" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F52" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B53" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C53" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D53" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E53" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F53" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B54" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C54" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D54" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E54" s="2" t="str">
         <v/>
       </c>
       <c r="F54" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B55" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C55" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D55" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E55" s="2" t="str">
         <v/>
       </c>
       <c r="F55" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D56" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E56" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B56" t="str">
+      <c r="B57" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C56" t="str">
+      <c r="C57" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D57" s="1">
         <v>9150</v>
       </c>
-      <c r="E56" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F56" t="str">
+      <c r="E57" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F56"/>
+  <autoFilter ref="A1:F57"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F57"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3545,7 +3565,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4485,36 +4505,36 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="B50" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="C50" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
-        <v>0</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="B51" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C51" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4523,17 +4543,17 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B52" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C52" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4542,17 +4562,17 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B53" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C53" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D53" s="1">
         <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E53" s="1">
         <f>C53-D53</f>
@@ -4561,17 +4581,17 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B54" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C54" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D54" s="1">
         <f>SUMIF('Payments'!$C:$C,$A54,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E54" s="1">
         <f>C54-D54</f>
@@ -4580,17 +4600,17 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B55" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C55" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D55" s="1">
         <f>SUMIF('Payments'!$C:$C,$A55,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E55" s="1">
         <f>C55-D55</f>
@@ -4599,17 +4619,17 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B56" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C56" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D56" s="1">
         <f>SUMIF('Payments'!$C:$C,$A56,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E56" s="1">
         <f>C56-D56</f>
@@ -4618,24 +4638,43 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C57" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D57" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A57,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E57" s="1">
+        <f>C57-D57</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
         <v>Total</v>
       </c>
-      <c r="C57" s="1">
-        <f>SUM(C2:C56)</f>
-        <v>1320679</v>
-      </c>
-      <c r="D57" s="1">
-        <f>SUM(D2:D56)</f>
+      <c r="C58" s="1">
+        <f>SUM(C2:C57)</f>
+        <v>1329679</v>
+      </c>
+      <c r="D58" s="1">
+        <f>SUM(D2:D57)</f>
         <v>1290679</v>
       </c>
-      <c r="E57" s="1">
-        <f>SUM(E2:E56)</f>
-        <v>30000</v>
+      <c r="E58" s="1">
+        <f>SUM(E2:E57)</f>
+        <v>39000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹9,000.00 by Umar Sayyed (Father) for Sehera, Har, Guche & Gajre
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H77</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1567,7 +1567,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3219,19 +3219,19 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>fc7adcbd</v>
+        <v>113db2d6</v>
       </c>
       <c r="B64" t="str">
-        <v>04ece648</v>
+        <v>5ddff322</v>
       </c>
       <c r="C64" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="D64" s="3">
-        <v>46300</v>
+        <v>46299</v>
       </c>
       <c r="E64" s="1">
-        <v>15000</v>
+        <v>9000</v>
       </c>
       <c r="F64" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3240,24 +3240,24 @@
         <v>Cash</v>
       </c>
       <c r="H64" t="str">
-        <v>payment done</v>
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>384605f7</v>
+        <v>fc7adcbd</v>
       </c>
       <c r="B65" t="str">
-        <v>22ff3fb2</v>
+        <v>04ece648</v>
       </c>
       <c r="C65" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="D65" s="3">
         <v>46300</v>
       </c>
       <c r="E65" s="1">
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="F65" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3266,24 +3266,24 @@
         <v>Cash</v>
       </c>
       <c r="H65" t="str">
-        <v/>
+        <v>payment done</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>d08ebf7d</v>
+        <v>384605f7</v>
       </c>
       <c r="B66" t="str">
-        <v>9b3747da</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C66" t="str">
-        <v>tampo traveller</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D66" s="3">
         <v>46300</v>
       </c>
       <c r="E66" s="1">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="F66" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3292,50 +3292,50 @@
         <v>Cash</v>
       </c>
       <c r="H66" t="str">
-        <v>cash</v>
+        <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>3adcd8de</v>
+        <v>d08ebf7d</v>
       </c>
       <c r="B67" t="str">
-        <v>4d3bd5b1</v>
+        <v>9b3747da</v>
       </c>
       <c r="C67" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>tampo traveller</v>
       </c>
       <c r="D67" s="3">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E67" s="1">
-        <v>24000</v>
+        <v>7500</v>
       </c>
       <c r="F67" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G67" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H67" t="str">
-        <v>Final payment</v>
+        <v>cash</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>4f298a0d</v>
+        <v>3adcd8de</v>
       </c>
       <c r="B68" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C68" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D68" s="3">
         <v>46302</v>
       </c>
       <c r="E68" s="1">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="F68" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3344,24 +3344,24 @@
         <v>UPI</v>
       </c>
       <c r="H68" t="str">
-        <v>Installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>141e8fbb</v>
+        <v>4f298a0d</v>
       </c>
       <c r="B69" t="str">
-        <v>4d3bd5b1</v>
+        <v>631875ca</v>
       </c>
       <c r="C69" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D69" s="3">
         <v>46302</v>
       </c>
       <c r="E69" s="1">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="F69" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3370,50 +3370,50 @@
         <v>UPI</v>
       </c>
       <c r="H69" t="str">
-        <v>paid</v>
+        <v>Installment</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>738b696a</v>
+        <v>141e8fbb</v>
       </c>
       <c r="B70" t="str">
-        <v>f31def6e</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C70" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D70" s="3">
         <v>46302</v>
       </c>
       <c r="E70" s="1">
-        <v>13000</v>
+        <v>500</v>
       </c>
       <c r="F70" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G70" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H70" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>ad864ef1</v>
+        <v>738b696a</v>
       </c>
       <c r="B71" t="str">
-        <v>c047acbd</v>
+        <v>f31def6e</v>
       </c>
       <c r="C71" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="D71" s="3">
         <v>46302</v>
       </c>
       <c r="E71" s="1">
-        <v>6000</v>
+        <v>13000</v>
       </c>
       <c r="F71" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3427,123 +3427,123 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>da6b0ec5</v>
+        <v>ad864ef1</v>
       </c>
       <c r="B72" t="str">
-        <v>631875ca</v>
+        <v>c047acbd</v>
       </c>
       <c r="C72" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="D72" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E72" s="1">
-        <v>33000</v>
+        <v>6000</v>
       </c>
       <c r="F72" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G72" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H72" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B73" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C73" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D73" s="3">
         <v>46303</v>
       </c>
       <c r="E73" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F73" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G73" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H73" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B74" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C74" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D74" s="3">
         <v>46303</v>
       </c>
       <c r="E74" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F74" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G74" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H74" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>79cb1a7e</v>
+        <v>80e653df</v>
       </c>
       <c r="B75" t="str">
-        <v>22ff3fb2</v>
+        <v>beb44857</v>
       </c>
       <c r="C75" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D75" s="3">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E75" s="1">
-        <v>1000</v>
+        <v>30000</v>
       </c>
       <c r="F75" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G75" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H75" t="str">
-        <v>final payment</v>
+        <v>Second last installment</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>fcb3d16a</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B76" t="str">
-        <v>70d7465c</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C76" t="str">
-        <v>3 kg asli ghee</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D76" s="3">
         <v>46306</v>
       </c>
       <c r="E76" s="1">
-        <v>1830</v>
+        <v>1000</v>
       </c>
       <c r="F76" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3552,13 +3552,39 @@
         <v>Cash</v>
       </c>
       <c r="H76" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B77" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C77" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D77" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E77" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F77" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G77" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H77" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H76"/>
+  <autoFilter ref="A1:H77"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H77"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4515,11 +4541,11 @@
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
-        <v>9000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -4665,11 +4691,11 @@
       </c>
       <c r="D58" s="1">
         <f>SUM(D2:D57)</f>
-        <v>1290679</v>
+        <v>1299679</v>
       </c>
       <c r="E58" s="1">
         <f>SUM(E2:E57)</f>
-        <v>39000</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Lunch After Mariage Shiv Sunder — ₹2,700.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H77</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1019,16 +1019,16 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>08cd3226</v>
+        <v>f7330587</v>
       </c>
       <c r="B31" t="str">
-        <v>Meher Amount</v>
+        <v>Lunch After Mariage Shiv Sunder</v>
       </c>
       <c r="C31" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D31" s="1">
-        <v>11111</v>
+        <v>2700</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
@@ -1039,16 +1039,16 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>a1def8e4</v>
+        <v>08cd3226</v>
       </c>
       <c r="B32" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Meher Amount</v>
       </c>
       <c r="C32" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D32" s="1">
-        <v>5412</v>
+        <v>11111</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
@@ -1059,16 +1059,16 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>87751d8e</v>
+        <v>a1def8e4</v>
       </c>
       <c r="B33" t="str">
-        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="C33" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D33" s="1">
-        <v>15000</v>
+        <v>5412</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
@@ -1079,116 +1079,116 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>c7e8b352</v>
+        <v>87751d8e</v>
       </c>
       <c r="B34" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
       </c>
       <c r="C34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D34" s="1">
-        <v>7604</v>
+        <v>15000</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B35" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C35" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B36" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C36" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B37" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C37" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D37" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B38" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C38" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D38" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B39" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C39" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D39" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
@@ -1199,16 +1199,16 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>f31def6e</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B40" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C40" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D40" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
@@ -1219,113 +1219,113 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>eebc3aaf</v>
+        <v>f31def6e</v>
       </c>
       <c r="B41" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="C41" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D41" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E41" s="2" t="str">
         <v/>
       </c>
       <c r="F41" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B42" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C42" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D42" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E42" s="2" t="str">
         <v/>
       </c>
       <c r="F42" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B43" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C43" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D43" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E43" s="2" t="str">
         <v/>
       </c>
       <c r="F43" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B44" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C44" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D44" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E44" s="2" t="str">
         <v/>
       </c>
       <c r="F44" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B45" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C45" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D45" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E45" s="2" t="str">
         <v/>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B46" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C46" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D46" s="1">
         <v>4000</v>
@@ -1339,96 +1339,96 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B47" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C47" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D47" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E47" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F47" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B48" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C48" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D48" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E48" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F48" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B49" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C49" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D49" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E49" s="2" t="str">
         <v/>
       </c>
       <c r="F49" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>5ddff322</v>
+        <v>6d180155</v>
       </c>
       <c r="B50" t="str">
-        <v>Sehera, Har, Guche &amp; Gajre</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C50" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D50" s="1">
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="E50" s="2" t="str">
         <v/>
       </c>
       <c r="F50" t="str">
-        <v/>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>c047acbd</v>
+        <v>5ddff322</v>
       </c>
       <c r="B51" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="C51" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="D51" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E51" s="2" t="str">
         <v/>
@@ -1439,128 +1439,148 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>d1aee56d</v>
+        <v>c047acbd</v>
       </c>
       <c r="B52" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="C52" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D52" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E52" s="2" t="str">
         <v/>
       </c>
       <c r="F52" t="str">
-        <v>Shireen Dress</v>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B53" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C53" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D53" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E53" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F53" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B54" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C54" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D54" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E54" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F54" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B55" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C55" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D55" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E55" s="2" t="str">
         <v/>
       </c>
       <c r="F55" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B56" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C56" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D56" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E56" s="2" t="str">
         <v/>
       </c>
       <c r="F56" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D57" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E57" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B57" t="str">
+      <c r="B58" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C57" t="str">
+      <c r="C58" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D57" s="1">
+      <c r="D58" s="1">
         <v>9150</v>
       </c>
-      <c r="E57" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F57" t="str">
+      <c r="E58" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F58" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F57"/>
+  <autoFilter ref="A1:F58"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F58"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3591,7 +3611,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4170,36 +4190,36 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Meher Amount</v>
+        <v>Lunch After Mariage Shiv Sunder</v>
       </c>
       <c r="B31" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C31" s="1">
-        <v>11111</v>
+        <v>2700</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>11111</v>
+        <v>0</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
-        <v>0</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Meher Amount</v>
       </c>
       <c r="B32" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C32" s="1">
-        <v>5412</v>
+        <v>11111</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>5412</v>
+        <v>11111</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -4208,17 +4228,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="B33" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C33" s="1">
-        <v>15000</v>
+        <v>5412</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>5412</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -4227,17 +4247,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
       </c>
       <c r="B34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C34" s="1">
-        <v>7604</v>
+        <v>15000</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>15000</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -4246,17 +4266,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B35" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -4265,17 +4285,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B36" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -4284,17 +4304,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B37" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C37" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -4303,17 +4323,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B38" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C38" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -4322,17 +4342,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B39" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C39" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -4341,17 +4361,17 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B40" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C40" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -4360,17 +4380,17 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="B41" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C41" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -4379,17 +4399,17 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B42" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C42" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
@@ -4398,17 +4418,17 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B43" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C43" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
@@ -4417,17 +4437,17 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B44" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C44" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
@@ -4436,17 +4456,17 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B45" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C45" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
@@ -4455,10 +4475,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B46" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C46" s="1">
         <v>4000</v>
@@ -4474,55 +4494,55 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B47" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C47" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B48" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C48" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B49" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C49" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
@@ -4531,17 +4551,17 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Sehera, Har, Guche &amp; Gajre</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B50" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C50" s="1">
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
@@ -4550,17 +4570,17 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="B51" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="C51" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4569,17 +4589,17 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="B52" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C52" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4588,17 +4608,17 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B53" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C53" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D53" s="1">
         <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E53" s="1">
         <f>C53-D53</f>
@@ -4607,17 +4627,17 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B54" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C54" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D54" s="1">
         <f>SUMIF('Payments'!$C:$C,$A54,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E54" s="1">
         <f>C54-D54</f>
@@ -4626,17 +4646,17 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B55" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C55" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D55" s="1">
         <f>SUMIF('Payments'!$C:$C,$A55,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E55" s="1">
         <f>C55-D55</f>
@@ -4645,17 +4665,17 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B56" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C56" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D56" s="1">
         <f>SUMIF('Payments'!$C:$C,$A56,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E56" s="1">
         <f>C56-D56</f>
@@ -4664,17 +4684,17 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B57" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C57" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D57" s="1">
         <f>SUMIF('Payments'!$C:$C,$A57,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E57" s="1">
         <f>C57-D57</f>
@@ -4683,24 +4703,43 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C58" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D58" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A58,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E58" s="1">
+        <f>C58-D58</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
         <v>Total</v>
       </c>
-      <c r="C58" s="1">
-        <f>SUM(C2:C57)</f>
-        <v>1329679</v>
-      </c>
-      <c r="D58" s="1">
-        <f>SUM(D2:D57)</f>
+      <c r="C59" s="1">
+        <f>SUM(C2:C58)</f>
+        <v>1332379</v>
+      </c>
+      <c r="D59" s="1">
+        <f>SUM(D2:D58)</f>
         <v>1299679</v>
       </c>
-      <c r="E58" s="1">
-        <f>SUM(E2:E57)</f>
-        <v>30000</v>
+      <c r="E59" s="1">
+        <f>SUM(E2:E58)</f>
+        <v>32700</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E59"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹2,700.00 by Waheeda (mother) for Lunch After Mariage Shiv Sunder
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F58</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H78</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1587,7 +1587,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3551,45 +3551,45 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>79cb1a7e</v>
+        <v>bb9651a4</v>
       </c>
       <c r="B76" t="str">
-        <v>22ff3fb2</v>
+        <v>f7330587</v>
       </c>
       <c r="C76" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Lunch After Mariage Shiv Sunder</v>
       </c>
       <c r="D76" s="3">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E76" s="1">
-        <v>1000</v>
+        <v>2700</v>
       </c>
       <c r="F76" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G76" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H76" t="str">
-        <v>final payment</v>
+        <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>fcb3d16a</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B77" t="str">
-        <v>70d7465c</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C77" t="str">
-        <v>3 kg asli ghee</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D77" s="3">
         <v>46306</v>
       </c>
       <c r="E77" s="1">
-        <v>1830</v>
+        <v>1000</v>
       </c>
       <c r="F77" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3598,13 +3598,39 @@
         <v>Cash</v>
       </c>
       <c r="H77" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B78" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C78" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D78" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E78" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G78" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H78" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H77"/>
+  <autoFilter ref="A1:H78"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H78"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4200,11 +4226,11 @@
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>2700</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
-        <v>2700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4730,11 +4756,11 @@
       </c>
       <c r="D59" s="1">
         <f>SUM(D2:D58)</f>
-        <v>1299679</v>
+        <v>1302379</v>
       </c>
       <c r="E59" s="1">
         <f>SUM(E2:E58)</f>
-        <v>32700</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Patti mudekhai — ₹5,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H78</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1319,16 +1319,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>0421ab42</v>
+        <v>9299bcdc</v>
       </c>
       <c r="B46" t="str">
-        <v>Petrol Glanza</v>
+        <v>Patti mudekhai</v>
       </c>
       <c r="C46" t="str">
-        <v>Miscellaneous</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D46" s="1">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="E46" s="2" t="str">
         <v/>
@@ -1339,13 +1339,13 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>84c049af</v>
+        <v>0421ab42</v>
       </c>
       <c r="B47" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C47" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D47" s="1">
         <v>4000</v>
@@ -1359,96 +1359,96 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B48" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C48" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D48" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E48" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F48" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B49" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C49" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D49" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E49" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F49" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B50" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C50" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D50" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E50" s="2" t="str">
         <v/>
       </c>
       <c r="F50" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>5ddff322</v>
+        <v>6d180155</v>
       </c>
       <c r="B51" t="str">
-        <v>Sehera, Har, Guche &amp; Gajre</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C51" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D51" s="1">
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="E51" s="2" t="str">
         <v/>
       </c>
       <c r="F51" t="str">
-        <v/>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>c047acbd</v>
+        <v>5ddff322</v>
       </c>
       <c r="B52" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="C52" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="D52" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E52" s="2" t="str">
         <v/>
@@ -1459,128 +1459,148 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>d1aee56d</v>
+        <v>c047acbd</v>
       </c>
       <c r="B53" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="C53" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D53" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E53" s="2" t="str">
         <v/>
       </c>
       <c r="F53" t="str">
-        <v>Shireen Dress</v>
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B54" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C54" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D54" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E54" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F54" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B55" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C55" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D55" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E55" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F55" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B56" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C56" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D56" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E56" s="2" t="str">
         <v/>
       </c>
       <c r="F56" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B57" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C57" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D57" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E57" s="2" t="str">
         <v/>
       </c>
       <c r="F57" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D58" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E58" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F58" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B58" t="str">
+      <c r="B59" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C58" t="str">
+      <c r="C59" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D59" s="1">
         <v>9150</v>
       </c>
-      <c r="E58" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F58" t="str">
+      <c r="E59" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F59" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F58"/>
+  <autoFilter ref="A1:F59"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F59"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3637,7 +3657,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E60"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4501,29 +4521,29 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Petrol Glanza</v>
+        <v>Patti mudekhai</v>
       </c>
       <c r="B46" t="str">
-        <v>Miscellaneous</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C46" s="1">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B47" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C47" s="1">
         <v>4000</v>
@@ -4539,55 +4559,55 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B48" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C48" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B49" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C49" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B50" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C50" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
@@ -4596,17 +4616,17 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Sehera, Har, Guche &amp; Gajre</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B51" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C51" s="1">
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4615,17 +4635,17 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="B52" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="C52" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4634,17 +4654,17 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="B53" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C53" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="D53" s="1">
         <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E53" s="1">
         <f>C53-D53</f>
@@ -4653,17 +4673,17 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B54" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C54" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D54" s="1">
         <f>SUMIF('Payments'!$C:$C,$A54,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E54" s="1">
         <f>C54-D54</f>
@@ -4672,17 +4692,17 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B55" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C55" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D55" s="1">
         <f>SUMIF('Payments'!$C:$C,$A55,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E55" s="1">
         <f>C55-D55</f>
@@ -4691,17 +4711,17 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B56" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C56" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D56" s="1">
         <f>SUMIF('Payments'!$C:$C,$A56,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E56" s="1">
         <f>C56-D56</f>
@@ -4710,17 +4730,17 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B57" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C57" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D57" s="1">
         <f>SUMIF('Payments'!$C:$C,$A57,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E57" s="1">
         <f>C57-D57</f>
@@ -4729,17 +4749,17 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B58" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C58" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D58" s="1">
         <f>SUMIF('Payments'!$C:$C,$A58,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E58" s="1">
         <f>C58-D58</f>
@@ -4748,24 +4768,43 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C59" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D59" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A59,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E59" s="1">
+        <f>C59-D59</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
         <v>Total</v>
       </c>
-      <c r="C59" s="1">
-        <f>SUM(C2:C58)</f>
-        <v>1332379</v>
-      </c>
-      <c r="D59" s="1">
-        <f>SUM(D2:D58)</f>
+      <c r="C60" s="1">
+        <f>SUM(C2:C59)</f>
+        <v>1337379</v>
+      </c>
+      <c r="D60" s="1">
+        <f>SUM(D2:D59)</f>
         <v>1302379</v>
       </c>
-      <c r="E59" s="1">
-        <f>SUM(E2:E58)</f>
-        <v>30000</v>
+      <c r="E60" s="1">
+        <f>SUM(E2:E59)</f>
+        <v>35000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E60"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹5,000.00 by Waheeda (mother) for Patti mudekhai
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H79</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1607,7 +1607,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3363,45 +3363,45 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>3adcd8de</v>
+        <v>c193f7b5</v>
       </c>
       <c r="B68" t="str">
-        <v>4d3bd5b1</v>
+        <v>9299bcdc</v>
       </c>
       <c r="C68" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Patti mudekhai</v>
       </c>
       <c r="D68" s="3">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E68" s="1">
-        <v>24000</v>
+        <v>5000</v>
       </c>
       <c r="F68" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G68" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H68" t="str">
-        <v>Final payment</v>
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>4f298a0d</v>
+        <v>3adcd8de</v>
       </c>
       <c r="B69" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C69" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D69" s="3">
         <v>46302</v>
       </c>
       <c r="E69" s="1">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="F69" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3410,24 +3410,24 @@
         <v>UPI</v>
       </c>
       <c r="H69" t="str">
-        <v>Installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>141e8fbb</v>
+        <v>4f298a0d</v>
       </c>
       <c r="B70" t="str">
-        <v>4d3bd5b1</v>
+        <v>631875ca</v>
       </c>
       <c r="C70" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D70" s="3">
         <v>46302</v>
       </c>
       <c r="E70" s="1">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="F70" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3436,50 +3436,50 @@
         <v>UPI</v>
       </c>
       <c r="H70" t="str">
-        <v>paid</v>
+        <v>Installment</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>738b696a</v>
+        <v>141e8fbb</v>
       </c>
       <c r="B71" t="str">
-        <v>f31def6e</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C71" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D71" s="3">
         <v>46302</v>
       </c>
       <c r="E71" s="1">
-        <v>13000</v>
+        <v>500</v>
       </c>
       <c r="F71" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G71" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H71" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>ad864ef1</v>
+        <v>738b696a</v>
       </c>
       <c r="B72" t="str">
-        <v>c047acbd</v>
+        <v>f31def6e</v>
       </c>
       <c r="C72" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="D72" s="3">
         <v>46302</v>
       </c>
       <c r="E72" s="1">
-        <v>6000</v>
+        <v>13000</v>
       </c>
       <c r="F72" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3493,149 +3493,149 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>da6b0ec5</v>
+        <v>ad864ef1</v>
       </c>
       <c r="B73" t="str">
-        <v>631875ca</v>
+        <v>c047acbd</v>
       </c>
       <c r="C73" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="D73" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E73" s="1">
-        <v>33000</v>
+        <v>6000</v>
       </c>
       <c r="F73" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G73" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H73" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B74" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C74" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D74" s="3">
         <v>46303</v>
       </c>
       <c r="E74" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F74" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G74" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H74" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B75" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C75" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D75" s="3">
         <v>46303</v>
       </c>
       <c r="E75" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F75" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G75" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H75" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>bb9651a4</v>
+        <v>80e653df</v>
       </c>
       <c r="B76" t="str">
-        <v>f7330587</v>
+        <v>beb44857</v>
       </c>
       <c r="C76" t="str">
-        <v>Lunch After Mariage Shiv Sunder</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D76" s="3">
         <v>46303</v>
       </c>
       <c r="E76" s="1">
-        <v>2700</v>
+        <v>30000</v>
       </c>
       <c r="F76" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G76" t="str">
         <v>UPI</v>
       </c>
       <c r="H76" t="str">
-        <v/>
+        <v>Second last installment</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>79cb1a7e</v>
+        <v>bb9651a4</v>
       </c>
       <c r="B77" t="str">
-        <v>22ff3fb2</v>
+        <v>f7330587</v>
       </c>
       <c r="C77" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Lunch After Mariage Shiv Sunder</v>
       </c>
       <c r="D77" s="3">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E77" s="1">
-        <v>1000</v>
+        <v>2700</v>
       </c>
       <c r="F77" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G77" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H77" t="str">
-        <v>final payment</v>
+        <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>fcb3d16a</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B78" t="str">
-        <v>70d7465c</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C78" t="str">
-        <v>3 kg asli ghee</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D78" s="3">
         <v>46306</v>
       </c>
       <c r="E78" s="1">
-        <v>1830</v>
+        <v>1000</v>
       </c>
       <c r="F78" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3644,13 +3644,39 @@
         <v>Cash</v>
       </c>
       <c r="H78" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B79" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C79" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D79" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E79" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F79" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G79" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H79" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H78"/>
+  <autoFilter ref="A1:H79"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H79"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4531,11 +4557,11 @@
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -4795,11 +4821,11 @@
       </c>
       <c r="D60" s="1">
         <f>SUM(D2:D59)</f>
-        <v>1302379</v>
+        <v>1307379</v>
       </c>
       <c r="E60" s="1">
         <f>SUM(E2:E59)</f>
-        <v>35000</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Petrol Glanza Darga visit — ₹3,226.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H79</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1359,16 +1359,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>84c049af</v>
+        <v>fed12b4d</v>
       </c>
       <c r="B48" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza Darga visit</v>
       </c>
       <c r="C48" t="str">
         <v>Transport</v>
       </c>
       <c r="D48" s="1">
-        <v>4000</v>
+        <v>3226</v>
       </c>
       <c r="E48" s="2" t="str">
         <v/>
@@ -1379,96 +1379,96 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B49" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C49" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D49" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E49" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F49" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B50" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C50" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D50" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E50" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F50" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B51" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C51" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D51" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E51" s="2" t="str">
         <v/>
       </c>
       <c r="F51" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>5ddff322</v>
+        <v>6d180155</v>
       </c>
       <c r="B52" t="str">
-        <v>Sehera, Har, Guche &amp; Gajre</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C52" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D52" s="1">
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="E52" s="2" t="str">
         <v/>
       </c>
       <c r="F52" t="str">
-        <v/>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>c047acbd</v>
+        <v>5ddff322</v>
       </c>
       <c r="B53" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="C53" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="D53" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E53" s="2" t="str">
         <v/>
@@ -1479,128 +1479,148 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>d1aee56d</v>
+        <v>c047acbd</v>
       </c>
       <c r="B54" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="C54" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D54" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E54" s="2" t="str">
         <v/>
       </c>
       <c r="F54" t="str">
-        <v>Shireen Dress</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B55" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C55" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D55" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E55" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F55" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B56" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C56" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D56" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E56" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F56" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B57" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C57" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D57" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E57" s="2" t="str">
         <v/>
       </c>
       <c r="F57" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B58" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C58" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D58" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E58" s="2" t="str">
         <v/>
       </c>
       <c r="F58" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D59" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E59" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F59" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B59" t="str">
+      <c r="B60" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C59" t="str">
+      <c r="C60" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D59" s="1">
+      <c r="D60" s="1">
         <v>9150</v>
       </c>
-      <c r="E59" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F59" t="str">
+      <c r="E60" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F59"/>
+  <autoFilter ref="A1:F60"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F60"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3683,7 +3703,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4585,74 +4605,74 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza Darga visit</v>
       </c>
       <c r="B48" t="str">
         <v>Transport</v>
       </c>
       <c r="C48" s="1">
-        <v>4000</v>
+        <v>3226</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
-        <v>0</v>
+        <v>3226</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B49" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C49" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B50" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C50" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B51" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C51" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
@@ -4661,17 +4681,17 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Sehera, Har, Guche &amp; Gajre</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B52" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C52" s="1">
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4680,17 +4700,17 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="B53" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="C53" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="D53" s="1">
         <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E53" s="1">
         <f>C53-D53</f>
@@ -4699,17 +4719,17 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="B54" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C54" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="D54" s="1">
         <f>SUMIF('Payments'!$C:$C,$A54,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E54" s="1">
         <f>C54-D54</f>
@@ -4718,17 +4738,17 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B55" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C55" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D55" s="1">
         <f>SUMIF('Payments'!$C:$C,$A55,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E55" s="1">
         <f>C55-D55</f>
@@ -4737,17 +4757,17 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B56" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C56" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D56" s="1">
         <f>SUMIF('Payments'!$C:$C,$A56,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E56" s="1">
         <f>C56-D56</f>
@@ -4756,17 +4776,17 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B57" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C57" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D57" s="1">
         <f>SUMIF('Payments'!$C:$C,$A57,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E57" s="1">
         <f>C57-D57</f>
@@ -4775,17 +4795,17 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B58" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C58" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D58" s="1">
         <f>SUMIF('Payments'!$C:$C,$A58,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E58" s="1">
         <f>C58-D58</f>
@@ -4794,17 +4814,17 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B59" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C59" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D59" s="1">
         <f>SUMIF('Payments'!$C:$C,$A59,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E59" s="1">
         <f>C59-D59</f>
@@ -4813,24 +4833,43 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C60" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D60" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A60,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E60" s="1">
+        <f>C60-D60</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
         <v>Total</v>
       </c>
-      <c r="C60" s="1">
-        <f>SUM(C2:C59)</f>
-        <v>1337379</v>
-      </c>
-      <c r="D60" s="1">
-        <f>SUM(D2:D59)</f>
+      <c r="C61" s="1">
+        <f>SUM(C2:C60)</f>
+        <v>1340605</v>
+      </c>
+      <c r="D61" s="1">
+        <f>SUM(D2:D60)</f>
         <v>1307379</v>
       </c>
-      <c r="E60" s="1">
-        <f>SUM(E2:E59)</f>
-        <v>30000</v>
+      <c r="E61" s="1">
+        <f>SUM(E2:E60)</f>
+        <v>33226</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹3,226.00 by Umar Sayyed (Father) for Petrol Glanza Darga visit
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H80</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1627,7 +1627,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3409,45 +3409,45 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>3adcd8de</v>
+        <v>5a34da87</v>
       </c>
       <c r="B69" t="str">
-        <v>4d3bd5b1</v>
+        <v>fed12b4d</v>
       </c>
       <c r="C69" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Petrol Glanza Darga visit</v>
       </c>
       <c r="D69" s="3">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E69" s="1">
-        <v>24000</v>
+        <v>3226</v>
       </c>
       <c r="F69" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G69" t="str">
-        <v>UPI</v>
+        <v>Debit Card</v>
       </c>
       <c r="H69" t="str">
-        <v>Final payment</v>
+        <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>4f298a0d</v>
+        <v>3adcd8de</v>
       </c>
       <c r="B70" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C70" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D70" s="3">
         <v>46302</v>
       </c>
       <c r="E70" s="1">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="F70" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3456,24 +3456,24 @@
         <v>UPI</v>
       </c>
       <c r="H70" t="str">
-        <v>Installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>141e8fbb</v>
+        <v>4f298a0d</v>
       </c>
       <c r="B71" t="str">
-        <v>4d3bd5b1</v>
+        <v>631875ca</v>
       </c>
       <c r="C71" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D71" s="3">
         <v>46302</v>
       </c>
       <c r="E71" s="1">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="F71" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3482,50 +3482,50 @@
         <v>UPI</v>
       </c>
       <c r="H71" t="str">
-        <v>paid</v>
+        <v>Installment</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>738b696a</v>
+        <v>141e8fbb</v>
       </c>
       <c r="B72" t="str">
-        <v>f31def6e</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C72" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D72" s="3">
         <v>46302</v>
       </c>
       <c r="E72" s="1">
-        <v>13000</v>
+        <v>500</v>
       </c>
       <c r="F72" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G72" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H72" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>ad864ef1</v>
+        <v>738b696a</v>
       </c>
       <c r="B73" t="str">
-        <v>c047acbd</v>
+        <v>f31def6e</v>
       </c>
       <c r="C73" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="D73" s="3">
         <v>46302</v>
       </c>
       <c r="E73" s="1">
-        <v>6000</v>
+        <v>13000</v>
       </c>
       <c r="F73" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3539,149 +3539,149 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>da6b0ec5</v>
+        <v>ad864ef1</v>
       </c>
       <c r="B74" t="str">
-        <v>631875ca</v>
+        <v>c047acbd</v>
       </c>
       <c r="C74" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="D74" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E74" s="1">
-        <v>33000</v>
+        <v>6000</v>
       </c>
       <c r="F74" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G74" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H74" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B75" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C75" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D75" s="3">
         <v>46303</v>
       </c>
       <c r="E75" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F75" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G75" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H75" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B76" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C76" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D76" s="3">
         <v>46303</v>
       </c>
       <c r="E76" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F76" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G76" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H76" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>bb9651a4</v>
+        <v>80e653df</v>
       </c>
       <c r="B77" t="str">
-        <v>f7330587</v>
+        <v>beb44857</v>
       </c>
       <c r="C77" t="str">
-        <v>Lunch After Mariage Shiv Sunder</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D77" s="3">
         <v>46303</v>
       </c>
       <c r="E77" s="1">
-        <v>2700</v>
+        <v>30000</v>
       </c>
       <c r="F77" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G77" t="str">
         <v>UPI</v>
       </c>
       <c r="H77" t="str">
-        <v/>
+        <v>Second last installment</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>79cb1a7e</v>
+        <v>bb9651a4</v>
       </c>
       <c r="B78" t="str">
-        <v>22ff3fb2</v>
+        <v>f7330587</v>
       </c>
       <c r="C78" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Lunch After Mariage Shiv Sunder</v>
       </c>
       <c r="D78" s="3">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E78" s="1">
-        <v>1000</v>
+        <v>2700</v>
       </c>
       <c r="F78" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G78" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H78" t="str">
-        <v>final payment</v>
+        <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>fcb3d16a</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B79" t="str">
-        <v>70d7465c</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C79" t="str">
-        <v>3 kg asli ghee</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D79" s="3">
         <v>46306</v>
       </c>
       <c r="E79" s="1">
-        <v>1830</v>
+        <v>1000</v>
       </c>
       <c r="F79" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3690,13 +3690,39 @@
         <v>Cash</v>
       </c>
       <c r="H79" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B80" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C80" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D80" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E80" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F80" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G80" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H80" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H79"/>
+  <autoFilter ref="A1:H80"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H79"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H80"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4615,11 +4641,11 @@
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>3226</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
-        <v>3226</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -4860,11 +4886,11 @@
       </c>
       <c r="D61" s="1">
         <f>SUM(D2:D60)</f>
-        <v>1307379</v>
+        <v>1310605</v>
       </c>
       <c r="E61" s="1">
         <f>SUM(E2:E60)</f>
-        <v>33226</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Gold & Silver — ₹10,70,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H80</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -899,156 +899,156 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>209d43b7</v>
+        <v>bf56437c</v>
       </c>
       <c r="B25" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Gold &amp; Silver</v>
       </c>
       <c r="C25" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>500</v>
+        <v>1070000</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B26" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C26" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D26" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E26" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F26" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>dc70b2a1</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B27" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C27" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D27" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E27" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F27" t="str">
-        <v>internal expense</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>aa710190</v>
+        <v>dc70b2a1</v>
       </c>
       <c r="B28" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="C28" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D28" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E28" s="2" t="str">
-        <v>7385125161</v>
+        <v/>
       </c>
       <c r="F28" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>internal expense</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B29" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C29" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D29" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E29" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F29" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>99d3617a</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B30" t="str">
-        <v>Lucky Mattan Shop (Bakra for haldi)</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C30" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D30" s="1">
-        <v>10000</v>
+        <v>3675</v>
       </c>
       <c r="E30" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F30" t="str">
-        <v>Rahim</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>f7330587</v>
+        <v>99d3617a</v>
       </c>
       <c r="B31" t="str">
-        <v>Lunch After Mariage Shiv Sunder</v>
+        <v>Lucky Mattan Shop (Bakra for haldi)</v>
       </c>
       <c r="C31" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D31" s="1">
-        <v>2700</v>
+        <v>10000</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>Rahim</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>08cd3226</v>
+        <v>f7330587</v>
       </c>
       <c r="B32" t="str">
-        <v>Meher Amount</v>
+        <v>Lunch After Mariage Shiv Sunder</v>
       </c>
       <c r="C32" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D32" s="1">
-        <v>11111</v>
+        <v>2700</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
@@ -1059,16 +1059,16 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>a1def8e4</v>
+        <v>08cd3226</v>
       </c>
       <c r="B33" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Meher Amount</v>
       </c>
       <c r="C33" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D33" s="1">
-        <v>5412</v>
+        <v>11111</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
@@ -1079,16 +1079,16 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>87751d8e</v>
+        <v>a1def8e4</v>
       </c>
       <c r="B34" t="str">
-        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="C34" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D34" s="1">
-        <v>15000</v>
+        <v>5412</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
@@ -1099,116 +1099,116 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>c7e8b352</v>
+        <v>87751d8e</v>
       </c>
       <c r="B35" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
       </c>
       <c r="C35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D35" s="1">
-        <v>7604</v>
+        <v>15000</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Bride reception dress</v>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B36" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C36" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B37" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C37" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D37" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E37" s="2" t="str">
         <v/>
       </c>
       <c r="F37" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B38" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C38" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D38" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E38" s="2" t="str">
         <v/>
       </c>
       <c r="F38" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>b1e7073e</v>
+        <v>a78dd739</v>
       </c>
       <c r="B39" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C39" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D39" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E39" s="2" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>30b69ec5</v>
+        <v>b1e7073e</v>
       </c>
       <c r="B40" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="C40" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D40" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E40" s="2" t="str">
         <v/>
@@ -1219,16 +1219,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>f31def6e</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B41" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C41" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D41" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E41" s="2" t="str">
         <v/>
@@ -1239,116 +1239,116 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>eebc3aaf</v>
+        <v>f31def6e</v>
       </c>
       <c r="B42" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="C42" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="D42" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E42" s="2" t="str">
         <v/>
       </c>
       <c r="F42" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B43" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C43" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D43" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E43" s="2" t="str">
         <v/>
       </c>
       <c r="F43" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B44" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C44" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D44" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E44" s="2" t="str">
         <v/>
       </c>
       <c r="F44" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B45" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C45" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D45" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E45" s="2" t="str">
         <v/>
       </c>
       <c r="F45" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>9299bcdc</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B46" t="str">
-        <v>Patti mudekhai</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C46" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D46" s="1">
-        <v>5000</v>
+        <v>24000</v>
       </c>
       <c r="E46" s="2" t="str">
         <v/>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>0421ab42</v>
+        <v>9299bcdc</v>
       </c>
       <c r="B47" t="str">
-        <v>Petrol Glanza</v>
+        <v>Patti mudekhai</v>
       </c>
       <c r="C47" t="str">
-        <v>Miscellaneous</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D47" s="1">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="E47" s="2" t="str">
         <v/>
@@ -1359,16 +1359,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>fed12b4d</v>
+        <v>0421ab42</v>
       </c>
       <c r="B48" t="str">
-        <v>Petrol Glanza Darga visit</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C48" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D48" s="1">
-        <v>3226</v>
+        <v>4000</v>
       </c>
       <c r="E48" s="2" t="str">
         <v/>
@@ -1379,16 +1379,16 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>84c049af</v>
+        <v>fed12b4d</v>
       </c>
       <c r="B49" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza Darga visit</v>
       </c>
       <c r="C49" t="str">
         <v>Transport</v>
       </c>
       <c r="D49" s="1">
-        <v>4000</v>
+        <v>3226</v>
       </c>
       <c r="E49" s="2" t="str">
         <v/>
@@ -1399,96 +1399,96 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>beb44857</v>
+        <v>84c049af</v>
       </c>
       <c r="B50" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="C50" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="D50" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E50" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F50" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B51" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C51" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D51" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E51" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F51" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B52" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C52" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D52" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E52" s="2" t="str">
         <v/>
       </c>
       <c r="F52" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>5ddff322</v>
+        <v>6d180155</v>
       </c>
       <c r="B53" t="str">
-        <v>Sehera, Har, Guche &amp; Gajre</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C53" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D53" s="1">
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="E53" s="2" t="str">
         <v/>
       </c>
       <c r="F53" t="str">
-        <v/>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>c047acbd</v>
+        <v>5ddff322</v>
       </c>
       <c r="B54" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="C54" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="D54" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E54" s="2" t="str">
         <v/>
@@ -1499,128 +1499,148 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>d1aee56d</v>
+        <v>c047acbd</v>
       </c>
       <c r="B55" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="C55" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D55" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E55" s="2" t="str">
         <v/>
       </c>
       <c r="F55" t="str">
-        <v>Shireen Dress</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B56" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C56" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D56" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E56" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F56" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B57" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C57" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D57" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E57" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F57" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>9b3747da</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B58" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C58" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D58" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E58" s="2" t="str">
         <v/>
       </c>
       <c r="F58" t="str">
-        <v/>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>db4969e8</v>
+        <v>9b3747da</v>
       </c>
       <c r="B59" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="C59" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="D59" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E59" s="2" t="str">
         <v/>
       </c>
       <c r="F59" t="str">
-        <v>Tushar Traders Oil</v>
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D60" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E60" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
         <v>9961a7bb</v>
       </c>
-      <c r="B60" t="str">
+      <c r="B61" t="str">
         <v>Untracked expenses Petrol, Food, small bills</v>
       </c>
-      <c r="C60" t="str">
+      <c r="C61" t="str">
         <v>Miscellaneous</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D61" s="1">
         <v>9150</v>
       </c>
-      <c r="E60" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F60" t="str">
+      <c r="E61" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F61" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F60"/>
+  <autoFilter ref="A1:F61"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3729,7 +3749,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -4194,36 +4214,36 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Gold &amp; Silver</v>
       </c>
       <c r="B25" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>500</v>
+        <v>1070000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>0</v>
+        <v>1070000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B26" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C26" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -4232,17 +4252,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B27" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C27" s="1">
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>3000</v>
+        <v>575000</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -4251,17 +4271,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Ice Cream, vada pav, Irani Cafe, Milk</v>
       </c>
       <c r="B28" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C28" s="1">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -4270,17 +4290,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B29" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C29" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -4289,17 +4309,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Lucky Mattan Shop (Bakra for haldi)</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B30" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C30" s="1">
-        <v>10000</v>
+        <v>3675</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>3675</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -4308,17 +4328,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Lunch After Mariage Shiv Sunder</v>
+        <v>Lucky Mattan Shop (Bakra for haldi)</v>
       </c>
       <c r="B31" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C31" s="1">
-        <v>2700</v>
+        <v>10000</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>2700</v>
+        <v>10000</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -4327,17 +4347,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Meher Amount</v>
+        <v>Lunch After Mariage Shiv Sunder</v>
       </c>
       <c r="B32" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C32" s="1">
-        <v>11111</v>
+        <v>2700</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>11111</v>
+        <v>2700</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -4346,17 +4366,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
+        <v>Meher Amount</v>
       </c>
       <c r="B33" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C33" s="1">
-        <v>5412</v>
+        <v>11111</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>5412</v>
+        <v>11111</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -4365,17 +4385,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
+        <v>miscellaneous ratjaka (chicken, tags, bartan)</v>
       </c>
       <c r="B34" t="str">
-        <v>Miscellaneous</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C34" s="1">
-        <v>15000</v>
+        <v>5412</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>5412</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -4384,17 +4404,17 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Mom Miscellaneous Bangals, Area cleaning other expence</v>
       </c>
       <c r="B35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C35" s="1">
-        <v>7604</v>
+        <v>15000</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>15000</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -4403,17 +4423,17 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B36" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -4422,17 +4442,17 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B37" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C37" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -4441,17 +4461,17 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B38" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C38" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D38" s="1">
         <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E38" s="1">
         <f>C38-D38</f>
@@ -4460,17 +4480,17 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Mummy Hospital Expence Mate Docter</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B39" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C39" s="1">
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="D39" s="1">
         <f>SUMIF('Payments'!$C:$C,$A39,'Payments'!$E:$E)</f>
-        <v>2900</v>
+        <v>400</v>
       </c>
       <c r="E39" s="1">
         <f>C39-D39</f>
@@ -4479,17 +4499,17 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Mummy sadi</v>
+        <v>Mummy Hospital Expence Mate Docter</v>
       </c>
       <c r="B40" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C40" s="1">
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="D40" s="1">
         <f>SUMIF('Payments'!$C:$C,$A40,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>2900</v>
       </c>
       <c r="E40" s="1">
         <f>C40-D40</f>
@@ -4498,17 +4518,17 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B41" t="str">
-        <v>Music &amp; Entertainment</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C41" s="1">
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="D41" s="1">
         <f>SUMIF('Payments'!$C:$C,$A41,'Payments'!$E:$E)</f>
-        <v>13000</v>
+        <v>1600</v>
       </c>
       <c r="E41" s="1">
         <f>C41-D41</f>
@@ -4517,17 +4537,17 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="B42" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Music &amp; Entertainment</v>
       </c>
       <c r="C42" s="1">
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="D42" s="1">
         <f>SUMIF('Payments'!$C:$C,$A42,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>13000</v>
       </c>
       <c r="E42" s="1">
         <f>C42-D42</f>
@@ -4536,17 +4556,17 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B43" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C43" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D43" s="1">
         <f>SUMIF('Payments'!$C:$C,$A43,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E43" s="1">
         <f>C43-D43</f>
@@ -4555,17 +4575,17 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B44" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C44" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D44" s="1">
         <f>SUMIF('Payments'!$C:$C,$A44,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E44" s="1">
         <f>C44-D44</f>
@@ -4574,17 +4594,17 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B45" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C45" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D45" s="1">
         <f>SUMIF('Payments'!$C:$C,$A45,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E45" s="1">
         <f>C45-D45</f>
@@ -4593,17 +4613,17 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Patti mudekhai</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B46" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C46" s="1">
-        <v>5000</v>
+        <v>24000</v>
       </c>
       <c r="D46" s="1">
         <f>SUMIF('Payments'!$C:$C,$A46,'Payments'!$E:$E)</f>
-        <v>5000</v>
+        <v>24000</v>
       </c>
       <c r="E46" s="1">
         <f>C46-D46</f>
@@ -4612,17 +4632,17 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Petrol Glanza</v>
+        <v>Patti mudekhai</v>
       </c>
       <c r="B47" t="str">
-        <v>Miscellaneous</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C47" s="1">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="D47" s="1">
         <f>SUMIF('Payments'!$C:$C,$A47,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="E47" s="1">
         <f>C47-D47</f>
@@ -4631,17 +4651,17 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Petrol Glanza Darga visit</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B48" t="str">
-        <v>Transport</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C48" s="1">
-        <v>3226</v>
+        <v>4000</v>
       </c>
       <c r="D48" s="1">
         <f>SUMIF('Payments'!$C:$C,$A48,'Payments'!$E:$E)</f>
-        <v>3226</v>
+        <v>4000</v>
       </c>
       <c r="E48" s="1">
         <f>C48-D48</f>
@@ -4650,17 +4670,17 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
+        <v>Petrol Glanza Darga visit</v>
       </c>
       <c r="B49" t="str">
         <v>Transport</v>
       </c>
       <c r="C49" s="1">
-        <v>4000</v>
+        <v>3226</v>
       </c>
       <c r="D49" s="1">
         <f>SUMIF('Payments'!$C:$C,$A49,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>3226</v>
       </c>
       <c r="E49" s="1">
         <f>C49-D49</f>
@@ -4669,55 +4689,55 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza, Himalyan, PUC, Wheel Alingment, Engine cover Advance</v>
       </c>
       <c r="B50" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Transport</v>
       </c>
       <c r="C50" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D50" s="1">
         <f>SUMIF('Payments'!$C:$C,$A50,'Payments'!$E:$E)</f>
-        <v>70000</v>
+        <v>4000</v>
       </c>
       <c r="E50" s="1">
         <f>C50-D50</f>
-        <v>30000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B51" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C51" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D51" s="1">
         <f>SUMIF('Payments'!$C:$C,$A51,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>70000</v>
       </c>
       <c r="E51" s="1">
         <f>C51-D51</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B52" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C52" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D52" s="1">
         <f>SUMIF('Payments'!$C:$C,$A52,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E52" s="1">
         <f>C52-D52</f>
@@ -4726,17 +4746,17 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Sehera, Har, Guche &amp; Gajre</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B53" t="str">
-        <v>Decoration</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C53" s="1">
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="D53" s="1">
         <f>SUMIF('Payments'!$C:$C,$A53,'Payments'!$E:$E)</f>
-        <v>9000</v>
+        <v>11840</v>
       </c>
       <c r="E53" s="1">
         <f>C53-D53</f>
@@ -4745,17 +4765,17 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Sehera, Har, Guche &amp; Gajre</v>
       </c>
       <c r="B54" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Decoration</v>
       </c>
       <c r="C54" s="1">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="D54" s="1">
         <f>SUMIF('Payments'!$C:$C,$A54,'Payments'!$E:$E)</f>
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="E54" s="1">
         <f>C54-D54</f>
@@ -4764,17 +4784,17 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Shireen Dress</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="B55" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C55" s="1">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="D55" s="1">
         <f>SUMIF('Payments'!$C:$C,$A55,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E55" s="1">
         <f>C55-D55</f>
@@ -4783,17 +4803,17 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B56" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C56" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D56" s="1">
         <f>SUMIF('Payments'!$C:$C,$A56,'Payments'!$E:$E)</f>
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E56" s="1">
         <f>C56-D56</f>
@@ -4802,17 +4822,17 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B57" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C57" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D57" s="1">
         <f>SUMIF('Payments'!$C:$C,$A57,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E57" s="1">
         <f>C57-D57</f>
@@ -4821,17 +4841,17 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>tampo traveller</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B58" t="str">
-        <v>Transport</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C58" s="1">
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="D58" s="1">
         <f>SUMIF('Payments'!$C:$C,$A58,'Payments'!$E:$E)</f>
-        <v>7500</v>
+        <v>6190</v>
       </c>
       <c r="E58" s="1">
         <f>C58-D58</f>
@@ -4840,17 +4860,17 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>tampo traveller</v>
       </c>
       <c r="B59" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Transport</v>
       </c>
       <c r="C59" s="1">
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="D59" s="1">
         <f>SUMIF('Payments'!$C:$C,$A59,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>7500</v>
       </c>
       <c r="E59" s="1">
         <f>C59-D59</f>
@@ -4859,17 +4879,17 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Untracked expenses Petrol, Food, small bills</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B60" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C60" s="1">
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="D60" s="1">
         <f>SUMIF('Payments'!$C:$C,$A60,'Payments'!$E:$E)</f>
-        <v>9150</v>
+        <v>5100</v>
       </c>
       <c r="E60" s="1">
         <f>C60-D60</f>
@@ -4878,24 +4898,43 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
+        <v>Untracked expenses Petrol, Food, small bills</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Miscellaneous</v>
+      </c>
+      <c r="C61" s="1">
+        <v>9150</v>
+      </c>
+      <c r="D61" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A61,'Payments'!$E:$E)</f>
+        <v>9150</v>
+      </c>
+      <c r="E61" s="1">
+        <f>C61-D61</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
         <v>Total</v>
       </c>
-      <c r="C61" s="1">
-        <f>SUM(C2:C60)</f>
-        <v>1340605</v>
-      </c>
-      <c r="D61" s="1">
-        <f>SUM(D2:D60)</f>
+      <c r="C62" s="1">
+        <f>SUM(C2:C61)</f>
+        <v>2410605</v>
+      </c>
+      <c r="D62" s="1">
+        <f>SUM(D2:D61)</f>
         <v>1310605</v>
       </c>
-      <c r="E61" s="1">
-        <f>SUM(E2:E60)</f>
-        <v>30000</v>
+      <c r="E62" s="1">
+        <f>SUM(E2:E61)</f>
+        <v>1100000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E62"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹10,70,000.00 by Umar Sayyed (Father) for Gold & Silver
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H81</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1647,7 +1647,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3325,19 +3325,19 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>fc7adcbd</v>
+        <v>1cdb3048</v>
       </c>
       <c r="B65" t="str">
-        <v>04ece648</v>
+        <v>bf56437c</v>
       </c>
       <c r="C65" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Gold &amp; Silver</v>
       </c>
       <c r="D65" s="3">
-        <v>46300</v>
+        <v>46299</v>
       </c>
       <c r="E65" s="1">
-        <v>15000</v>
+        <v>1070000</v>
       </c>
       <c r="F65" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3346,24 +3346,24 @@
         <v>Cash</v>
       </c>
       <c r="H65" t="str">
-        <v>payment done</v>
+        <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>384605f7</v>
+        <v>fc7adcbd</v>
       </c>
       <c r="B66" t="str">
-        <v>22ff3fb2</v>
+        <v>04ece648</v>
       </c>
       <c r="C66" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="D66" s="3">
         <v>46300</v>
       </c>
       <c r="E66" s="1">
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="F66" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3372,24 +3372,24 @@
         <v>Cash</v>
       </c>
       <c r="H66" t="str">
-        <v/>
+        <v>payment done</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>d08ebf7d</v>
+        <v>384605f7</v>
       </c>
       <c r="B67" t="str">
-        <v>9b3747da</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C67" t="str">
-        <v>tampo traveller</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D67" s="3">
         <v>46300</v>
       </c>
       <c r="E67" s="1">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="F67" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3398,56 +3398,56 @@
         <v>Cash</v>
       </c>
       <c r="H67" t="str">
-        <v>cash</v>
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>c193f7b5</v>
+        <v>d08ebf7d</v>
       </c>
       <c r="B68" t="str">
-        <v>9299bcdc</v>
+        <v>9b3747da</v>
       </c>
       <c r="C68" t="str">
-        <v>Patti mudekhai</v>
+        <v>tampo traveller</v>
       </c>
       <c r="D68" s="3">
         <v>46300</v>
       </c>
       <c r="E68" s="1">
-        <v>5000</v>
+        <v>7500</v>
       </c>
       <c r="F68" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G68" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H68" t="str">
-        <v/>
+        <v>cash</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>5a34da87</v>
+        <v>c193f7b5</v>
       </c>
       <c r="B69" t="str">
-        <v>fed12b4d</v>
+        <v>9299bcdc</v>
       </c>
       <c r="C69" t="str">
-        <v>Petrol Glanza Darga visit</v>
+        <v>Patti mudekhai</v>
       </c>
       <c r="D69" s="3">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="E69" s="1">
-        <v>3226</v>
+        <v>5000</v>
       </c>
       <c r="F69" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G69" t="str">
-        <v>Debit Card</v>
+        <v>UPI</v>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -3455,45 +3455,45 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>3adcd8de</v>
+        <v>5a34da87</v>
       </c>
       <c r="B70" t="str">
-        <v>4d3bd5b1</v>
+        <v>fed12b4d</v>
       </c>
       <c r="C70" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Petrol Glanza Darga visit</v>
       </c>
       <c r="D70" s="3">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E70" s="1">
-        <v>24000</v>
+        <v>3226</v>
       </c>
       <c r="F70" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G70" t="str">
-        <v>UPI</v>
+        <v>Debit Card</v>
       </c>
       <c r="H70" t="str">
-        <v>Final payment</v>
+        <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>4f298a0d</v>
+        <v>3adcd8de</v>
       </c>
       <c r="B71" t="str">
-        <v>631875ca</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C71" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D71" s="3">
         <v>46302</v>
       </c>
       <c r="E71" s="1">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="F71" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3502,24 +3502,24 @@
         <v>UPI</v>
       </c>
       <c r="H71" t="str">
-        <v>Installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>141e8fbb</v>
+        <v>4f298a0d</v>
       </c>
       <c r="B72" t="str">
-        <v>4d3bd5b1</v>
+        <v>631875ca</v>
       </c>
       <c r="C72" t="str">
-        <v>Ganesh Bhondve Mandva + decoration</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D72" s="3">
         <v>46302</v>
       </c>
       <c r="E72" s="1">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="F72" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -3528,50 +3528,50 @@
         <v>UPI</v>
       </c>
       <c r="H72" t="str">
-        <v>paid</v>
+        <v>Installment</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>738b696a</v>
+        <v>141e8fbb</v>
       </c>
       <c r="B73" t="str">
-        <v>f31def6e</v>
+        <v>4d3bd5b1</v>
       </c>
       <c r="C73" t="str">
-        <v>Music in reception &amp; sangit</v>
+        <v>Ganesh Bhondve Mandva + decoration</v>
       </c>
       <c r="D73" s="3">
         <v>46302</v>
       </c>
       <c r="E73" s="1">
-        <v>13000</v>
+        <v>500</v>
       </c>
       <c r="F73" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G73" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H73" t="str">
-        <v/>
+        <v>paid</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>ad864ef1</v>
+        <v>738b696a</v>
       </c>
       <c r="B74" t="str">
-        <v>c047acbd</v>
+        <v>f31def6e</v>
       </c>
       <c r="C74" t="str">
-        <v>Shadi &amp; reception Rasam</v>
+        <v>Music in reception &amp; sangit</v>
       </c>
       <c r="D74" s="3">
         <v>46302</v>
       </c>
       <c r="E74" s="1">
-        <v>6000</v>
+        <v>13000</v>
       </c>
       <c r="F74" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3585,149 +3585,149 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>da6b0ec5</v>
+        <v>ad864ef1</v>
       </c>
       <c r="B75" t="str">
-        <v>631875ca</v>
+        <v>c047acbd</v>
       </c>
       <c r="C75" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Shadi &amp; reception Rasam</v>
       </c>
       <c r="D75" s="3">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E75" s="1">
-        <v>33000</v>
+        <v>6000</v>
       </c>
       <c r="F75" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G75" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H75" t="str">
-        <v>Payment done</v>
+        <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>658c49d2</v>
+        <v>da6b0ec5</v>
       </c>
       <c r="B76" t="str">
-        <v>168b7bbd</v>
+        <v>631875ca</v>
       </c>
       <c r="C76" t="str">
-        <v>Huseni Caterers</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="D76" s="3">
         <v>46303</v>
       </c>
       <c r="E76" s="1">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="F76" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G76" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H76" t="str">
-        <v>Final payment</v>
+        <v>Payment done</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>80e653df</v>
+        <v>658c49d2</v>
       </c>
       <c r="B77" t="str">
-        <v>beb44857</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C77" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D77" s="3">
         <v>46303</v>
       </c>
       <c r="E77" s="1">
-        <v>30000</v>
+        <v>125000</v>
       </c>
       <c r="F77" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G77" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H77" t="str">
-        <v>Second last installment</v>
+        <v>Final payment</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>bb9651a4</v>
+        <v>80e653df</v>
       </c>
       <c r="B78" t="str">
-        <v>f7330587</v>
+        <v>beb44857</v>
       </c>
       <c r="C78" t="str">
-        <v>Lunch After Mariage Shiv Sunder</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D78" s="3">
         <v>46303</v>
       </c>
       <c r="E78" s="1">
-        <v>2700</v>
+        <v>30000</v>
       </c>
       <c r="F78" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G78" t="str">
         <v>UPI</v>
       </c>
       <c r="H78" t="str">
-        <v/>
+        <v>Second last installment</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>79cb1a7e</v>
+        <v>bb9651a4</v>
       </c>
       <c r="B79" t="str">
-        <v>22ff3fb2</v>
+        <v>f7330587</v>
       </c>
       <c r="C79" t="str">
-        <v>chair arrangment soyarik gardan</v>
+        <v>Lunch After Mariage Shiv Sunder</v>
       </c>
       <c r="D79" s="3">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E79" s="1">
-        <v>1000</v>
+        <v>2700</v>
       </c>
       <c r="F79" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G79" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H79" t="str">
-        <v>final payment</v>
+        <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>fcb3d16a</v>
+        <v>79cb1a7e</v>
       </c>
       <c r="B80" t="str">
-        <v>70d7465c</v>
+        <v>22ff3fb2</v>
       </c>
       <c r="C80" t="str">
-        <v>3 kg asli ghee</v>
+        <v>chair arrangment soyarik gardan</v>
       </c>
       <c r="D80" s="3">
         <v>46306</v>
       </c>
       <c r="E80" s="1">
-        <v>1830</v>
+        <v>1000</v>
       </c>
       <c r="F80" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -3736,13 +3736,39 @@
         <v>Cash</v>
       </c>
       <c r="H80" t="str">
+        <v>final payment</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>fcb3d16a</v>
+      </c>
+      <c r="B81" t="str">
+        <v>70d7465c</v>
+      </c>
+      <c r="C81" t="str">
+        <v>3 kg asli ghee</v>
+      </c>
+      <c r="D81" s="3">
+        <v>46306</v>
+      </c>
+      <c r="E81" s="1">
+        <v>1830</v>
+      </c>
+      <c r="F81" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G81" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H81" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H80"/>
+  <autoFilter ref="A1:H81"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H80"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H81"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4224,11 +4250,11 @@
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>1070000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>1070000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -4925,11 +4951,11 @@
       </c>
       <c r="D62" s="1">
         <f>SUM(D2:D61)</f>
-        <v>1310605</v>
+        <v>2380605</v>
       </c>
       <c r="E62" s="1">
         <f>SUM(E2:E61)</f>
-        <v>1100000</v>
+        <v>30000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>